<commit_message>
chore(qa): regenerate report for VC-030 and VC-049
Both transitioned to Done in Jira with fix notes.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA/reports/VelChat-QA-Report.xlsx
+++ b/QA/reports/VelChat-QA-Report.xlsx
@@ -629,7 +629,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-12 05:00 UTC</t>
+          <t>Generated 2026-09-13 15:11 UTC</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -14572,7 +14572,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>VC-UNIT-206</t>
+          <t>failureScenarios.test.ts: receipt reassertion after a reconnect with many owed conversations</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
@@ -14592,7 +14592,7 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
@@ -14692,7 +14692,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AA26" s="5" t="inlineStr"/>
+      <c r="AA26" s="5" t="inlineStr">
+        <is>
+          <t>FIX: flushReceipts() (SyncEngine.ts) sent one frame per owed conversation in a single synchronous tick on every reconnect reassert, with no cap — the gateway silently drops inbound frames past ~40/sec per connection (ws-fabric.ts), and the client never learns which ones were dropped since socket.send() only checks readyState, so noteSent() recorded them all as delivered regardless. Added a per-tick cap (MAX_RECEIPT_FRAMES_PER_FLUSH=20, comfortably under the shared 40/sec budget) and, when a flush goes over budget, re-marks the remaining conversations dirty and reschedules a continuation chunk 1100ms later (longer than the gateway rate-limit window, so consecutive chunks land in separate windows) via the existing scheduleReceiptFlush/receiptTimer machinery. Nothing is ever dropped, only spread across more ticks. Verified: full jest suite 485/485 pass, tsc --noEmit clean, eslint 0 errors. Added 2 new tests (failureScenarios.test.ts) with 60 owed conversations (past the real ~40/sec budget): the first synchronous flush stays under 60, and every owed receipt eventually goes out across later chunks.</t>
+        </is>
+      </c>
       <c r="AB26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
@@ -14848,7 +14852,7 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>VC-UNIT-208</t>
+          <t>failureScenarios.test.ts: loading older history across a wide deletion hole</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -14868,7 +14872,7 @@
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
@@ -14967,7 +14971,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AA28" s="5" t="inlineStr"/>
+      <c r="AA28" s="5" t="inlineStr">
+        <is>
+          <t>FIX: fetchOlderMessages() (SyncEngine.ts) treated an empty page from the server as end-of-history, but the backend filters deleted:false — a contiguous deleted run wider than one page comes back completely empty even though real history exists further back. Since the UI (useMessages.ts) only grows its window when loadOlderMessages returns true, and only fires another load on a scroll past a NEW oldest bubble, a false end-of-history report is a permanent dead end with no way for the user to retry. Converted the single fetch into a loop that steps the cursor back over an empty page and tries again, up to a generous safety cap (MAX_HOLE_HOPS=200, purely a circuit breaker against a pathological/corrupt history) before genuinely giving up. One loadOlderMessages() call now reaches all the way past a hole (or to the true start of history) in one go. Verified: full jest suite 485/485 pass, tsc --noEmit clean, eslint 0 errors. Added 2 new tests (failureScenarios.test.ts) with a 70-message-wide deletion hole (wider than the 50-message page): one call steps past it and loads the older page, and the true end-of-history case is unaffected.</t>
+        </is>
+      </c>
       <c r="AB28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
@@ -15257,7 +15265,7 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>VC-UNIT-211</t>
+          <t>messageOrdering.test.ts: VC-030 — a device clock running ahead of the server</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
@@ -15277,7 +15285,7 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
@@ -15377,7 +15385,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AA31" s="5" t="inlineStr"/>
+      <c r="AA31" s="5" t="inlineStr">
+        <is>
+          <t>FIX: two causes, both in the created_at-as-sort-key design. (1) markMessageSent() re-stamped createdAt to the server clock FORWARD ONLY (if (ack.serverTs &gt; m.createdAt)), a rule meant to stop a slow server clock re-burying an offline-composed bubble. Forward-only mixes two clocks in one sort key: on a device whose clock leads the server, an own message keeps its future local stamp and beats every server timestamp that follows it, permanently. The server clock is the same authority that assigns seq, so its timestamp is now adopted in EITHER direction. (2) messageWindowClauses() (extracted from observeMessages so the real query is testable rather than duplicated in a test) now sorts by created_at DESC then seq DESC — seq is the ordering identity per backend-integration-reference §5, and the gateway fans bursts out inside one millisecond, so identical created_at values are normal and were previously resolved by whatever order rows happened to be written. seq is the SECOND key, not the first, because an unsent message has no seq and sorting on it first would file every pending bubble under a null and drag it out of the newest-first window. The pre-existing test never drags a message backwards in time encoded the defect; it was rewritten to assert the concern it actually cared about — that a backwards re-stamp does not change the bubble POSITION — which now holds because seq decides the order. Verified: full jest suite 492/492 pass, tsc --noEmit clean, eslint 0 errors.</t>
+        </is>
+      </c>
       <c r="AB31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
@@ -17888,7 +17900,11 @@
           <t>VC-49</t>
         </is>
       </c>
-      <c r="C50" s="5" t="inlineStr"/>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>profileGate.test.ts: VC-049</t>
+        </is>
+      </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
           <t>Email-prompt bottom sheet reappears on every login even when an email is already saved</t>
@@ -17906,7 +17922,7 @@
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H50" s="5" t="inlineStr">
@@ -18003,7 +18019,7 @@
       </c>
       <c r="AA50" s="5" t="inlineStr">
         <is>
-          <t>Reported by Tusha Bhadouriya during production QA testing.</t>
+          <t>FIX (root-caused): the email is NOT a directory-profile field — profileShape.ts states it is a separately-verified identifier owned by the auth-service (GET /auth/account). useProfileGate decided purely from the LOCAL MMKV mirror, and purgeAccountData() wipes KVKeys.email on every sign-out, so immediately after any login the mirror is empty and the gate prompted unconditionally. useAccountInfo() does fetch the real email and mirror it, but it runs in parallel from AppTabs, so its answer always lost the race — and dismissal is session-only, which is why it returned every single login. The gate now asks the auth-service itself before deciding, via a new pure shouldPromptForProfile() (features/user/model/profileGate.ts): a mirrored email means never prompt; a server email means never prompt (and is re-mirrored so later launches short-circuit with no network); an UNANSWERED server (in flight or unreachable) means WAIT rather than prompt, which also removes the flash of the sheet before the answer lands. Only a definitive server no-email prompts. Verified: full jest suite 492/492 pass (5 new decision tests), tsc --noEmit clean, eslint 0 errors, no eslint-plugin-boundaries violation for the user→auth import (authApi depends only on infra, so no cycle). Not reproduced on a device — no Android hardware attached to this machine; fix is verified at the unit level against the exact reported condition.</t>
         </is>
       </c>
       <c r="AB50" s="5" t="inlineStr">
@@ -18024,7 +18040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C50"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -18210,7 +18226,7 @@
         </is>
       </c>
       <c r="B18" s="22" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C18" s="23" t="inlineStr"/>
     </row>
@@ -18221,7 +18237,7 @@
         </is>
       </c>
       <c r="B19" s="22" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C19" s="23" t="inlineStr"/>
     </row>
@@ -18280,7 +18296,7 @@
       </c>
       <c r="C26" s="25" t="inlineStr">
         <is>
-          <t>22 open P0/P1 defect(s) block the build.</t>
+          <t>19 open P0/P1 defect(s) block the build.</t>
         </is>
       </c>
     </row>
@@ -18483,7 +18499,7 @@
     <row r="40">
       <c r="A40" s="21" t="inlineStr">
         <is>
-          <t>VC-025</t>
+          <t>VC-028</t>
         </is>
       </c>
       <c r="B40" s="22" t="inlineStr">
@@ -18493,14 +18509,14 @@
       </c>
       <c r="C40" s="23" t="inlineStr">
         <is>
-          <t>reassertReceipts() on every connect emits an unbounded burst the gateway silently drops</t>
+          <t>No event_id dedup anywhere — the documented at-least-once guard does not exist</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="21" t="inlineStr">
         <is>
-          <t>VC-028</t>
+          <t>VC-032</t>
         </is>
       </c>
       <c r="B41" s="22" t="inlineStr">
@@ -18510,14 +18526,14 @@
       </c>
       <c r="C41" s="23" t="inlineStr">
         <is>
-          <t>No event_id dedup anywhere — the documented at-least-once guard does not exist</t>
+          <t>No duplicate-notification suppression, though the monotonic watermark to do it already exists</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="21" t="inlineStr">
         <is>
-          <t>VC-030</t>
+          <t>VC-033</t>
         </is>
       </c>
       <c r="B42" s="22" t="inlineStr">
@@ -18527,31 +18543,31 @@
       </c>
       <c r="C42" s="23" t="inlineStr">
         <is>
-          <t>Message window sorts by created_at, not seq — a device clock ahead of the server permanently mis-orders own messages</t>
+          <t>Native pending-event queue is a lock-free read-modify-write that can wipe a reply enqueued mid-drain</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="21" t="inlineStr">
         <is>
-          <t>VC-032</t>
+          <t>VC-039</t>
         </is>
       </c>
       <c r="B43" s="22" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="C43" s="23" t="inlineStr">
         <is>
-          <t>No duplicate-notification suppression, though the monotonic watermark to do it already exists</t>
+          <t>Any authenticated user can READ and WRITE any conversation — no authorization on the chat routes, and conversation ids are derivable offline</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="21" t="inlineStr">
         <is>
-          <t>VC-033</t>
+          <t>VC-040</t>
         </is>
       </c>
       <c r="B44" s="22" t="inlineStr">
@@ -18561,31 +18577,31 @@
       </c>
       <c r="C44" s="23" t="inlineStr">
         <is>
-          <t>Native pending-event queue is a lock-free read-modify-write that can wipe a reply enqueued mid-drain</t>
+          <t>A push endpoint can be registered against another account's userId, redirecting their push wake-ups</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="21" t="inlineStr">
         <is>
-          <t>VC-039</t>
+          <t>VC-041</t>
         </is>
       </c>
       <c r="B45" s="22" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="C45" s="23" t="inlineStr">
         <is>
-          <t>Any authenticated user can READ and WRITE any conversation — no authorization on the chat routes, and conversation ids are derivable offline</t>
+          <t>POST /chat/messages accepts a conversationId that does not exist</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="21" t="inlineStr">
         <is>
-          <t>VC-040</t>
+          <t>VC-043</t>
         </is>
       </c>
       <c r="B46" s="22" t="inlineStr">
@@ -18595,14 +18611,14 @@
       </c>
       <c r="C46" s="23" t="inlineStr">
         <is>
-          <t>A push endpoint can be registered against another account's userId, redirecting their push wake-ups</t>
+          <t>Concurrent refresh-token requests can all succeed — rotation is not race-safe</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="21" t="inlineStr">
         <is>
-          <t>VC-041</t>
+          <t>VC-045</t>
         </is>
       </c>
       <c r="B47" s="22" t="inlineStr">
@@ -18612,58 +18628,7 @@
       </c>
       <c r="C47" s="23" t="inlineStr">
         <is>
-          <t>POST /chat/messages accepts a conversationId that does not exist</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="21" t="inlineStr">
-        <is>
-          <t>VC-043</t>
-        </is>
-      </c>
-      <c r="B48" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C48" s="23" t="inlineStr">
-        <is>
-          <t>Concurrent refresh-token requests can all succeed — rotation is not race-safe</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="21" t="inlineStr">
-        <is>
-          <t>VC-045</t>
-        </is>
-      </c>
-      <c r="B49" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C49" s="23" t="inlineStr">
-        <is>
           <t>Real-time messaging and notification-reply sync needs multi-scenario two-device verification</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="21" t="inlineStr">
-        <is>
-          <t>VC-049</t>
-        </is>
-      </c>
-      <c r="B50" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C50" s="23" t="inlineStr">
-        <is>
-          <t>Email-prompt bottom sheet reappears on every login even when an email is already saved</t>
         </is>
       </c>
     </row>
@@ -18816,7 +18781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -19292,12 +19257,12 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>VC-026</t>
+          <t>VC-025</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Unread count climbs and the read watermark stalls for messages backfilled into the chat you are reading</t>
+          <t>reassertReceipts() on every connect emits an unbounded burst the gateway silently drops</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -19312,7 +19277,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>VC-UNIT-207</t>
+          <t>failureScenarios.test.ts: receipt reassertion after a reconnect with many owed conversations</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr"/>
@@ -19323,24 +19288,24 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>VC-001 makes backfills constant, so this fires often. FIX: pageBackfill now mirrors the live-message path: if the backfilled page lands in the conversation on screen, it marks read (noteRead + clearUnread) instead of only noteDelivered. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
+          <t>FIX: flushReceipts() (SyncEngine.ts) sent one frame per owed conversation in a single synchronous tick on every reconnect reassert, with no cap — the gateway silently drops inbound frames past ~40/sec per connection (ws-fabric.ts), and the client never learns which ones were dropped since socket.send() only checks readyState, so noteSent() recorded them all as delivered regardless. Added a per-tick cap (MAX_RECEIPT_FRAMES_PER_FLUSH=20, comfortably under the shared 40/sec budget) and, when a flush goes over budget, re-marks the remaining conversations dirty and reschedules a continuation chunk 1100ms later (longer than the gateway rate-limit window, so consecutive chunks land in separate windows) via the existing scheduleReceiptFlush/receiptTimer machinery. Nothing is ever dropped, only spread across more ticks. Verified: full jest suite 485/485 pass, tsc --noEmit clean, eslint 0 errors. Added 2 new tests (failureScenarios.test.ts) with 60 owed conversations (past the real ~40/sec budget): the first synchronous flush stays under 60, and every owed receipt eventually goes out across later chunks.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>VC-029</t>
+          <t>VC-026</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Outbox backoff exhaustion is unreachable — MAX_SEND_ATTEMPTS can never fire</t>
+          <t>Unread count climbs and the read watermark stalls for messages backfilled into the chat you are reading</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -19350,7 +19315,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>VC-UNIT-210</t>
+          <t>VC-UNIT-207</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr"/>
@@ -19361,19 +19326,19 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>FIX: removed the dead attempt-count exhaustion path (MAX_SEND_ATTEMPTS/nextOutboxRetry in syncLogic.ts) that markFailed() fell back to only when permanent was omitted — a fallback no real call site ever triggered (SyncEngine.ts always passes a classified boolean from classifySendFailure()). This mechanism contradicted the documented WhatsApp-style policy (sendFailurePolicy.ts: reachability failures retry forever, never auto-fail by attempt count) and had no basis in the HLD/LLD spec (§L6 outbox semantics: classification-based retryable-vs-permanent only, no attempt cap). Made markFailed()'s permanent parameter required (compiler now prevents the dead path from ever coming back), updated the one test that accidentally relied on the old default (realtime-hardening.test.ts) to pass permanent explicitly, removed the 4 tests for the deleted dead function, and added a new regression test proving a retryable cause stays queued past a high attempt count. Verified: full jest suite 452/452 pass (455 - 4 removed + 1 added), tsc --noEmit clean, eslint 0 errors.</t>
+          <t>VC-001 makes backfills constant, so this fires often. FIX: pageBackfill now mirrors the live-message path: if the backfilled page lands in the conversation on screen, it marks read (noteRead + clearUnread) instead of only noteDelivered. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>VC-034</t>
+          <t>VC-027</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Retry-After is honored with an unbounded, uncancellable sleep</t>
+          <t>'Load older' dead-ends permanently on a deletion hole wider than one page</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -19388,7 +19353,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>VC-UNIT-215</t>
+          <t>failureScenarios.test.ts: loading older history across a wide deletion hole</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr"/>
@@ -19399,19 +19364,19 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>FIX: Retry-After is now clamped to [0, 10s] (MAX_RETRY_AFTER_MS, client.ts) before the wait, instead of obeying a server-supplied value unbounded. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
+          <t>FIX: fetchOlderMessages() (SyncEngine.ts) treated an empty page from the server as end-of-history, but the backend filters deleted:false — a contiguous deleted run wider than one page comes back completely empty even though real history exists further back. Since the UI (useMessages.ts) only grows its window when loadOlderMessages returns true, and only fires another load on a scroll past a NEW oldest bubble, a false end-of-history report is a permanent dead end with no way for the user to retry. Converted the single fetch into a loop that steps the cursor back over an empty page and tries again, up to a generous safety cap (MAX_HOLE_HOPS=200, purely a circuit breaker against a pathological/corrupt history) before genuinely giving up. One loadOlderMessages() call now reaches all the way past a hole (or to the true start of history) in one go. Verified: full jest suite 485/485 pass, tsc --noEmit clean, eslint 0 errors. Added 2 new tests (failureScenarios.test.ts) with a 70-message-wide deletion hole (wider than the 50-message page): one call steps past it and loads the older page, and the true end-of-history case is unaffected.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>VC-035</t>
+          <t>VC-029</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>A misbuilt binary reports env:'dev' while talking to production</t>
+          <t>Outbox backoff exhaustion is unreachable — MAX_SEND_ATTEMPTS can never fire</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -19426,7 +19391,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>VC-UNIT-216</t>
+          <t>VC-UNIT-210</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr"/>
@@ -19437,34 +19402,34 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>The prod URL fallback direction is defensible; make `name` fall back to 'prod' alongside it, or log.error when Config.API_BASE_URL is absent. FIX: Extracted the pure resolveAppEnv(rawName, rawApiBaseUrl, rawWsUrl) so the fallback logic is unit-testable. An unrecognised/missing ENV now falls back to 'prod' alongside the URL fallback (previously 'dev'), so a misbuilt binary can never report a safe-sounding name while actually pointing at production. Verified: full jest suite 455/455 pass, tsc --noEmit clean, eslint 0 errors.</t>
+          <t>FIX: removed the dead attempt-count exhaustion path (MAX_SEND_ATTEMPTS/nextOutboxRetry in syncLogic.ts) that markFailed() fell back to only when permanent was omitted — a fallback no real call site ever triggered (SyncEngine.ts always passes a classified boolean from classifySendFailure()). This mechanism contradicted the documented WhatsApp-style policy (sendFailurePolicy.ts: reachability failures retry forever, never auto-fail by attempt count) and had no basis in the HLD/LLD spec (§L6 outbox semantics: classification-based retryable-vs-permanent only, no attempt cap). Made markFailed()'s permanent parameter required (compiler now prevents the dead path from ever coming back), updated the one test that accidentally relied on the old default (realtime-hardening.test.ts) to pass permanent explicitly, removed the 4 tests for the deleted dead function, and added a new regression test proving a retryable cause stays queued past a high attempt count. Verified: full jest suite 452/452 pass (455 - 4 removed + 1 added), tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>VC-036</t>
+          <t>VC-030</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Cold start after &gt;15 min idle opens the WebSocket with a certainly-expired token</t>
+          <t>Message window sorts by created_at, not seq — a device clock ahead of the server permanently mis-orders own messages</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>dev branch, 2026-09-12</t>
+          <t>dev branch, 2026-09-13</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>VC-UNIT-217</t>
+          <t>messageOrdering.test.ts: VC-030 — a device clock running ahead of the server</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr"/>
@@ -19475,7 +19440,159 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
+          <t>FIX: two causes, both in the created_at-as-sort-key design. (1) markMessageSent() re-stamped createdAt to the server clock FORWARD ONLY (if (ack.serverTs &gt; m.createdAt)), a rule meant to stop a slow server clock re-burying an offline-composed bubble. Forward-only mixes two clocks in one sort key: on a device whose clock leads the server, an own message keeps its future local stamp and beats every server timestamp that follows it, permanently. The server clock is the same authority that assigns seq, so its timestamp is now adopted in EITHER direction. (2) messageWindowClauses() (extracted from observeMessages so the real query is testable rather than duplicated in a test) now sorts by created_at DESC then seq DESC — seq is the ordering identity per backend-integration-reference §5, and the gateway fans bursts out inside one millisecond, so identical created_at values are normal and were previously resolved by whatever order rows happened to be written. seq is the SECOND key, not the first, because an unsent message has no seq and sorting on it first would file every pending bubble under a null and drag it out of the newest-first window. The pre-existing test never drags a message backwards in time encoded the defect; it was rewritten to assert the concern it actually cared about — that a backwards re-stamp does not change the bubble POSITION — which now holds because seq decides the order. Verified: full jest suite 492/492 pass, tsc --noEmit clean, eslint 0 errors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>VC-034</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Retry-After is honored with an unbounded, uncancellable sleep</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>dev branch, 2026-09-12</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>VC-UNIT-215</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr"/>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Not independently tested</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>FIX: Retry-After is now clamped to [0, 10s] (MAX_RETRY_AFTER_MS, client.ts) before the wait, instead of obeying a server-supplied value unbounded. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>VC-035</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>A misbuilt binary reports env:'dev' while talking to production</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>dev branch, 2026-09-12</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>VC-UNIT-216</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr"/>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>Not independently tested</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>The prod URL fallback direction is defensible; make `name` fall back to 'prod' alongside it, or log.error when Config.API_BASE_URL is absent. FIX: Extracted the pure resolveAppEnv(rawName, rawApiBaseUrl, rawWsUrl) so the fallback logic is unit-testable. An unrecognised/missing ENV now falls back to 'prod' alongside the URL fallback (previously 'dev'), so a misbuilt binary can never report a safe-sounding name while actually pointing at production. Verified: full jest suite 455/455 pass, tsc --noEmit clean, eslint 0 errors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>VC-036</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Cold start after &gt;15 min idle opens the WebSocket with a certainly-expired token</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>dev branch, 2026-09-12</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>VC-UNIT-217</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr"/>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Not independently tested</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
           <t>FIX: hasValidSession() added (tokens.ts); useAuthBootstrap now refreshes before hydrating on an expired-but-present token. hasSession() deliberately left presence-only to protect SyncEngine reconnect guards. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>VC-049</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Email-prompt bottom sheet reappears on every login even when an email is already saved</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>dev branch, 2026-09-13</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>profileGate.test.ts: VC-049</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr"/>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Not independently tested</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>FIX (root-caused): the email is NOT a directory-profile field — profileShape.ts states it is a separately-verified identifier owned by the auth-service (GET /auth/account). useProfileGate decided purely from the LOCAL MMKV mirror, and purgeAccountData() wipes KVKeys.email on every sign-out, so immediately after any login the mirror is empty and the gate prompted unconditionally. useAccountInfo() does fetch the real email and mirror it, but it runs in parallel from AppTabs, so its answer always lost the race — and dismissal is session-only, which is why it returned every single login. The gate now asks the auth-service itself before deciding, via a new pure shouldPromptForProfile() (features/user/model/profileGate.ts): a mirrored email means never prompt; a server email means never prompt (and is re-mirrored so later launches short-circuit with no network); an UNANSWERED server (in flight or unreachable) means WAIT rather than prompt, which also removes the flash of the sheet before the answer lands. Only a definitive server no-email prompts. Verified: full jest suite 492/492 pass (5 new decision tests), tsc --noEmit clean, eslint 0 errors, no eslint-plugin-boundaries violation for the user→auth import (authApi depends only on infra, so no cycle). Not reproduced on a device — no Android hardware attached to this machine; fix is verified at the unit level against the exact reported condition.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(qa): regenerate report for VC-047
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA/reports/VelChat-QA-Report.xlsx
+++ b/QA/reports/VelChat-QA-Report.xlsx
@@ -629,7 +629,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-13 15:11 UTC</t>
+          <t>Generated 2026-09-13 15:24 UTC</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -17334,7 +17334,7 @@
       </c>
       <c r="AA45" s="5" t="inlineStr">
         <is>
-          <t>Reported by Tusha Bhadouriya during production QA testing.</t>
+          <t>PARTIALLY FIXED — still open pending the remaining half. The name-precedence half is done (see VC-047): a saved contact name now wins over the registered one and resolves at READ time in the chat list and chat header, so it no longer requires opening the chat first, and a background revalidation can no longer overwrite it. What is NOT fixed, and why this stays open: the residual complaint is DISCOVERY TIMING, not precedence — a contact saved in the phone while VelChat is running is not matched until the next discovery run (app resume / prewarm), so until then that peer is genuinely unknown to the client and still renders as the number. Making that immediate needs the address-book snapshot to notify its readers (or a contacts-changed observer) so an already-mounted chat list re-renders, which is a separate change and is deliberately NOT bolted on here. Re-test after the VC-047 fix: the wrong-name-shown symptoms should be gone; only the just-saved-while-app-open case should remain.</t>
         </is>
       </c>
       <c r="AB45" s="5" t="inlineStr">
@@ -17626,7 +17626,11 @@
           <t>VC-47</t>
         </is>
       </c>
-      <c r="C48" s="5" t="inlineStr"/>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>peerDisplayName.test.ts: VC-044 / VC-047, conversationRow.test.ts: VC-044 / VC-047</t>
+        </is>
+      </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
           <t>Chat List shows the registered VelChat name instead of the saved contact name until a chat is opened</t>
@@ -17644,7 +17648,7 @@
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H48" s="5" t="inlineStr">
@@ -17743,7 +17747,7 @@
       </c>
       <c r="AA48" s="5" t="inlineStr">
         <is>
-          <t>Reported by Tusha Bhadouriya during production QA testing. May share a root cause with the contact-sync issue reported as a separate entry.</t>
+          <t>FIX (root-caused): the address book was consulted on exactly ONE path. startDm() writes the saved name when a chat is opened from New Chat / Message Yourself — which is why the name corrected itself after opening — while every other path used server data, and refreshPeerIdentity() actively OVERWROTE a saved name with the registered one on its next background revalidation (once per TTL/session). Introduced peerDisplayName() (features/contacts/model), the single precedence rule: the name YOU saved wins over the name the peer registered; falls back to the registered name for someone not in your book or when the book has not loaded; returns undefined when neither side has a usable name so callers keep what they have; group rows are untouched (no peerId to look up). Applied at both the WRITE side (refreshPeerIdentity, both the TTL path and the profile-changed push, so a revalidation can no longer downgrade a saved name) and the READ side (toConversationRow for the chat list, useConversationIdentity for the chat header), the latter being what makes a saved name appear WITHOUT having to open the chat first. Exposed discoveredContacts() from the contacts barrel as a cache read (no re-discovery). Verified: full jest suite 502/502 pass (10 new tests), tsc --noEmit clean, eslint 0 errors and no boundary violation. Not re-tested on a device — no Android hardware attached to this machine.</t>
         </is>
       </c>
       <c r="AB48" s="5" t="inlineStr">
@@ -18226,7 +18230,7 @@
         </is>
       </c>
       <c r="B18" s="22" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C18" s="23" t="inlineStr"/>
     </row>
@@ -18237,7 +18241,7 @@
         </is>
       </c>
       <c r="B19" s="22" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C19" s="23" t="inlineStr"/>
     </row>
@@ -18781,7 +18785,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -19561,17 +19565,17 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>VC-049</t>
+          <t>VC-047</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Email-prompt bottom sheet reappears on every login even when an email is already saved</t>
+          <t>Chat List shows the registered VelChat name instead of the saved contact name until a chat is opened</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
@@ -19581,7 +19585,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>profileGate.test.ts: VC-049</t>
+          <t>peerDisplayName.test.ts: VC-044 / VC-047, conversationRow.test.ts: VC-044 / VC-047</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr"/>
@@ -19591,6 +19595,44 @@
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>FIX (root-caused): the address book was consulted on exactly ONE path. startDm() writes the saved name when a chat is opened from New Chat / Message Yourself — which is why the name corrected itself after opening — while every other path used server data, and refreshPeerIdentity() actively OVERWROTE a saved name with the registered one on its next background revalidation (once per TTL/session). Introduced peerDisplayName() (features/contacts/model), the single precedence rule: the name YOU saved wins over the name the peer registered; falls back to the registered name for someone not in your book or when the book has not loaded; returns undefined when neither side has a usable name so callers keep what they have; group rows are untouched (no peerId to look up). Applied at both the WRITE side (refreshPeerIdentity, both the TTL path and the profile-changed push, so a revalidation can no longer downgrade a saved name) and the READ side (toConversationRow for the chat list, useConversationIdentity for the chat header), the latter being what makes a saved name appear WITHOUT having to open the chat first. Exposed discoveredContacts() from the contacts barrel as a cache read (no re-discovery). Verified: full jest suite 502/502 pass (10 new tests), tsc --noEmit clean, eslint 0 errors and no boundary violation. Not re-tested on a device — no Android hardware attached to this machine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>VC-049</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Email-prompt bottom sheet reappears on every login even when an email is already saved</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>dev branch, 2026-09-13</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>profileGate.test.ts: VC-049</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr"/>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Not independently tested</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>FIX (root-caused): the email is NOT a directory-profile field — profileShape.ts states it is a separately-verified identifier owned by the auth-service (GET /auth/account). useProfileGate decided purely from the LOCAL MMKV mirror, and purgeAccountData() wipes KVKeys.email on every sign-out, so immediately after any login the mirror is empty and the gate prompted unconditionally. useAccountInfo() does fetch the real email and mirror it, but it runs in parallel from AppTabs, so its answer always lost the race — and dismissal is session-only, which is why it returned every single login. The gate now asks the auth-service itself before deciding, via a new pure shouldPromptForProfile() (features/user/model/profileGate.ts): a mirrored email means never prompt; a server email means never prompt (and is re-mirrored so later launches short-circuit with no network); an UNANSWERED server (in flight or unreachable) means WAIT rather than prompt, which also removes the flash of the sheet before the answer lands. Only a definitive server no-email prompts. Verified: full jest suite 492/492 pass (5 new decision tests), tsc --noEmit clean, eslint 0 errors, no eslint-plugin-boundaries violation for the user→auth import (authApi depends only on infra, so no cycle). Not reproduced on a device — no Android hardware attached to this machine; fix is verified at the unit level against the exact reported condition.</t>
         </is>

</xml_diff>

<commit_message>
chore(qa): regenerate report for VC-031 and VC-028
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA/reports/VelChat-QA-Report.xlsx
+++ b/QA/reports/VelChat-QA-Report.xlsx
@@ -629,7 +629,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-13 15:24 UTC</t>
+          <t>Generated 2026-09-13 15:30 UTC</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -15011,7 +15011,7 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Won't Fix</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
@@ -15110,7 +15110,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AA29" s="5" t="inlineStr"/>
+      <c r="AA29" s="5" t="inlineStr">
+        <is>
+          <t>NO CODE CHANGE — not reproducible as filed; closing with evidence rather than building the suggested LRU. Two points. (1) The premise has been overtaken: the report says dedup relies on DB client_msg_id/seq paths "which VC-020 shows are not race-safe" — VC-020 was fixed earlier in this run (the batch lookups were moved INSIDE db.write, making check-and-act atomic), so those paths ARE now race-safe. (2) The reported impact (duplicate bubbles on redelivery) is already covered by passing tests: failureScenarios.test.ts "a duplicate realtime frame produces one row, one unread and one preview — however many times it lands" delivers the IDENTICAL frame three times and asserts a single row, and "does not duplicate when a whole catch-up is replayed" re-serves an entire window. Also note socket.ts:7 does not promise an LRU — it documents where event_id LIVES in the envelope, not that the client indexes it. An event_id LRU would be a second, redundant dedup layer in front of one the database already provides idempotently (seq is the server-assigned identity), with its own memory and eviction to get wrong. Recommend reopening only if a real duplicate is ever observed on a device.</t>
+        </is>
+      </c>
       <c r="AB29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
@@ -15405,7 +15409,7 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>VC-UNIT-212</t>
+          <t>runSequentially.test.ts: VC-031</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
@@ -15425,7 +15429,7 @@
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H32" s="5" t="inlineStr">
@@ -15527,7 +15531,7 @@
       </c>
       <c r="AA32" s="5" t="inlineStr">
         <is>
-          <t>The existing test passes only because sendText is invoked synchronously at the top of each handler — it cannot fail for the reason it claims.</t>
+          <t>FIX: the drain mapped each queued event to a thunk and then IMMEDIATELY mapped again to call it — events.map(e =&gt; () =&gt; handle(e)).map(run =&gt; run()) — so every handler was already in flight before Promise.allSettled waited on anything. The code did the exact opposite of the comment directly above it. Replaced with a new runSequentially() helper (features/notifications/model) that awaits each action in turn while still collecting per-item outcomes, so one failing action cannot abandon the rest (a reply must go out even if a preceding mute threw) — allSettle gives that second property but cannot give the first, since it can only wait on promises that have already been started. Verified: full jest suite 506/506 pass (4 new tests, including a max-concurrency assertion that fails against the old eager implementation), tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
       <c r="AB32" s="5" t="inlineStr"/>
@@ -18044,7 +18048,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -18230,7 +18234,7 @@
         </is>
       </c>
       <c r="B18" s="22" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C18" s="23" t="inlineStr"/>
     </row>
@@ -18241,7 +18245,7 @@
         </is>
       </c>
       <c r="B19" s="22" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C19" s="23" t="inlineStr"/>
     </row>
@@ -18300,7 +18304,7 @@
       </c>
       <c r="C26" s="25" t="inlineStr">
         <is>
-          <t>19 open P0/P1 defect(s) block the build.</t>
+          <t>18 open P0/P1 defect(s) block the build.</t>
         </is>
       </c>
     </row>
@@ -18503,7 +18507,7 @@
     <row r="40">
       <c r="A40" s="21" t="inlineStr">
         <is>
-          <t>VC-028</t>
+          <t>VC-032</t>
         </is>
       </c>
       <c r="B40" s="22" t="inlineStr">
@@ -18513,14 +18517,14 @@
       </c>
       <c r="C40" s="23" t="inlineStr">
         <is>
-          <t>No event_id dedup anywhere — the documented at-least-once guard does not exist</t>
+          <t>No duplicate-notification suppression, though the monotonic watermark to do it already exists</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="21" t="inlineStr">
         <is>
-          <t>VC-032</t>
+          <t>VC-033</t>
         </is>
       </c>
       <c r="B41" s="22" t="inlineStr">
@@ -18530,48 +18534,48 @@
       </c>
       <c r="C41" s="23" t="inlineStr">
         <is>
-          <t>No duplicate-notification suppression, though the monotonic watermark to do it already exists</t>
+          <t>Native pending-event queue is a lock-free read-modify-write that can wipe a reply enqueued mid-drain</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="21" t="inlineStr">
         <is>
-          <t>VC-033</t>
+          <t>VC-039</t>
         </is>
       </c>
       <c r="B42" s="22" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="C42" s="23" t="inlineStr">
         <is>
-          <t>Native pending-event queue is a lock-free read-modify-write that can wipe a reply enqueued mid-drain</t>
+          <t>Any authenticated user can READ and WRITE any conversation — no authorization on the chat routes, and conversation ids are derivable offline</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="21" t="inlineStr">
         <is>
-          <t>VC-039</t>
+          <t>VC-040</t>
         </is>
       </c>
       <c r="B43" s="22" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="C43" s="23" t="inlineStr">
         <is>
-          <t>Any authenticated user can READ and WRITE any conversation — no authorization on the chat routes, and conversation ids are derivable offline</t>
+          <t>A push endpoint can be registered against another account's userId, redirecting their push wake-ups</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="21" t="inlineStr">
         <is>
-          <t>VC-040</t>
+          <t>VC-041</t>
         </is>
       </c>
       <c r="B44" s="22" t="inlineStr">
@@ -18581,14 +18585,14 @@
       </c>
       <c r="C44" s="23" t="inlineStr">
         <is>
-          <t>A push endpoint can be registered against another account's userId, redirecting their push wake-ups</t>
+          <t>POST /chat/messages accepts a conversationId that does not exist</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="21" t="inlineStr">
         <is>
-          <t>VC-041</t>
+          <t>VC-043</t>
         </is>
       </c>
       <c r="B45" s="22" t="inlineStr">
@@ -18598,14 +18602,14 @@
       </c>
       <c r="C45" s="23" t="inlineStr">
         <is>
-          <t>POST /chat/messages accepts a conversationId that does not exist</t>
+          <t>Concurrent refresh-token requests can all succeed — rotation is not race-safe</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="21" t="inlineStr">
         <is>
-          <t>VC-043</t>
+          <t>VC-045</t>
         </is>
       </c>
       <c r="B46" s="22" t="inlineStr">
@@ -18614,23 +18618,6 @@
         </is>
       </c>
       <c r="C46" s="23" t="inlineStr">
-        <is>
-          <t>Concurrent refresh-token requests can all succeed — rotation is not race-safe</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="21" t="inlineStr">
-        <is>
-          <t>VC-045</t>
-        </is>
-      </c>
-      <c r="B47" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C47" s="23" t="inlineStr">
         <is>
           <t>Real-time messaging and notification-reply sync needs multi-scenario two-device verification</t>
         </is>
@@ -18785,7 +18772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -19451,12 +19438,12 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>VC-034</t>
+          <t>VC-031</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Retry-After is honored with an unbounded, uncancellable sleep</t>
+          <t>runQueuedPushActions runs queued notification actions concurrently while claiming to serialize them</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -19466,12 +19453,12 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>dev branch, 2026-09-12</t>
+          <t>dev branch, 2026-09-13</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>VC-UNIT-215</t>
+          <t>runSequentially.test.ts: VC-031</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr"/>
@@ -19482,19 +19469,19 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>FIX: Retry-After is now clamped to [0, 10s] (MAX_RETRY_AFTER_MS, client.ts) before the wait, instead of obeying a server-supplied value unbounded. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
+          <t>FIX: the drain mapped each queued event to a thunk and then IMMEDIATELY mapped again to call it — events.map(e =&gt; () =&gt; handle(e)).map(run =&gt; run()) — so every handler was already in flight before Promise.allSettled waited on anything. The code did the exact opposite of the comment directly above it. Replaced with a new runSequentially() helper (features/notifications/model) that awaits each action in turn while still collecting per-item outcomes, so one failing action cannot abandon the rest (a reply must go out even if a preceding mute threw) — allSettle gives that second property but cannot give the first, since it can only wait on promises that have already been started. Verified: full jest suite 506/506 pass (4 new tests, including a max-concurrency assertion that fails against the old eager implementation), tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>VC-035</t>
+          <t>VC-034</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>A misbuilt binary reports env:'dev' while talking to production</t>
+          <t>Retry-After is honored with an unbounded, uncancellable sleep</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -19509,7 +19496,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>VC-UNIT-216</t>
+          <t>VC-UNIT-215</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr"/>
@@ -19520,19 +19507,19 @@
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>The prod URL fallback direction is defensible; make `name` fall back to 'prod' alongside it, or log.error when Config.API_BASE_URL is absent. FIX: Extracted the pure resolveAppEnv(rawName, rawApiBaseUrl, rawWsUrl) so the fallback logic is unit-testable. An unrecognised/missing ENV now falls back to 'prod' alongside the URL fallback (previously 'dev'), so a misbuilt binary can never report a safe-sounding name while actually pointing at production. Verified: full jest suite 455/455 pass, tsc --noEmit clean, eslint 0 errors.</t>
+          <t>FIX: Retry-After is now clamped to [0, 10s] (MAX_RETRY_AFTER_MS, client.ts) before the wait, instead of obeying a server-supplied value unbounded. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>VC-036</t>
+          <t>VC-035</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Cold start after &gt;15 min idle opens the WebSocket with a certainly-expired token</t>
+          <t>A misbuilt binary reports env:'dev' while talking to production</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -19547,7 +19534,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>VC-UNIT-217</t>
+          <t>VC-UNIT-216</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr"/>
@@ -19558,19 +19545,19 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>FIX: hasValidSession() added (tokens.ts); useAuthBootstrap now refreshes before hydrating on an expired-but-present token. hasSession() deliberately left presence-only to protect SyncEngine reconnect guards. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
+          <t>The prod URL fallback direction is defensible; make `name` fall back to 'prod' alongside it, or log.error when Config.API_BASE_URL is absent. FIX: Extracted the pure resolveAppEnv(rawName, rawApiBaseUrl, rawWsUrl) so the fallback logic is unit-testable. An unrecognised/missing ENV now falls back to 'prod' alongside the URL fallback (previously 'dev'), so a misbuilt binary can never report a safe-sounding name while actually pointing at production. Verified: full jest suite 455/455 pass, tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>VC-047</t>
+          <t>VC-036</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Chat List shows the registered VelChat name instead of the saved contact name until a chat is opened</t>
+          <t>Cold start after &gt;15 min idle opens the WebSocket with a certainly-expired token</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -19580,12 +19567,12 @@
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>dev branch, 2026-09-13</t>
+          <t>dev branch, 2026-09-12</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>peerDisplayName.test.ts: VC-044 / VC-047, conversationRow.test.ts: VC-044 / VC-047</t>
+          <t>VC-UNIT-217</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr"/>
@@ -19596,24 +19583,24 @@
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>FIX (root-caused): the address book was consulted on exactly ONE path. startDm() writes the saved name when a chat is opened from New Chat / Message Yourself — which is why the name corrected itself after opening — while every other path used server data, and refreshPeerIdentity() actively OVERWROTE a saved name with the registered one on its next background revalidation (once per TTL/session). Introduced peerDisplayName() (features/contacts/model), the single precedence rule: the name YOU saved wins over the name the peer registered; falls back to the registered name for someone not in your book or when the book has not loaded; returns undefined when neither side has a usable name so callers keep what they have; group rows are untouched (no peerId to look up). Applied at both the WRITE side (refreshPeerIdentity, both the TTL path and the profile-changed push, so a revalidation can no longer downgrade a saved name) and the READ side (toConversationRow for the chat list, useConversationIdentity for the chat header), the latter being what makes a saved name appear WITHOUT having to open the chat first. Exposed discoveredContacts() from the contacts barrel as a cache read (no re-discovery). Verified: full jest suite 502/502 pass (10 new tests), tsc --noEmit clean, eslint 0 errors and no boundary violation. Not re-tested on a device — no Android hardware attached to this machine.</t>
+          <t>FIX: hasValidSession() added (tokens.ts); useAuthBootstrap now refreshes before hydrating on an expired-but-present token. hasSession() deliberately left presence-only to protect SyncEngine reconnect guards. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>VC-049</t>
+          <t>VC-047</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Email-prompt bottom sheet reappears on every login even when an email is already saved</t>
+          <t>Chat List shows the registered VelChat name instead of the saved contact name until a chat is opened</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -19623,7 +19610,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>profileGate.test.ts: VC-049</t>
+          <t>peerDisplayName.test.ts: VC-044 / VC-047, conversationRow.test.ts: VC-044 / VC-047</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr"/>
@@ -19633,6 +19620,44 @@
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>FIX (root-caused): the address book was consulted on exactly ONE path. startDm() writes the saved name when a chat is opened from New Chat / Message Yourself — which is why the name corrected itself after opening — while every other path used server data, and refreshPeerIdentity() actively OVERWROTE a saved name with the registered one on its next background revalidation (once per TTL/session). Introduced peerDisplayName() (features/contacts/model), the single precedence rule: the name YOU saved wins over the name the peer registered; falls back to the registered name for someone not in your book or when the book has not loaded; returns undefined when neither side has a usable name so callers keep what they have; group rows are untouched (no peerId to look up). Applied at both the WRITE side (refreshPeerIdentity, both the TTL path and the profile-changed push, so a revalidation can no longer downgrade a saved name) and the READ side (toConversationRow for the chat list, useConversationIdentity for the chat header), the latter being what makes a saved name appear WITHOUT having to open the chat first. Exposed discoveredContacts() from the contacts barrel as a cache read (no re-discovery). Verified: full jest suite 502/502 pass (10 new tests), tsc --noEmit clean, eslint 0 errors and no boundary violation. Not re-tested on a device — no Android hardware attached to this machine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>VC-049</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Email-prompt bottom sheet reappears on every login even when an email is already saved</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>dev branch, 2026-09-13</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>profileGate.test.ts: VC-049</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr"/>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>Not independently tested</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
         <is>
           <t>FIX (root-caused): the email is NOT a directory-profile field — profileShape.ts states it is a separately-verified identifier owned by the auth-service (GET /auth/account). useProfileGate decided purely from the LOCAL MMKV mirror, and purgeAccountData() wipes KVKeys.email on every sign-out, so immediately after any login the mirror is empty and the gate prompted unconditionally. useAccountInfo() does fetch the real email and mirror it, but it runs in parallel from AppTabs, so its answer always lost the race — and dismissal is session-only, which is why it returned every single login. The gate now asks the auth-service itself before deciding, via a new pure shouldPromptForProfile() (features/user/model/profileGate.ts): a mirrored email means never prompt; a server email means never prompt (and is re-mirrored so later launches short-circuit with no network); an UNANSWERED server (in flight or unreachable) means WAIT rather than prompt, which also removes the flash of the sheet before the answer lands. Only a definitive server no-email prompts. Verified: full jest suite 492/492 pass (5 new decision tests), tsc --noEmit clean, eslint 0 errors, no eslint-plugin-boundaries violation for the user→auth import (authApi depends only on infra, so no cycle). Not reproduced on a device — no Android hardware attached to this machine; fix is verified at the unit level against the exact reported condition.</t>
         </is>

</xml_diff>

<commit_message>
chore(qa): regenerate report for VC-038
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA/reports/VelChat-QA-Report.xlsx
+++ b/QA/reports/VelChat-QA-Report.xlsx
@@ -629,7 +629,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-13 15:30 UTC</t>
+          <t>Generated 2026-09-13 15:47 UTC</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -16405,7 +16405,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr">
@@ -16504,7 +16504,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AA39" s="5" t="inlineStr"/>
+      <c r="AA39" s="5" t="inlineStr">
+        <is>
+          <t>FIX (root cause found by instrumentation, not guesswork): --detectOpenHandles reported NOTHING, so the leak was invisible to it. A probe dumping process.getActiveResourcesInfo() in afterAll showed four live Timeouts while _getActiveHandles() was empty. Traced to WatermelonDB: adapters/lokijs/worker/lokiExtensions.js constructs the Loki database with autosave:true, autosaveInterval:500 — a 500ms setInterval that is only ever cleared by loki.close(), which the app never calls because its database lives for the life of the process. Correct in production (which uses the real native SQLite adapter and never sees this code) but under Jest that interval outlives the run and holds the worker event loop open. Fixed at the source by passing extraLokiOptions:{autosave:false} to the LokiJSAdapter mock in jest.setup.ts — a first-class documented adapter option that WatermelonDB spreads AFTER its own defaults, so it overrides them; there is nothing to autosave in an in-memory adapter that starts fresh every run. MEASURED before/after with the same command: a DB-touching suite went from never exiting (killed at 90-120s, exit 124) to exit 0, and the full suite from blowing past a 120s timeout to completing and exiting in ~18s — --forceExit is no longer needed. RESIDUAL, stated honestly: the "worker process has failed to exit gracefully" text can still appear with &gt;=2 jest workers. That is worker-pool teardown timing, not a leak in our test code — verified by the warning being absent at --maxWorkers=1 (35s) and absent for every heavy suite run individually (failureScenarios, restart, realtime-hardening all clean), while present at --maxWorkers=2 (19s) and 4 (12s). Verified: full jest suite 506/506 pass, tsc --noEmit clean, eslint clean.</t>
+        </is>
+      </c>
       <c r="AB39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
@@ -18234,7 +18238,7 @@
         </is>
       </c>
       <c r="B18" s="22" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C18" s="23" t="inlineStr"/>
     </row>
@@ -18245,7 +18249,7 @@
         </is>
       </c>
       <c r="B19" s="22" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C19" s="23" t="inlineStr"/>
     </row>
@@ -18772,7 +18776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -19590,17 +19594,17 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>VC-047</t>
+          <t>VC-038</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Chat List shows the registered VelChat name instead of the saved contact name until a chat is opened</t>
+          <t>Jest reports a worker that failed to exit gracefully — a leaked timer or handle in the test path</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -19610,7 +19614,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>peerDisplayName.test.ts: VC-044 / VC-047, conversationRow.test.ts: VC-044 / VC-047</t>
+          <t>VC-UNIT-001</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr"/>
@@ -19621,24 +19625,24 @@
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>FIX (root-caused): the address book was consulted on exactly ONE path. startDm() writes the saved name when a chat is opened from New Chat / Message Yourself — which is why the name corrected itself after opening — while every other path used server data, and refreshPeerIdentity() actively OVERWROTE a saved name with the registered one on its next background revalidation (once per TTL/session). Introduced peerDisplayName() (features/contacts/model), the single precedence rule: the name YOU saved wins over the name the peer registered; falls back to the registered name for someone not in your book or when the book has not loaded; returns undefined when neither side has a usable name so callers keep what they have; group rows are untouched (no peerId to look up). Applied at both the WRITE side (refreshPeerIdentity, both the TTL path and the profile-changed push, so a revalidation can no longer downgrade a saved name) and the READ side (toConversationRow for the chat list, useConversationIdentity for the chat header), the latter being what makes a saved name appear WITHOUT having to open the chat first. Exposed discoveredContacts() from the contacts barrel as a cache read (no re-discovery). Verified: full jest suite 502/502 pass (10 new tests), tsc --noEmit clean, eslint 0 errors and no boundary violation. Not re-tested on a device — no Android hardware attached to this machine.</t>
+          <t>FIX (root cause found by instrumentation, not guesswork): --detectOpenHandles reported NOTHING, so the leak was invisible to it. A probe dumping process.getActiveResourcesInfo() in afterAll showed four live Timeouts while _getActiveHandles() was empty. Traced to WatermelonDB: adapters/lokijs/worker/lokiExtensions.js constructs the Loki database with autosave:true, autosaveInterval:500 — a 500ms setInterval that is only ever cleared by loki.close(), which the app never calls because its database lives for the life of the process. Correct in production (which uses the real native SQLite adapter and never sees this code) but under Jest that interval outlives the run and holds the worker event loop open. Fixed at the source by passing extraLokiOptions:{autosave:false} to the LokiJSAdapter mock in jest.setup.ts — a first-class documented adapter option that WatermelonDB spreads AFTER its own defaults, so it overrides them; there is nothing to autosave in an in-memory adapter that starts fresh every run. MEASURED before/after with the same command: a DB-touching suite went from never exiting (killed at 90-120s, exit 124) to exit 0, and the full suite from blowing past a 120s timeout to completing and exiting in ~18s — --forceExit is no longer needed. RESIDUAL, stated honestly: the "worker process has failed to exit gracefully" text can still appear with &gt;=2 jest workers. That is worker-pool teardown timing, not a leak in our test code — verified by the warning being absent at --maxWorkers=1 (35s) and absent for every heavy suite run individually (failureScenarios, restart, realtime-hardening all clean), while present at --maxWorkers=2 (19s) and 4 (12s). Verified: full jest suite 506/506 pass, tsc --noEmit clean, eslint clean.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>VC-049</t>
+          <t>VC-047</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Email-prompt bottom sheet reappears on every login even when an email is already saved</t>
+          <t>Chat List shows the registered VelChat name instead of the saved contact name until a chat is opened</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
@@ -19648,7 +19652,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>profileGate.test.ts: VC-049</t>
+          <t>peerDisplayName.test.ts: VC-044 / VC-047, conversationRow.test.ts: VC-044 / VC-047</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr"/>
@@ -19658,6 +19662,44 @@
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>FIX (root-caused): the address book was consulted on exactly ONE path. startDm() writes the saved name when a chat is opened from New Chat / Message Yourself — which is why the name corrected itself after opening — while every other path used server data, and refreshPeerIdentity() actively OVERWROTE a saved name with the registered one on its next background revalidation (once per TTL/session). Introduced peerDisplayName() (features/contacts/model), the single precedence rule: the name YOU saved wins over the name the peer registered; falls back to the registered name for someone not in your book or when the book has not loaded; returns undefined when neither side has a usable name so callers keep what they have; group rows are untouched (no peerId to look up). Applied at both the WRITE side (refreshPeerIdentity, both the TTL path and the profile-changed push, so a revalidation can no longer downgrade a saved name) and the READ side (toConversationRow for the chat list, useConversationIdentity for the chat header), the latter being what makes a saved name appear WITHOUT having to open the chat first. Exposed discoveredContacts() from the contacts barrel as a cache read (no re-discovery). Verified: full jest suite 502/502 pass (10 new tests), tsc --noEmit clean, eslint 0 errors and no boundary violation. Not re-tested on a device — no Android hardware attached to this machine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>VC-049</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Email-prompt bottom sheet reappears on every login even when an email is already saved</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>dev branch, 2026-09-13</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>profileGate.test.ts: VC-049</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr"/>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Not independently tested</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
         <is>
           <t>FIX (root-caused): the email is NOT a directory-profile field — profileShape.ts states it is a separately-verified identifier owned by the auth-service (GET /auth/account). useProfileGate decided purely from the LOCAL MMKV mirror, and purgeAccountData() wipes KVKeys.email on every sign-out, so immediately after any login the mirror is empty and the gate prompted unconditionally. useAccountInfo() does fetch the real email and mirror it, but it runs in parallel from AppTabs, so its answer always lost the race — and dismissal is session-only, which is why it returned every single login. The gate now asks the auth-service itself before deciding, via a new pure shouldPromptForProfile() (features/user/model/profileGate.ts): a mirrored email means never prompt; a server email means never prompt (and is re-mirrored so later launches short-circuit with no network); an UNANSWERED server (in flight or unreachable) means WAIT rather than prompt, which also removes the flash of the sheet before the answer lands. Only a definitive server no-email prompts. Verified: full jest suite 492/492 pass (5 new decision tests), tsc --noEmit clean, eslint 0 errors, no eslint-plugin-boundaries violation for the user→auth import (authApi depends only on infra, so no cycle). Not reproduced on a device — no Android hardware attached to this machine; fix is verified at the unit level against the exact reported condition.</t>
         </is>

</xml_diff>

<commit_message>
chore(qa): record VC-046 presence-latency analysis
Left open: the client poll is correct (leading fetch, scoped to the open
chat). The ~20s online / ~50s offline latency is the 20s poll plus the
30s server-side TTL expiry, with no presence fan-out to listen for. The
real fix is backend; the only client lever trades battery for latency
and is a product call.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA/reports/VelChat-QA-Report.xlsx
+++ b/QA/reports/VelChat-QA-Report.xlsx
@@ -629,7 +629,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-13 15:47 UTC</t>
+          <t>Generated 2026-09-13 15:49 UTC</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -17588,12 +17588,12 @@
       </c>
       <c r="U47" s="5" t="inlineStr">
         <is>
-          <t>Not yet investigated — could be a client-side polling/debounce delay or a backend presence-propagation delay.</t>
+          <t>Polling + server TTL, because the backend has no presence push. Not a client defect.</t>
         </is>
       </c>
       <c r="V47" s="5" t="inlineStr">
         <is>
-          <t>Not yet investigated.</t>
+          <t>Root-caused, but the fix is NOT client-side. Quantified below.</t>
         </is>
       </c>
       <c r="W47" s="5" t="inlineStr"/>
@@ -17614,7 +17614,7 @@
       </c>
       <c r="AA47" s="5" t="inlineStr">
         <is>
-          <t>Reported by Tusha Bhadouriya during production QA testing. Root cause (client vs backend) not yet isolated.</t>
+          <t>INVESTIGATED — left OPEN deliberately, no code change. The client side is already correct: activatePresence() does a LEADING await refreshPeerPresence() before it starts the interval, so there is no missing first read, and the poll is correctly scoped to the open chat and paused when suspended/offline (§M13 battery). The delay is architectural and has two additive parts. (1) There is NO live presence push to wait for: the realtime gateway FanoutConsumer subscribes to message/receipt/caption only, never presence.changed, so a presence change cannot reach a socket — this is already documented at the top of infra/network/presence.ts and is why a REST snapshot poll exists at all. (2) The numbers: peer COMES ONLINE is seen at the next poll, PEER_PRESENCE_POLL_MS = 20s, so up to ~20s. Peer GOES OFFLINE is worse, because nobody publishes a leaving event — their online:{userId} Redis key has to EXPIRE server-side (PRESENCE_ONLINE_TTL_MS = 30s from their last 20s heartbeat) and only then can our next poll observe it, so up to ~50s. That matches the reported "noticeable delay" exactly. THE REAL FIX IS BACKEND: have the gateway fan out presence.changed over the WS; the client already has the receiving path (onInboundPresence + normalizePresenceEvent are written and forward-compatible), so it would light up with no client change. The only client-side lever is lowering PEER_PRESENCE_POLL_MS, which buys latency with a REST request per interval per open chat and is a direct trade against the §R5/§R6 battery and request budgets on the 3GB reference device — a product call, not one to make silently, so it is NOT done here. Needs a decision: accept the delay, lower the poll interval (say what latency is acceptable), or schedule the backend fan-out.</t>
         </is>
       </c>
       <c r="AB47" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore(qa): re-verification run against a live backend
92 API/WS/two-device tests: 78 pass, 14 fail. Every failure maps to an
already-filed BACKEND bug (VC-001/002/003/004/005/006/039/040/041/042) —
no new defects and nothing client-side. Flaky detector flags VC-AUTH-027
and VC-RT-030, both symptoms of filed races (VC-043, VC-002) rather than
separate issues.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA/reports/VelChat-QA-Report.xlsx
+++ b/QA/reports/VelChat-QA-Report.xlsx
@@ -30,7 +30,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -66,6 +66,10 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="009A3412"/>
+    </font>
+    <font>
+      <b val="1"/>
       <i val="1"/>
       <color rgb="001E3A8A"/>
     </font>
@@ -98,7 +102,7 @@
       <color rgb="0092400E"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -118,6 +122,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FEE2E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEDD5"/>
       </patternFill>
     </fill>
     <fill>
@@ -172,7 +181,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -203,40 +212,43 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -629,7 +641,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-13 15:49 UTC</t>
+          <t>Generated 2026-09-13 16:07 UTC</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -1981,9 +1993,9 @@
           <t>node-harness</t>
         </is>
       </c>
-      <c r="C40" s="10" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="C40" s="12" t="inlineStr">
+        <is>
+          <t>FLAKY</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -1993,7 +2005,7 @@
       </c>
       <c r="E40" s="8" t="inlineStr">
         <is>
-          <t>Logs + Repro script</t>
+          <t>Logs</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
@@ -2795,7 +2807,7 @@
           <t>node-harness</t>
         </is>
       </c>
-      <c r="C62" s="12" t="inlineStr">
+      <c r="C62" s="13" t="inlineStr">
         <is>
           <t>PASS (verified from phone by Aayush)</t>
         </is>
@@ -2869,19 +2881,19 @@
           <t>node-harness</t>
         </is>
       </c>
-      <c r="C64" s="7" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="D64" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C64" s="12" t="inlineStr">
+        <is>
+          <t>FLAKY</t>
+        </is>
+      </c>
+      <c r="D64" s="11" t="inlineStr">
+        <is>
+          <t>VC-002</t>
         </is>
       </c>
       <c r="E64" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Logs</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
@@ -4257,11 +4269,11 @@
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:08:23</t>
+          <t>2026-09-13 16:05:03</t>
         </is>
       </c>
       <c r="N2" s="5" t="n">
-        <v>1061</v>
+        <v>1232</v>
       </c>
       <c r="O2" s="5" t="inlineStr">
         <is>
@@ -4330,11 +4342,11 @@
       </c>
       <c r="M3" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:08:24</t>
+          <t>2026-09-13 16:05:04</t>
         </is>
       </c>
       <c r="N3" s="5" t="n">
-        <v>810</v>
+        <v>939</v>
       </c>
       <c r="O3" s="5" t="inlineStr">
         <is>
@@ -4407,11 +4419,11 @@
       </c>
       <c r="M4" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:08:27</t>
+          <t>2026-09-13 16:05:08</t>
         </is>
       </c>
       <c r="N4" s="5" t="n">
-        <v>3579</v>
+        <v>3920</v>
       </c>
       <c r="O4" s="5" t="inlineStr">
         <is>
@@ -4482,11 +4494,11 @@
       </c>
       <c r="M5" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:08:34</t>
+          <t>2026-09-13 16:05:15</t>
         </is>
       </c>
       <c r="N5" s="5" t="n">
-        <v>6413</v>
+        <v>6483</v>
       </c>
       <c r="O5" s="5" t="inlineStr">
         <is>
@@ -4558,11 +4570,11 @@
       </c>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:08:36</t>
+          <t>2026-09-13 16:05:17</t>
         </is>
       </c>
       <c r="N6" s="5" t="n">
-        <v>2393</v>
+        <v>2484</v>
       </c>
       <c r="O6" s="5" t="inlineStr">
         <is>
@@ -4632,11 +4644,11 @@
       </c>
       <c r="M7" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:08:39</t>
+          <t>2026-09-13 16:05:20</t>
         </is>
       </c>
       <c r="N7" s="5" t="n">
-        <v>2533</v>
+        <v>2437</v>
       </c>
       <c r="O7" s="5" t="inlineStr">
         <is>
@@ -4706,11 +4718,11 @@
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:08:39</t>
+          <t>2026-09-13 16:05:20</t>
         </is>
       </c>
       <c r="N8" s="5" t="n">
-        <v>379</v>
+        <v>484</v>
       </c>
       <c r="O8" s="5" t="inlineStr">
         <is>
@@ -4779,11 +4791,11 @@
       </c>
       <c r="M9" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:08:42</t>
+          <t>2026-09-13 16:05:23</t>
         </is>
       </c>
       <c r="N9" s="5" t="n">
-        <v>3016</v>
+        <v>3160</v>
       </c>
       <c r="O9" s="5" t="inlineStr">
         <is>
@@ -4852,11 +4864,11 @@
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:08:48</t>
+          <t>2026-09-13 16:05:33</t>
         </is>
       </c>
       <c r="N10" s="5" t="n">
-        <v>5807</v>
+        <v>9469</v>
       </c>
       <c r="O10" s="5" t="inlineStr">
         <is>
@@ -4924,11 +4936,11 @@
       </c>
       <c r="M11" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:08:53</t>
+          <t>2026-09-13 16:05:41</t>
         </is>
       </c>
       <c r="N11" s="5" t="n">
-        <v>4937</v>
+        <v>6752</v>
       </c>
       <c r="O11" s="5" t="inlineStr">
         <is>
@@ -4996,11 +5008,11 @@
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:08:58</t>
+          <t>2026-09-13 16:05:50</t>
         </is>
       </c>
       <c r="N12" s="5" t="n">
-        <v>5297</v>
+        <v>9615</v>
       </c>
       <c r="O12" s="5" t="inlineStr">
         <is>
@@ -5069,11 +5081,11 @@
       </c>
       <c r="M13" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:08:59</t>
+          <t>2026-09-13 16:05:51</t>
         </is>
       </c>
       <c r="N13" s="5" t="n">
-        <v>650</v>
+        <v>567</v>
       </c>
       <c r="O13" s="5" t="inlineStr">
         <is>
@@ -5121,7 +5133,7 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="I14" s="13" t="inlineStr">
+      <c r="I14" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -5143,11 +5155,11 @@
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:08:59</t>
+          <t>2026-09-13 16:05:51</t>
         </is>
       </c>
       <c r="N14" s="5" t="n">
-        <v>270</v>
+        <v>361</v>
       </c>
       <c r="O14" s="5" t="inlineStr">
         <is>
@@ -5197,7 +5209,7 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="I15" s="14" t="inlineStr">
+      <c r="I15" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -5219,11 +5231,11 @@
       </c>
       <c r="M15" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:09:00</t>
+          <t>2026-09-13 16:05:52</t>
         </is>
       </c>
       <c r="N15" s="5" t="n">
-        <v>321</v>
+        <v>357</v>
       </c>
       <c r="O15" s="5" t="inlineStr">
         <is>
@@ -5297,11 +5309,11 @@
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:09</t>
+          <t>2026-09-13 16:03:01</t>
         </is>
       </c>
       <c r="N16" s="5" t="n">
-        <v>370</v>
+        <v>448</v>
       </c>
       <c r="O16" s="5" t="inlineStr">
         <is>
@@ -5369,7 +5381,7 @@
       </c>
       <c r="M17" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:09</t>
+          <t>2026-09-13 16:03:01</t>
         </is>
       </c>
       <c r="N17" s="5" t="n">
@@ -5419,7 +5431,7 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="I18" s="14" t="inlineStr">
+      <c r="I18" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -5441,11 +5453,11 @@
       </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:09</t>
+          <t>2026-09-13 16:03:01</t>
         </is>
       </c>
       <c r="N18" s="5" t="n">
-        <v>279</v>
+        <v>217</v>
       </c>
       <c r="O18" s="5" t="inlineStr">
         <is>
@@ -5495,7 +5507,7 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="I19" s="13" t="inlineStr">
+      <c r="I19" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -5517,11 +5529,11 @@
       </c>
       <c r="M19" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:10</t>
+          <t>2026-09-13 16:03:01</t>
         </is>
       </c>
       <c r="N19" s="5" t="n">
-        <v>397</v>
+        <v>409</v>
       </c>
       <c r="O19" s="5" t="inlineStr">
         <is>
@@ -5593,11 +5605,11 @@
       </c>
       <c r="M20" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:10</t>
+          <t>2026-09-13 16:03:01</t>
         </is>
       </c>
       <c r="N20" s="5" t="n">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="O20" s="5" t="inlineStr">
         <is>
@@ -5665,11 +5677,11 @@
       </c>
       <c r="M21" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:10</t>
+          <t>2026-09-13 16:03:01</t>
         </is>
       </c>
       <c r="N21" s="5" t="n">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="O21" s="5" t="inlineStr">
         <is>
@@ -5739,11 +5751,11 @@
       </c>
       <c r="M22" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:12</t>
+          <t>2026-09-13 16:03:03</t>
         </is>
       </c>
       <c r="N22" s="5" t="n">
-        <v>1722</v>
+        <v>1541</v>
       </c>
       <c r="O22" s="5" t="inlineStr">
         <is>
@@ -5812,11 +5824,11 @@
       </c>
       <c r="M23" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:13</t>
+          <t>2026-09-13 16:03:04</t>
         </is>
       </c>
       <c r="N23" s="5" t="n">
-        <v>1409</v>
+        <v>1545</v>
       </c>
       <c r="O23" s="5" t="inlineStr">
         <is>
@@ -5885,11 +5897,11 @@
       </c>
       <c r="M24" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:13</t>
+          <t>2026-09-13 16:03:05</t>
         </is>
       </c>
       <c r="N24" s="5" t="n">
-        <v>364</v>
+        <v>420</v>
       </c>
       <c r="O24" s="5" t="inlineStr">
         <is>
@@ -5957,11 +5969,11 @@
       </c>
       <c r="M25" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:14</t>
+          <t>2026-09-13 16:03:05</t>
         </is>
       </c>
       <c r="N25" s="5" t="n">
-        <v>315</v>
+        <v>341</v>
       </c>
       <c r="O25" s="5" t="inlineStr">
         <is>
@@ -6029,11 +6041,11 @@
       </c>
       <c r="M26" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:14</t>
+          <t>2026-09-13 16:03:06</t>
         </is>
       </c>
       <c r="N26" s="5" t="n">
-        <v>321</v>
+        <v>370</v>
       </c>
       <c r="O26" s="5" t="inlineStr">
         <is>
@@ -6101,11 +6113,11 @@
       </c>
       <c r="M27" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:14</t>
+          <t>2026-09-13 16:03:06</t>
         </is>
       </c>
       <c r="N27" s="5" t="n">
-        <v>334</v>
+        <v>376</v>
       </c>
       <c r="O27" s="5" t="inlineStr">
         <is>
@@ -6173,11 +6185,11 @@
       </c>
       <c r="M28" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:15</t>
+          <t>2026-09-13 16:03:06</t>
         </is>
       </c>
       <c r="N28" s="5" t="n">
-        <v>306</v>
+        <v>347</v>
       </c>
       <c r="O28" s="5" t="inlineStr">
         <is>
@@ -6245,11 +6257,11 @@
       </c>
       <c r="M29" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:15</t>
+          <t>2026-09-13 16:03:06</t>
         </is>
       </c>
       <c r="N29" s="5" t="n">
-        <v>63</v>
+        <v>89</v>
       </c>
       <c r="O29" s="5" t="inlineStr">
         <is>
@@ -6319,11 +6331,11 @@
       </c>
       <c r="M30" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:17</t>
+          <t>2026-09-13 16:03:09</t>
         </is>
       </c>
       <c r="N30" s="5" t="n">
-        <v>583</v>
+        <v>752</v>
       </c>
       <c r="O30" s="5" t="inlineStr">
         <is>
@@ -6393,11 +6405,11 @@
       </c>
       <c r="M31" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:17</t>
+          <t>2026-09-13 16:03:09</t>
         </is>
       </c>
       <c r="N31" s="5" t="n">
-        <v>255</v>
+        <v>305</v>
       </c>
       <c r="O31" s="5" t="inlineStr">
         <is>
@@ -6467,11 +6479,11 @@
       </c>
       <c r="M32" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:18</t>
+          <t>2026-09-13 16:03:10</t>
         </is>
       </c>
       <c r="N32" s="5" t="n">
-        <v>804</v>
+        <v>867</v>
       </c>
       <c r="O32" s="5" t="inlineStr">
         <is>
@@ -6539,11 +6551,11 @@
       </c>
       <c r="M33" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:20</t>
+          <t>2026-09-13 16:03:12</t>
         </is>
       </c>
       <c r="N33" s="5" t="n">
-        <v>1855</v>
+        <v>2000</v>
       </c>
       <c r="O33" s="5" t="inlineStr">
         <is>
@@ -6614,11 +6626,11 @@
       </c>
       <c r="M34" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:22</t>
+          <t>2026-09-13 16:03:14</t>
         </is>
       </c>
       <c r="N34" s="5" t="n">
-        <v>2243</v>
+        <v>2451</v>
       </c>
       <c r="O34" s="5" t="inlineStr">
         <is>
@@ -6686,11 +6698,11 @@
       </c>
       <c r="M35" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:22</t>
+          <t>2026-09-13 16:03:14</t>
         </is>
       </c>
       <c r="N35" s="5" t="n">
-        <v>102</v>
+        <v>136</v>
       </c>
       <c r="O35" s="5" t="inlineStr">
         <is>
@@ -6760,11 +6772,11 @@
       </c>
       <c r="M36" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:24</t>
+          <t>2026-09-13 16:03:16</t>
         </is>
       </c>
       <c r="N36" s="5" t="n">
-        <v>1736</v>
+        <v>1931</v>
       </c>
       <c r="O36" s="5" t="inlineStr">
         <is>
@@ -6803,17 +6815,17 @@
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>at most one concurrent refresh may succeed; 3 of 3 did</t>
-        </is>
-      </c>
-      <c r="H37" s="10" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="I37" s="14" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>As expected</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="J37" s="5" t="inlineStr">
@@ -6833,11 +6845,11 @@
       </c>
       <c r="M37" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:25</t>
+          <t>2026-09-13 16:03:19</t>
         </is>
       </c>
       <c r="N37" s="5" t="n">
-        <v>1724</v>
+        <v>2346</v>
       </c>
       <c r="O37" s="5" t="inlineStr">
         <is>
@@ -6909,11 +6921,11 @@
       </c>
       <c r="M38" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:26</t>
+          <t>2026-09-13 16:03:19</t>
         </is>
       </c>
       <c r="N38" s="5" t="n">
-        <v>181</v>
+        <v>22</v>
       </c>
       <c r="O38" s="5" t="inlineStr">
         <is>
@@ -6981,11 +6993,11 @@
       </c>
       <c r="M39" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:26</t>
+          <t>2026-09-13 16:03:19</t>
         </is>
       </c>
       <c r="N39" s="5" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="O39" s="5" t="inlineStr">
         <is>
@@ -7054,11 +7066,11 @@
       </c>
       <c r="M40" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:26</t>
+          <t>2026-09-13 16:03:19</t>
         </is>
       </c>
       <c r="N40" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="O40" s="5" t="inlineStr">
         <is>
@@ -7127,11 +7139,11 @@
       </c>
       <c r="M41" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:26</t>
+          <t>2026-09-13 16:03:19</t>
         </is>
       </c>
       <c r="N41" s="5" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="O41" s="5" t="inlineStr">
         <is>
@@ -7200,11 +7212,11 @@
       </c>
       <c r="M42" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:27</t>
+          <t>2026-09-13 16:03:20</t>
         </is>
       </c>
       <c r="N42" s="5" t="n">
-        <v>1573</v>
+        <v>1530</v>
       </c>
       <c r="O42" s="5" t="inlineStr">
         <is>
@@ -7272,11 +7284,11 @@
       </c>
       <c r="M43" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:27</t>
+          <t>2026-09-13 16:03:20</t>
         </is>
       </c>
       <c r="N43" s="5" t="n">
-        <v>122</v>
+        <v>135</v>
       </c>
       <c r="O43" s="5" t="inlineStr">
         <is>
@@ -7344,7 +7356,7 @@
       </c>
       <c r="M44" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:27</t>
+          <t>2026-09-13 16:03:20</t>
         </is>
       </c>
       <c r="N44" s="5" t="n">
@@ -7416,11 +7428,11 @@
       </c>
       <c r="M45" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:27</t>
+          <t>2026-09-13 16:03:20</t>
         </is>
       </c>
       <c r="N45" s="5" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="O45" s="5" t="inlineStr">
         <is>
@@ -7490,11 +7502,11 @@
       </c>
       <c r="M46" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:23</t>
+          <t>2026-09-13 16:03:53</t>
         </is>
       </c>
       <c r="N46" s="5" t="n">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="O46" s="5" t="inlineStr">
         <is>
@@ -7562,11 +7574,11 @@
       </c>
       <c r="M47" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:23</t>
+          <t>2026-09-13 16:03:53</t>
         </is>
       </c>
       <c r="N47" s="5" t="n">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="O47" s="5" t="inlineStr">
         <is>
@@ -7634,11 +7646,11 @@
       </c>
       <c r="M48" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:23</t>
+          <t>2026-09-13 16:03:53</t>
         </is>
       </c>
       <c r="N48" s="5" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="O48" s="5" t="inlineStr">
         <is>
@@ -7707,7 +7719,7 @@
       </c>
       <c r="M49" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:23</t>
+          <t>2026-09-13 16:03:53</t>
         </is>
       </c>
       <c r="N49" s="5" t="n">
@@ -7780,11 +7792,11 @@
       </c>
       <c r="M50" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:24</t>
+          <t>2026-09-13 16:03:53</t>
         </is>
       </c>
       <c r="N50" s="5" t="n">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="O50" s="5" t="inlineStr">
         <is>
@@ -7853,11 +7865,11 @@
       </c>
       <c r="M51" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:24</t>
+          <t>2026-09-13 16:03:53</t>
         </is>
       </c>
       <c r="N51" s="5" t="n">
-        <v>239</v>
+        <v>260</v>
       </c>
       <c r="O51" s="5" t="inlineStr">
         <is>
@@ -7926,11 +7938,11 @@
       </c>
       <c r="M52" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:24</t>
+          <t>2026-09-13 16:03:53</t>
         </is>
       </c>
       <c r="N52" s="5" t="n">
-        <v>122</v>
+        <v>138</v>
       </c>
       <c r="O52" s="5" t="inlineStr">
         <is>
@@ -7998,11 +8010,11 @@
       </c>
       <c r="M53" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:24</t>
+          <t>2026-09-13 16:03:54</t>
         </is>
       </c>
       <c r="N53" s="5" t="n">
-        <v>260</v>
+        <v>241</v>
       </c>
       <c r="O53" s="5" t="inlineStr">
         <is>
@@ -8070,11 +8082,11 @@
       </c>
       <c r="M54" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:24</t>
+          <t>2026-09-13 16:03:54</t>
         </is>
       </c>
       <c r="N54" s="5" t="n">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="O54" s="5" t="inlineStr">
         <is>
@@ -8142,11 +8154,11 @@
       </c>
       <c r="M55" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:25</t>
+          <t>2026-09-13 16:03:54</t>
         </is>
       </c>
       <c r="N55" s="5" t="n">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="O55" s="5" t="inlineStr">
         <is>
@@ -8214,11 +8226,11 @@
       </c>
       <c r="M56" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:25</t>
+          <t>2026-09-13 16:03:54</t>
         </is>
       </c>
       <c r="N56" s="5" t="n">
-        <v>238</v>
+        <v>255</v>
       </c>
       <c r="O56" s="5" t="inlineStr">
         <is>
@@ -8288,11 +8300,11 @@
       </c>
       <c r="M57" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:31</t>
+          <t>2026-09-13 16:04:00</t>
         </is>
       </c>
       <c r="N57" s="5" t="n">
-        <v>5753</v>
+        <v>5246</v>
       </c>
       <c r="O57" s="5" t="inlineStr">
         <is>
@@ -8361,11 +8373,11 @@
       </c>
       <c r="M58" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:32</t>
+          <t>2026-09-13 16:04:01</t>
         </is>
       </c>
       <c r="N58" s="5" t="n">
-        <v>1143</v>
+        <v>1051</v>
       </c>
       <c r="O58" s="5" t="inlineStr">
         <is>
@@ -8416,19 +8428,19 @@
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">DURABLE MESSAGE LOSS: REST acked seqs [2,3,4,5,6,7,8,9,10,11] but the recipient's socket only received [4,6,9] — missing [2,3,5,7,8,10,11]. Durable frames must never be dropped.
+          <t xml:space="preserve">DURABLE MESSAGE LOSS: REST acked seqs [2,3,4,5,6,7,8,9,10,11] but the recipient's socket only received [2,5,8,11] — missing [3,4,6,7,9,10]. Durable frames must never be dropped.
 + actual - expected
   [
--   2,
+    2,
 -   3,
-    4,
--   5,
-    6,
+-   4,
+    5,
+-   6,
 -   7,
--   8,
-    9,
+    8,
+-   9,
 -   10,
--   11
+    11
   ]
 </t>
         </is>
@@ -8438,7 +8450,7 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="I59" s="15" t="inlineStr">
+      <c r="I59" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -8460,11 +8472,11 @@
       </c>
       <c r="M59" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:41</t>
+          <t>2026-09-13 16:04:10</t>
         </is>
       </c>
       <c r="N59" s="5" t="n">
-        <v>9342</v>
+        <v>9044</v>
       </c>
       <c r="O59" s="5" t="inlineStr">
         <is>
@@ -8539,11 +8551,11 @@
       </c>
       <c r="M60" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:43</t>
+          <t>2026-09-13 16:04:12</t>
         </is>
       </c>
       <c r="N60" s="5" t="n">
-        <v>1285</v>
+        <v>1523</v>
       </c>
       <c r="O60" s="5" t="inlineStr">
         <is>
@@ -8588,17 +8600,17 @@
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>As expected</t>
-        </is>
-      </c>
-      <c r="H61" s="7" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="I61" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>[VC-RT-030-A] timed out after 10000ms awaiting delivered receipt for seq 17</t>
+        </is>
+      </c>
+      <c r="H61" s="10" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="I61" s="16" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="J61" s="5" t="inlineStr">
@@ -8618,11 +8630,11 @@
       </c>
       <c r="M61" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:44</t>
+          <t>2026-09-13 16:04:22</t>
         </is>
       </c>
       <c r="N61" s="5" t="n">
-        <v>1095</v>
+        <v>10398</v>
       </c>
       <c r="O61" s="5" t="inlineStr">
         <is>
@@ -8674,7 +8686,7 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="I62" s="15" t="inlineStr">
+      <c r="I62" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -8696,11 +8708,11 @@
       </c>
       <c r="M62" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:54</t>
+          <t>2026-09-13 16:04:33</t>
         </is>
       </c>
       <c r="N62" s="5" t="n">
-        <v>10395</v>
+        <v>10409</v>
       </c>
       <c r="O62" s="5" t="inlineStr">
         <is>
@@ -8757,7 +8769,7 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="I63" s="15" t="inlineStr">
+      <c r="I63" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -8779,11 +8791,11 @@
       </c>
       <c r="M63" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:08:00</t>
+          <t>2026-09-13 16:04:38</t>
         </is>
       </c>
       <c r="N63" s="5" t="n">
-        <v>5418</v>
+        <v>5467</v>
       </c>
       <c r="O63" s="5" t="inlineStr">
         <is>
@@ -8857,11 +8869,11 @@
       </c>
       <c r="M64" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:08:01</t>
+          <t>2026-09-13 16:04:40</t>
         </is>
       </c>
       <c r="N64" s="5" t="n">
-        <v>1649</v>
+        <v>1664</v>
       </c>
       <c r="O64" s="5" t="inlineStr">
         <is>
@@ -8929,11 +8941,11 @@
       </c>
       <c r="M65" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:08:06</t>
+          <t>2026-09-13 16:04:45</t>
         </is>
       </c>
       <c r="N65" s="5" t="n">
-        <v>4907</v>
+        <v>4981</v>
       </c>
       <c r="O65" s="5" t="inlineStr">
         <is>
@@ -8983,7 +8995,7 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="I66" s="15" t="inlineStr">
+      <c r="I66" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -9005,11 +9017,11 @@
       </c>
       <c r="M66" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:08:12</t>
+          <t>2026-09-13 16:04:51</t>
         </is>
       </c>
       <c r="N66" s="5" t="n">
-        <v>5981</v>
+        <v>6080</v>
       </c>
       <c r="O66" s="5" t="inlineStr">
         <is>
@@ -9082,11 +9094,11 @@
       </c>
       <c r="M67" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:08:13</t>
+          <t>2026-09-13 16:04:52</t>
         </is>
       </c>
       <c r="N67" s="5" t="n">
-        <v>353</v>
+        <v>447</v>
       </c>
       <c r="O67" s="5" t="inlineStr">
         <is>
@@ -9155,11 +9167,11 @@
       </c>
       <c r="M68" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:08:15</t>
+          <t>2026-09-13 16:04:54</t>
         </is>
       </c>
       <c r="N68" s="5" t="n">
-        <v>1815</v>
+        <v>1971</v>
       </c>
       <c r="O68" s="5" t="inlineStr">
         <is>
@@ -9227,11 +9239,11 @@
       </c>
       <c r="M69" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:08:19</t>
+          <t>2026-09-13 16:04:59</t>
         </is>
       </c>
       <c r="N69" s="5" t="n">
-        <v>4527</v>
+        <v>4763</v>
       </c>
       <c r="O69" s="5" t="inlineStr">
         <is>
@@ -9299,11 +9311,11 @@
       </c>
       <c r="M70" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:28</t>
+          <t>2026-09-13 16:03:00</t>
         </is>
       </c>
       <c r="N70" s="5" t="n">
-        <v>90</v>
+        <v>119</v>
       </c>
       <c r="O70" s="5" t="inlineStr">
         <is>
@@ -9371,11 +9383,11 @@
       </c>
       <c r="M71" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:28</t>
+          <t>2026-09-13 16:03:00</t>
         </is>
       </c>
       <c r="N71" s="5" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="O71" s="5" t="inlineStr">
         <is>
@@ -9443,11 +9455,11 @@
       </c>
       <c r="M72" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:28</t>
+          <t>2026-09-13 16:03:00</t>
         </is>
       </c>
       <c r="N72" s="5" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="O72" s="5" t="inlineStr">
         <is>
@@ -9515,11 +9527,11 @@
       </c>
       <c r="M73" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:28</t>
+          <t>2026-09-13 16:03:00</t>
         </is>
       </c>
       <c r="N73" s="5" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="O73" s="5" t="inlineStr">
         <is>
@@ -9588,11 +9600,11 @@
       </c>
       <c r="M74" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:29</t>
+          <t>2026-09-13 16:03:02</t>
         </is>
       </c>
       <c r="N74" s="5" t="n">
-        <v>1352</v>
+        <v>1749</v>
       </c>
       <c r="O74" s="5" t="inlineStr">
         <is>
@@ -9662,11 +9674,11 @@
       </c>
       <c r="M75" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:30</t>
+          <t>2026-09-13 16:03:04</t>
         </is>
       </c>
       <c r="N75" s="5" t="n">
-        <v>1417</v>
+        <v>1497</v>
       </c>
       <c r="O75" s="5" t="inlineStr">
         <is>
@@ -9735,11 +9747,11 @@
       </c>
       <c r="M76" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:30</t>
+          <t>2026-09-13 16:03:04</t>
         </is>
       </c>
       <c r="N76" s="5" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="O76" s="5" t="inlineStr">
         <is>
@@ -9788,7 +9800,7 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="I77" s="15" t="inlineStr">
+      <c r="I77" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -9810,11 +9822,11 @@
       </c>
       <c r="M77" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:34</t>
+          <t>2026-09-13 16:03:08</t>
         </is>
       </c>
       <c r="N77" s="5" t="n">
-        <v>2018</v>
+        <v>2056</v>
       </c>
       <c r="O77" s="5" t="inlineStr">
         <is>
@@ -9888,11 +9900,11 @@
       </c>
       <c r="M78" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:34</t>
+          <t>2026-09-13 16:03:08</t>
         </is>
       </c>
       <c r="N78" s="5" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="O78" s="5" t="inlineStr">
         <is>
@@ -9960,11 +9972,11 @@
       </c>
       <c r="M79" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:34</t>
+          <t>2026-09-13 16:03:08</t>
         </is>
       </c>
       <c r="N79" s="5" t="n">
-        <v>115</v>
+        <v>140</v>
       </c>
       <c r="O79" s="5" t="inlineStr">
         <is>
@@ -10032,11 +10044,11 @@
       </c>
       <c r="M80" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:34</t>
+          <t>2026-09-13 16:03:08</t>
         </is>
       </c>
       <c r="N80" s="5" t="n">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="O80" s="5" t="inlineStr">
         <is>
@@ -10082,7 +10094,7 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="I81" s="14" t="inlineStr">
+      <c r="I81" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -10104,11 +10116,11 @@
       </c>
       <c r="M81" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:34</t>
+          <t>2026-09-13 16:03:08</t>
         </is>
       </c>
       <c r="N81" s="5" t="n">
-        <v>115</v>
+        <v>134</v>
       </c>
       <c r="O81" s="5" t="inlineStr">
         <is>
@@ -10180,11 +10192,11 @@
       </c>
       <c r="M82" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:36</t>
+          <t>2026-09-13 16:03:10</t>
         </is>
       </c>
       <c r="N82" s="5" t="n">
-        <v>1442</v>
+        <v>1502</v>
       </c>
       <c r="O82" s="5" t="inlineStr">
         <is>
@@ -10253,11 +10265,11 @@
       </c>
       <c r="M83" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:38</t>
+          <t>2026-09-13 16:03:12</t>
         </is>
       </c>
       <c r="N83" s="5" t="n">
-        <v>1736</v>
+        <v>1962</v>
       </c>
       <c r="O83" s="5" t="inlineStr">
         <is>
@@ -10326,11 +10338,11 @@
       </c>
       <c r="M84" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:39</t>
+          <t>2026-09-13 16:03:13</t>
         </is>
       </c>
       <c r="N84" s="5" t="n">
-        <v>1768</v>
+        <v>1817</v>
       </c>
       <c r="O84" s="5" t="inlineStr">
         <is>
@@ -10382,7 +10394,7 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="I85" s="14" t="inlineStr">
+      <c r="I85" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -10404,11 +10416,11 @@
       </c>
       <c r="M85" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:40</t>
+          <t>2026-09-13 16:03:14</t>
         </is>
       </c>
       <c r="N85" s="5" t="n">
-        <v>199</v>
+        <v>226</v>
       </c>
       <c r="O85" s="5" t="inlineStr">
         <is>
@@ -10460,7 +10472,7 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="I86" s="14" t="inlineStr">
+      <c r="I86" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -10482,11 +10494,11 @@
       </c>
       <c r="M86" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:40</t>
+          <t>2026-09-13 16:03:14</t>
         </is>
       </c>
       <c r="N86" s="5" t="n">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="O86" s="5" t="inlineStr">
         <is>
@@ -10542,7 +10554,7 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="I87" s="15" t="inlineStr">
+      <c r="I87" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -10564,11 +10576,11 @@
       </c>
       <c r="M87" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:41</t>
+          <t>2026-09-13 16:03:15</t>
         </is>
       </c>
       <c r="N87" s="5" t="n">
-        <v>1288</v>
+        <v>1377</v>
       </c>
       <c r="O87" s="5" t="inlineStr">
         <is>
@@ -10640,11 +10652,11 @@
       </c>
       <c r="M88" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:41</t>
+          <t>2026-09-13 16:03:15</t>
         </is>
       </c>
       <c r="N88" s="5" t="n">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="O88" s="5" t="inlineStr">
         <is>
@@ -10712,11 +10724,11 @@
       </c>
       <c r="M89" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:43</t>
+          <t>2026-09-13 16:03:17</t>
         </is>
       </c>
       <c r="N89" s="5" t="n">
-        <v>1426</v>
+        <v>1579</v>
       </c>
       <c r="O89" s="5" t="inlineStr">
         <is>
@@ -10785,11 +10797,11 @@
       </c>
       <c r="M90" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:43</t>
+          <t>2026-09-13 16:03:17</t>
         </is>
       </c>
       <c r="N90" s="5" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="O90" s="5" t="inlineStr">
         <is>
@@ -10860,11 +10872,11 @@
       </c>
       <c r="M91" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:44</t>
+          <t>2026-09-13 16:03:19</t>
         </is>
       </c>
       <c r="N91" s="5" t="n">
-        <v>1592</v>
+        <v>2349</v>
       </c>
       <c r="O91" s="5" t="inlineStr">
         <is>
@@ -10934,11 +10946,11 @@
       </c>
       <c r="M92" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:46</t>
+          <t>2026-09-13 16:03:21</t>
         </is>
       </c>
       <c r="N92" s="5" t="n">
-        <v>2102</v>
+        <v>2109</v>
       </c>
       <c r="O92" s="5" t="inlineStr">
         <is>
@@ -11006,11 +11018,11 @@
       </c>
       <c r="M93" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11 15:07:48</t>
+          <t>2026-09-13 16:03:23</t>
         </is>
       </c>
       <c r="N93" s="5" t="n">
-        <v>1616</v>
+        <v>1597</v>
       </c>
       <c r="O93" s="5" t="inlineStr">
         <is>
@@ -11207,7 +11219,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="inlineStr">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>VC-001</t>
         </is>
@@ -11227,17 +11239,17 @@
           <t>Realtime fan-out silently drops up to 63% of durable messages sent within ~250ms of each other</t>
         </is>
       </c>
-      <c r="E2" s="15" t="inlineStr">
+      <c r="E2" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr">
+      <c r="F2" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="G2" s="17" t="inlineStr">
+      <c r="G2" s="18" t="inlineStr">
         <is>
           <t>In Progress (Aayush is fixing this now)</t>
         </is>
@@ -11331,12 +11343,12 @@
       </c>
       <c r="X2" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="Y2" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="Z2" s="5" t="inlineStr">
@@ -11352,7 +11364,7 @@
       <c r="AB2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>VC-002</t>
         </is>
@@ -11372,12 +11384,12 @@
           <t>Blue tick never arrives: a `read` receipt sent in the same tick as `delivered` is lost</t>
         </is>
       </c>
-      <c r="E3" s="15" t="inlineStr">
+      <c r="E3" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F3" s="15" t="inlineStr">
+      <c r="F3" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -11472,12 +11484,12 @@
       </c>
       <c r="X3" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="Y3" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="Z3" s="5" t="inlineStr">
@@ -11493,7 +11505,7 @@
       <c r="AB3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>VC-003</t>
         </is>
@@ -11513,12 +11525,12 @@
           <t>Read watermark can regress: the higher receipt is lost and a lower one survives</t>
         </is>
       </c>
-      <c r="E4" s="15" t="inlineStr">
+      <c r="E4" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F4" s="15" t="inlineStr">
+      <c r="F4" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -11614,12 +11626,12 @@
       </c>
       <c r="X4" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="Y4" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="Z4" s="5" t="inlineStr">
@@ -11631,7 +11643,7 @@
       <c r="AB4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>VC-004</t>
         </is>
@@ -11651,12 +11663,12 @@
           <t>POST /auth/register accepts an arbitrary non-phone string and provisions a full account with real tokens</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="E5" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F5" s="14" t="inlineStr">
+      <c r="F5" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -11750,12 +11762,12 @@
       </c>
       <c r="X5" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="Y5" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="Z5" s="5" t="inlineStr">
@@ -11767,7 +11779,7 @@
       <c r="AB5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>VC-005</t>
         </is>
@@ -11787,12 +11799,12 @@
           <t>POST /auth/register accepts a non-base64 device public key, permanently breaking device-key login for that install</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
+      <c r="E6" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F6" s="14" t="inlineStr">
+      <c r="F6" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -11886,12 +11898,12 @@
       </c>
       <c r="X6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="Y6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="Z6" s="5" t="inlineStr">
@@ -11903,7 +11915,7 @@
       <c r="AB6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>VC-006</t>
         </is>
@@ -11923,12 +11935,12 @@
           <t>POST /auth/revotp/webhook is @Public with no shared secret — an unauthenticated account-provisioning primitive</t>
         </is>
       </c>
-      <c r="E7" s="15" t="inlineStr">
+      <c r="E7" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F7" s="15" t="inlineStr">
+      <c r="F7" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -12022,12 +12034,12 @@
       </c>
       <c r="X7" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="Y7" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="Z7" s="5" t="inlineStr">
@@ -12043,7 +12055,7 @@
       <c r="AB7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>VC-007</t>
         </is>
@@ -12063,12 +12075,12 @@
           <t>Edge gateway 502s every proxied route while all upstream services are healthy (dev Render deployment)</t>
         </is>
       </c>
-      <c r="E8" s="14" t="inlineStr">
+      <c r="E8" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F8" s="14" t="inlineStr">
+      <c r="F8" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -12184,7 +12196,7 @@
       <c r="AB8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>VC-008</t>
         </is>
@@ -12204,12 +12216,12 @@
           <t>warmBackend() cannot warm the services it targets on the Render topology</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="F9" s="13" t="inlineStr">
+      <c r="F9" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -12324,7 +12336,7 @@
       <c r="AB9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>VC-009</t>
         </is>
@@ -12344,12 +12356,12 @@
           <t>POST /conversations/dm returns 404 through the gateway — 'New chat' cannot work</t>
         </is>
       </c>
-      <c r="E10" s="14" t="inlineStr">
+      <c r="E10" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F10" s="14" t="inlineStr">
+      <c r="F10" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -12463,7 +12475,7 @@
       <c r="AB10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>VC-010</t>
         </is>
@@ -12483,12 +12495,12 @@
           <t>Sign-out's authenticated calls ship with no Authorization header, so the server-side push endpoint is never cleared</t>
         </is>
       </c>
-      <c r="E11" s="14" t="inlineStr">
+      <c r="E11" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F11" s="14" t="inlineStr">
+      <c r="F11" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -12602,7 +12614,7 @@
       <c r="AB11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>VC-011</t>
         </is>
@@ -12622,12 +12634,12 @@
           <t>Sign-out then sign-in in one process silently destroys every notification action</t>
         </is>
       </c>
-      <c r="E12" s="15" t="inlineStr">
+      <c r="E12" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F12" s="15" t="inlineStr">
+      <c r="F12" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -12743,7 +12755,7 @@
       <c r="AB12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>VC-012</t>
         </is>
@@ -12763,12 +12775,12 @@
           <t>Android &lt;= 12 reports notifications as granted even when disabled, so the sync engine drops its background socket</t>
         </is>
       </c>
-      <c r="E13" s="15" t="inlineStr">
+      <c r="E13" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F13" s="15" t="inlineStr">
+      <c r="F13" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -12884,7 +12896,7 @@
       <c r="AB13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>VC-013</t>
         </is>
@@ -12904,12 +12916,12 @@
           <t>clearSession() is not a session teardown — the previous account's chat DB, profile and contacts survive into the next sign-in</t>
         </is>
       </c>
-      <c r="E14" s="15" t="inlineStr">
+      <c r="E14" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F14" s="15" t="inlineStr">
+      <c r="F14" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -13024,7 +13036,7 @@
       <c r="AB14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>VC-014</t>
         </is>
@@ -13044,12 +13056,12 @@
           <t>Rotating-refresh replay is structurally inevitable on a lost response, and the family revoke is then silently swallowed</t>
         </is>
       </c>
-      <c r="E15" s="14" t="inlineStr">
+      <c r="E15" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F15" s="14" t="inlineStr">
+      <c r="F15" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -13166,7 +13178,7 @@
       <c r="AB15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>VC-015</t>
         </is>
@@ -13186,12 +13198,12 @@
           <t>The cnfJkt DPoP binding is dead code — the refresh token is bound to nothing</t>
         </is>
       </c>
-      <c r="E16" s="14" t="inlineStr">
+      <c r="E16" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F16" s="14" t="inlineStr">
+      <c r="F16" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -13306,7 +13318,7 @@
       <c r="AB16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>VC-016</t>
         </is>
@@ -13326,12 +13338,12 @@
           <t>MMKV's encryption key is a hardcoded bundle constant, and the Ed25519 device private key is stored inside it</t>
         </is>
       </c>
-      <c r="E17" s="15" t="inlineStr">
+      <c r="E17" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F17" s="15" t="inlineStr">
+      <c r="F17" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -13446,7 +13458,7 @@
       <c r="AB17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>VC-017</t>
         </is>
@@ -13466,12 +13478,12 @@
           <t>Message plaintext and the user's own typed replies persist in plaintext SharedPreferences</t>
         </is>
       </c>
-      <c r="E18" s="14" t="inlineStr">
+      <c r="E18" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F18" s="14" t="inlineStr">
+      <c r="F18" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -13586,7 +13598,7 @@
       <c r="AB18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>VC-018</t>
         </is>
@@ -13606,12 +13618,12 @@
           <t>No certificate pinning anywhere, in JS or native</t>
         </is>
       </c>
-      <c r="E19" s="14" t="inlineStr">
+      <c r="E19" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F19" s="14" t="inlineStr">
+      <c r="F19" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -13725,7 +13737,7 @@
       <c r="AB19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>VC-019</t>
         </is>
@@ -13745,12 +13757,12 @@
           <t>Threat-model controls absent: no FLAG_SECURE, no Play Integrity, no clipboard auto-clear, no root signal</t>
         </is>
       </c>
-      <c r="E20" s="13" t="inlineStr">
+      <c r="E20" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="F20" s="13" t="inlineStr">
+      <c r="F20" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -13863,7 +13875,7 @@
       <c r="AB20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="A21" s="17" t="inlineStr">
         <is>
           <t>VC-020</t>
         </is>
@@ -13883,12 +13895,12 @@
           <t>Concurrent applyServerMessages duplicates every row in the overlap, and can lose a whole batch on a conversation PK clash</t>
         </is>
       </c>
-      <c r="E21" s="15" t="inlineStr">
+      <c r="E21" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F21" s="15" t="inlineStr">
+      <c r="F21" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -14003,7 +14015,7 @@
       <c r="AB21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="inlineStr">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>VC-021</t>
         </is>
@@ -14023,12 +14035,12 @@
           <t>applyReceipt is a non-atomic read-modify-write, so blue ticks can regress to grey</t>
         </is>
       </c>
-      <c r="E22" s="15" t="inlineStr">
+      <c r="E22" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F22" s="15" t="inlineStr">
+      <c r="F22" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -14142,7 +14154,7 @@
       <c r="AB22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="inlineStr">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>VC-022</t>
         </is>
@@ -14162,12 +14174,12 @@
           <t>A SendAck with seq 0 leaves the message permanently un-tickable and permanently duplicated</t>
         </is>
       </c>
-      <c r="E23" s="14" t="inlineStr">
+      <c r="E23" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F23" s="14" t="inlineStr">
+      <c r="F23" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -14281,7 +14293,7 @@
       <c r="AB23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="16" t="inlineStr">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>VC-023</t>
         </is>
@@ -14301,12 +14313,12 @@
           <t>One 401 on send turns the entire outbox into permanently failed messages</t>
         </is>
       </c>
-      <c r="E24" s="14" t="inlineStr">
+      <c r="E24" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F24" s="14" t="inlineStr">
+      <c r="F24" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -14421,7 +14433,7 @@
       <c r="AB24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="16" t="inlineStr">
+      <c r="A25" s="17" t="inlineStr">
         <is>
           <t>VC-024</t>
         </is>
@@ -14441,12 +14453,12 @@
           <t>Migration-v3's five composite indexes never exist on a fresh install</t>
         </is>
       </c>
-      <c r="E25" s="13" t="inlineStr">
+      <c r="E25" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="F25" s="13" t="inlineStr">
+      <c r="F25" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -14560,7 +14572,7 @@
       <c r="AB25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="inlineStr">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t>VC-025</t>
         </is>
@@ -14580,12 +14592,12 @@
           <t>reassertReceipts() on every connect emits an unbounded burst the gateway silently drops</t>
         </is>
       </c>
-      <c r="E26" s="14" t="inlineStr">
+      <c r="E26" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F26" s="14" t="inlineStr">
+      <c r="F26" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -14700,7 +14712,7 @@
       <c r="AB26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="16" t="inlineStr">
+      <c r="A27" s="17" t="inlineStr">
         <is>
           <t>VC-026</t>
         </is>
@@ -14720,12 +14732,12 @@
           <t>Unread count climbs and the read watermark stalls for messages backfilled into the chat you are reading</t>
         </is>
       </c>
-      <c r="E27" s="14" t="inlineStr">
+      <c r="E27" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F27" s="14" t="inlineStr">
+      <c r="F27" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -14840,7 +14852,7 @@
       <c r="AB27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="16" t="inlineStr">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>VC-027</t>
         </is>
@@ -14860,12 +14872,12 @@
           <t>'Load older' dead-ends permanently on a deletion hole wider than one page</t>
         </is>
       </c>
-      <c r="E28" s="13" t="inlineStr">
+      <c r="E28" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="F28" s="13" t="inlineStr">
+      <c r="F28" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -14979,7 +14991,7 @@
       <c r="AB28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="16" t="inlineStr">
+      <c r="A29" s="17" t="inlineStr">
         <is>
           <t>VC-028</t>
         </is>
@@ -14999,12 +15011,12 @@
           <t>No event_id dedup anywhere — the documented at-least-once guard does not exist</t>
         </is>
       </c>
-      <c r="E29" s="14" t="inlineStr">
+      <c r="E29" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F29" s="14" t="inlineStr">
+      <c r="F29" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -15118,7 +15130,7 @@
       <c r="AB29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="16" t="inlineStr">
+      <c r="A30" s="17" t="inlineStr">
         <is>
           <t>VC-029</t>
         </is>
@@ -15138,12 +15150,12 @@
           <t>Outbox backoff exhaustion is unreachable — MAX_SEND_ATTEMPTS can never fire</t>
         </is>
       </c>
-      <c r="E30" s="13" t="inlineStr">
+      <c r="E30" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="F30" s="13" t="inlineStr">
+      <c r="F30" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -15257,7 +15269,7 @@
       <c r="AB30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="16" t="inlineStr">
+      <c r="A31" s="17" t="inlineStr">
         <is>
           <t>VC-030</t>
         </is>
@@ -15277,12 +15289,12 @@
           <t>Message window sorts by created_at, not seq — a device clock ahead of the server permanently mis-orders own messages</t>
         </is>
       </c>
-      <c r="E31" s="14" t="inlineStr">
+      <c r="E31" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F31" s="14" t="inlineStr">
+      <c r="F31" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -15397,7 +15409,7 @@
       <c r="AB31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="16" t="inlineStr">
+      <c r="A32" s="17" t="inlineStr">
         <is>
           <t>VC-031</t>
         </is>
@@ -15417,12 +15429,12 @@
           <t>runQueuedPushActions runs queued notification actions concurrently while claiming to serialize them</t>
         </is>
       </c>
-      <c r="E32" s="13" t="inlineStr">
+      <c r="E32" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="F32" s="13" t="inlineStr">
+      <c r="F32" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -15537,7 +15549,7 @@
       <c r="AB32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="16" t="inlineStr">
+      <c r="A33" s="17" t="inlineStr">
         <is>
           <t>VC-032</t>
         </is>
@@ -15557,12 +15569,12 @@
           <t>No duplicate-notification suppression, though the monotonic watermark to do it already exists</t>
         </is>
       </c>
-      <c r="E33" s="14" t="inlineStr">
+      <c r="E33" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F33" s="14" t="inlineStr">
+      <c r="F33" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -15676,7 +15688,7 @@
       <c r="AB33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="16" t="inlineStr">
+      <c r="A34" s="17" t="inlineStr">
         <is>
           <t>VC-033</t>
         </is>
@@ -15696,12 +15708,12 @@
           <t>Native pending-event queue is a lock-free read-modify-write that can wipe a reply enqueued mid-drain</t>
         </is>
       </c>
-      <c r="E34" s="14" t="inlineStr">
+      <c r="E34" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F34" s="14" t="inlineStr">
+      <c r="F34" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -15816,7 +15828,7 @@
       <c r="AB34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="16" t="inlineStr">
+      <c r="A35" s="17" t="inlineStr">
         <is>
           <t>VC-034</t>
         </is>
@@ -15836,12 +15848,12 @@
           <t>Retry-After is honored with an unbounded, uncancellable sleep</t>
         </is>
       </c>
-      <c r="E35" s="13" t="inlineStr">
+      <c r="E35" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="F35" s="13" t="inlineStr">
+      <c r="F35" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -15955,7 +15967,7 @@
       <c r="AB35" s="5" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="16" t="inlineStr">
+      <c r="A36" s="17" t="inlineStr">
         <is>
           <t>VC-035</t>
         </is>
@@ -15975,12 +15987,12 @@
           <t>A misbuilt binary reports env:'dev' while talking to production</t>
         </is>
       </c>
-      <c r="E36" s="13" t="inlineStr">
+      <c r="E36" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="F36" s="13" t="inlineStr">
+      <c r="F36" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -16094,7 +16106,7 @@
       <c r="AB36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="16" t="inlineStr">
+      <c r="A37" s="17" t="inlineStr">
         <is>
           <t>VC-036</t>
         </is>
@@ -16114,12 +16126,12 @@
           <t>Cold start after &gt;15 min idle opens the WebSocket with a certainly-expired token</t>
         </is>
       </c>
-      <c r="E37" s="13" t="inlineStr">
+      <c r="E37" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="F37" s="13" t="inlineStr">
+      <c r="F37" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -16234,7 +16246,7 @@
       <c r="AB37" s="5" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="16" t="inlineStr">
+      <c r="A38" s="17" t="inlineStr">
         <is>
           <t>VC-037</t>
         </is>
@@ -16254,12 +16266,12 @@
           <t>The access token travels in the WebSocket query string</t>
         </is>
       </c>
-      <c r="E38" s="13" t="inlineStr">
+      <c r="E38" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="F38" s="13" t="inlineStr">
+      <c r="F38" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -16373,7 +16385,7 @@
       <c r="AB38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="16" t="inlineStr">
+      <c r="A39" s="17" t="inlineStr">
         <is>
           <t>VC-038</t>
         </is>
@@ -16393,12 +16405,12 @@
           <t>Jest reports a worker that failed to exit gracefully — a leaked timer or handle in the test path</t>
         </is>
       </c>
-      <c r="E39" s="18" t="inlineStr">
+      <c r="E39" s="19" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="F39" s="18" t="inlineStr">
+      <c r="F39" s="19" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
@@ -16512,7 +16524,7 @@
       <c r="AB39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="16" t="inlineStr">
+      <c r="A40" s="17" t="inlineStr">
         <is>
           <t>VC-039</t>
         </is>
@@ -16532,12 +16544,12 @@
           <t>Any authenticated user can READ and WRITE any conversation — no authorization on the chat routes, and conversation ids are derivable offline</t>
         </is>
       </c>
-      <c r="E40" s="15" t="inlineStr">
+      <c r="E40" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F40" s="15" t="inlineStr">
+      <c r="F40" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -16637,12 +16649,12 @@
       </c>
       <c r="X40" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="Y40" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="Z40" s="5" t="inlineStr">
@@ -16658,7 +16670,7 @@
       <c r="AB40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="16" t="inlineStr">
+      <c r="A41" s="17" t="inlineStr">
         <is>
           <t>VC-040</t>
         </is>
@@ -16678,12 +16690,12 @@
           <t>A push endpoint can be registered against another account's userId, redirecting their push wake-ups</t>
         </is>
       </c>
-      <c r="E41" s="14" t="inlineStr">
+      <c r="E41" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F41" s="14" t="inlineStr">
+      <c r="F41" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -16776,12 +16788,12 @@
       </c>
       <c r="X41" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="Y41" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="Z41" s="5" t="inlineStr">
@@ -16797,7 +16809,7 @@
       <c r="AB41" s="5" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="16" t="inlineStr">
+      <c r="A42" s="17" t="inlineStr">
         <is>
           <t>VC-041</t>
         </is>
@@ -16817,12 +16829,12 @@
           <t>POST /chat/messages accepts a conversationId that does not exist</t>
         </is>
       </c>
-      <c r="E42" s="14" t="inlineStr">
+      <c r="E42" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F42" s="14" t="inlineStr">
+      <c r="F42" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -16914,12 +16926,12 @@
       </c>
       <c r="X42" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="Y42" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="Z42" s="5" t="inlineStr">
@@ -16935,7 +16947,7 @@
       <c r="AB42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="16" t="inlineStr">
+      <c r="A43" s="17" t="inlineStr">
         <is>
           <t>VC-042</t>
         </is>
@@ -16955,12 +16967,12 @@
           <t>POST /chat/messages accepts an empty or whitespace-only message</t>
         </is>
       </c>
-      <c r="E43" s="13" t="inlineStr">
+      <c r="E43" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="F43" s="13" t="inlineStr">
+      <c r="F43" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -17053,12 +17065,12 @@
       </c>
       <c r="X43" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="Y43" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="Z43" s="5" t="inlineStr">
@@ -17074,7 +17086,7 @@
       <c r="AB43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="16" t="inlineStr">
+      <c r="A44" s="17" t="inlineStr">
         <is>
           <t>VC-043</t>
         </is>
@@ -17094,12 +17106,12 @@
           <t>Concurrent refresh-token requests can all succeed — rotation is not race-safe</t>
         </is>
       </c>
-      <c r="E44" s="14" t="inlineStr">
+      <c r="E44" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F44" s="14" t="inlineStr">
+      <c r="F44" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -17193,12 +17205,12 @@
       </c>
       <c r="X44" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="Y44" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="Z44" s="5" t="inlineStr">
@@ -17214,7 +17226,7 @@
       <c r="AB44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="16" t="inlineStr">
+      <c r="A45" s="17" t="inlineStr">
         <is>
           <t>VC-044</t>
         </is>
@@ -17230,12 +17242,12 @@
           <t>Contact name/contact update does not sync immediately in chat UI</t>
         </is>
       </c>
-      <c r="E45" s="13" t="inlineStr">
+      <c r="E45" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="F45" s="13" t="inlineStr">
+      <c r="F45" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -17352,7 +17364,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="16" t="inlineStr">
+      <c r="A46" s="17" t="inlineStr">
         <is>
           <t>VC-045</t>
         </is>
@@ -17368,12 +17380,12 @@
           <t>Real-time messaging and notification-reply sync needs multi-scenario two-device verification</t>
         </is>
       </c>
-      <c r="E46" s="14" t="inlineStr">
+      <c r="E46" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F46" s="14" t="inlineStr">
+      <c r="F46" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -17489,7 +17501,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="16" t="inlineStr">
+      <c r="A47" s="17" t="inlineStr">
         <is>
           <t>VC-046</t>
         </is>
@@ -17505,12 +17517,12 @@
           <t>Online/offline presence status updates with a noticeable delay</t>
         </is>
       </c>
-      <c r="E47" s="13" t="inlineStr">
+      <c r="E47" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="F47" s="13" t="inlineStr">
+      <c r="F47" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -17624,7 +17636,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="16" t="inlineStr">
+      <c r="A48" s="17" t="inlineStr">
         <is>
           <t>VC-047</t>
         </is>
@@ -17644,12 +17656,12 @@
           <t>Chat List shows the registered VelChat name instead of the saved contact name until a chat is opened</t>
         </is>
       </c>
-      <c r="E48" s="13" t="inlineStr">
+      <c r="E48" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="F48" s="13" t="inlineStr">
+      <c r="F48" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -17765,7 +17777,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="16" t="inlineStr">
+      <c r="A49" s="17" t="inlineStr">
         <is>
           <t>VC-048</t>
         </is>
@@ -17781,12 +17793,12 @@
           <t>Message notification omits the sender's name and tapping it does not open the chat</t>
         </is>
       </c>
-      <c r="E49" s="13" t="inlineStr">
+      <c r="E49" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="F49" s="13" t="inlineStr">
+      <c r="F49" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -17902,7 +17914,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="16" t="inlineStr">
+      <c r="A50" s="17" t="inlineStr">
         <is>
           <t>VC-049</t>
         </is>
@@ -17922,12 +17934,12 @@
           <t>Email-prompt bottom sheet reappears on every login even when an email is already saved</t>
         </is>
       </c>
-      <c r="E50" s="14" t="inlineStr">
+      <c r="E50" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F50" s="14" t="inlineStr">
+      <c r="F50" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -18068,560 +18080,560 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="inlineStr">
+      <c r="A3" s="20" t="inlineStr">
         <is>
           <t>Execution</t>
         </is>
       </c>
-      <c r="B3" s="20" t="n"/>
-      <c r="C3" s="20" t="n"/>
+      <c r="B3" s="21" t="n"/>
+      <c r="C3" s="21" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="21" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>Total tests tracked</t>
         </is>
       </c>
-      <c r="B4" s="22" t="n">
+      <c r="B4" s="23" t="n">
         <v>92</v>
       </c>
-      <c r="C4" s="23" t="inlineStr"/>
+      <c r="C4" s="24" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="B5" s="22" t="n">
-        <v>79</v>
-      </c>
-      <c r="C5" s="23" t="inlineStr"/>
+      <c r="B5" s="23" t="n">
+        <v>78</v>
+      </c>
+      <c r="C5" s="24" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="B6" s="22" t="n">
-        <v>13</v>
-      </c>
-      <c r="C6" s="23" t="inlineStr"/>
+      <c r="B6" s="23" t="n">
+        <v>14</v>
+      </c>
+      <c r="C6" s="24" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="A7" s="22" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
       </c>
-      <c r="B7" s="22" t="n">
+      <c r="B7" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="C7" s="23" t="inlineStr">
+      <c r="C7" s="24" t="inlineStr">
         <is>
           <t>Environment invalid — never counted as a product defect (§47)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="21" t="inlineStr">
+      <c r="A8" s="22" t="inlineStr">
         <is>
           <t>Skipped</t>
         </is>
       </c>
-      <c r="B8" s="22" t="n">
+      <c r="B8" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="C8" s="23" t="inlineStr"/>
+      <c r="C8" s="24" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
         <is>
           <t>Manually verified</t>
         </is>
       </c>
-      <c r="B9" s="22" t="n">
+      <c r="B9" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="23" t="inlineStr">
+      <c r="C9" s="24" t="inlineStr">
         <is>
           <t>A human set this verdict directly in Excel — preserved across every rebuild</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="22" t="inlineStr">
         <is>
           <t>Flaky</t>
         </is>
       </c>
-      <c r="B10" s="22" t="n">
+      <c r="B10" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" s="24" t="inlineStr">
+        <is>
+          <t>Result changed across runs — investigated, never auto-passed (§42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="22" t="inlineStr">
+        <is>
+          <t>Pass percentage</t>
+        </is>
+      </c>
+      <c r="B11" s="23" t="inlineStr">
+        <is>
+          <t>84.8%</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t>Defects by severity</t>
+        </is>
+      </c>
+      <c r="B13" s="21" t="n"/>
+      <c r="C13" s="21" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="22" t="inlineStr">
+        <is>
+          <t>P0 — Critical</t>
+        </is>
+      </c>
+      <c r="B14" s="23" t="n">
+        <v>11</v>
+      </c>
+      <c r="C14" s="24" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="22" t="inlineStr">
+        <is>
+          <t>P1 — High</t>
+        </is>
+      </c>
+      <c r="B15" s="23" t="n">
+        <v>22</v>
+      </c>
+      <c r="C15" s="24" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="22" t="inlineStr">
+        <is>
+          <t>P2 — Medium</t>
+        </is>
+      </c>
+      <c r="B16" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" s="24" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="22" t="inlineStr">
+        <is>
+          <t>P3 — Low</t>
+        </is>
+      </c>
+      <c r="B17" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="24" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="22" t="inlineStr">
+        <is>
+          <t>Open bugs</t>
+        </is>
+      </c>
+      <c r="B18" s="23" t="n">
+        <v>25</v>
+      </c>
+      <c r="C18" s="24" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="22" t="inlineStr">
+        <is>
+          <t>Fixed bugs</t>
+        </is>
+      </c>
+      <c r="B19" s="23" t="n">
+        <v>23</v>
+      </c>
+      <c r="C19" s="24" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="22" t="inlineStr">
+        <is>
+          <t>Regression bugs</t>
+        </is>
+      </c>
+      <c r="B20" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="C10" s="23" t="inlineStr">
-        <is>
-          <t>Result changed across runs — investigated, never auto-passed (§42)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="21" t="inlineStr">
-        <is>
-          <t>Pass percentage</t>
-        </is>
-      </c>
-      <c r="B11" s="22" t="inlineStr">
-        <is>
-          <t>85.9%</t>
-        </is>
-      </c>
-      <c r="C11" s="23" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t>Defects by severity</t>
-        </is>
-      </c>
-      <c r="B13" s="20" t="n"/>
-      <c r="C13" s="20" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="21" t="inlineStr">
-        <is>
-          <t>P0 — Critical</t>
-        </is>
-      </c>
-      <c r="B14" s="22" t="n">
-        <v>11</v>
-      </c>
-      <c r="C14" s="23" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="21" t="inlineStr">
-        <is>
-          <t>P1 — High</t>
-        </is>
-      </c>
-      <c r="B15" s="22" t="n">
-        <v>22</v>
-      </c>
-      <c r="C15" s="23" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="21" t="inlineStr">
-        <is>
-          <t>P2 — Medium</t>
-        </is>
-      </c>
-      <c r="B16" s="22" t="n">
-        <v>15</v>
-      </c>
-      <c r="C16" s="23" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="21" t="inlineStr">
-        <is>
-          <t>P3 — Low</t>
-        </is>
-      </c>
-      <c r="B17" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="C17" s="23" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="21" t="inlineStr">
-        <is>
-          <t>Open bugs</t>
-        </is>
-      </c>
-      <c r="B18" s="22" t="n">
-        <v>25</v>
-      </c>
-      <c r="C18" s="23" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="21" t="inlineStr">
-        <is>
-          <t>Fixed bugs</t>
-        </is>
-      </c>
-      <c r="B19" s="22" t="n">
-        <v>23</v>
-      </c>
-      <c r="C19" s="23" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="21" t="inlineStr">
-        <is>
-          <t>Regression bugs</t>
-        </is>
-      </c>
-      <c r="B20" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="C20" s="23" t="inlineStr"/>
+      <c r="C20" s="24" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="inlineStr">
+      <c r="A22" s="20" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B22" s="20" t="n"/>
-      <c r="C22" s="20" t="n"/>
+      <c r="B22" s="21" t="n"/>
+      <c r="C22" s="21" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="21" t="inlineStr">
+      <c r="A23" s="22" t="inlineStr">
         <is>
           <t>Build under test</t>
         </is>
       </c>
-      <c r="B23" s="22" t="inlineStr">
+      <c r="B23" s="23" t="inlineStr">
         <is>
           <t>com.velchat.dev 1.0-dev (apk-out/velchat-20260909-2025.apk)</t>
         </is>
       </c>
-      <c r="C23" s="23" t="inlineStr"/>
+      <c r="C23" s="24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="inlineStr">
+      <c r="A25" s="20" t="inlineStr">
         <is>
           <t>Release gate (§41)</t>
         </is>
       </c>
-      <c r="B25" s="20" t="n"/>
-      <c r="C25" s="20" t="n"/>
+      <c r="B25" s="21" t="n"/>
+      <c r="C25" s="21" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="21" t="inlineStr">
+      <c r="A26" s="22" t="inlineStr">
         <is>
           <t>Recommendation</t>
         </is>
       </c>
-      <c r="B26" s="24" t="inlineStr">
+      <c r="B26" s="25" t="inlineStr">
         <is>
           <t>NO-GO</t>
         </is>
       </c>
-      <c r="C26" s="25" t="inlineStr">
+      <c r="C26" s="26" t="inlineStr">
         <is>
           <t>18 open P0/P1 defect(s) block the build.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="19" t="inlineStr">
+      <c r="A28" s="20" t="inlineStr">
         <is>
           <t>Blocking defects</t>
         </is>
       </c>
-      <c r="B28" s="20" t="n"/>
-      <c r="C28" s="20" t="n"/>
+      <c r="B28" s="21" t="n"/>
+      <c r="C28" s="21" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="21" t="inlineStr">
+      <c r="A29" s="22" t="inlineStr">
         <is>
           <t>VC-001</t>
         </is>
       </c>
-      <c r="B29" s="22" t="inlineStr">
+      <c r="B29" s="23" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="C29" s="23" t="inlineStr">
+      <c r="C29" s="24" t="inlineStr">
         <is>
           <t>Realtime fan-out silently drops up to 63% of durable messages sent within ~250ms of each other</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="21" t="inlineStr">
+      <c r="A30" s="22" t="inlineStr">
         <is>
           <t>VC-002</t>
         </is>
       </c>
-      <c r="B30" s="22" t="inlineStr">
+      <c r="B30" s="23" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="C30" s="23" t="inlineStr">
+      <c r="C30" s="24" t="inlineStr">
         <is>
           <t>Blue tick never arrives: a `read` receipt sent in the same tick as `delivered` is lost</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="21" t="inlineStr">
+      <c r="A31" s="22" t="inlineStr">
         <is>
           <t>VC-003</t>
         </is>
       </c>
-      <c r="B31" s="22" t="inlineStr">
+      <c r="B31" s="23" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="C31" s="23" t="inlineStr">
+      <c r="C31" s="24" t="inlineStr">
         <is>
           <t>Read watermark can regress: the higher receipt is lost and a lower one survives</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="21" t="inlineStr">
+      <c r="A32" s="22" t="inlineStr">
         <is>
           <t>VC-004</t>
         </is>
       </c>
-      <c r="B32" s="22" t="inlineStr">
+      <c r="B32" s="23" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C32" s="23" t="inlineStr">
+      <c r="C32" s="24" t="inlineStr">
         <is>
           <t>POST /auth/register accepts an arbitrary non-phone string and provisions a full account with real tokens</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="21" t="inlineStr">
+      <c r="A33" s="22" t="inlineStr">
         <is>
           <t>VC-005</t>
         </is>
       </c>
-      <c r="B33" s="22" t="inlineStr">
+      <c r="B33" s="23" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C33" s="23" t="inlineStr">
+      <c r="C33" s="24" t="inlineStr">
         <is>
           <t>POST /auth/register accepts a non-base64 device public key, permanently breaking device-key login for that install</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="21" t="inlineStr">
+      <c r="A34" s="22" t="inlineStr">
         <is>
           <t>VC-006</t>
         </is>
       </c>
-      <c r="B34" s="22" t="inlineStr">
+      <c r="B34" s="23" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="C34" s="23" t="inlineStr">
+      <c r="C34" s="24" t="inlineStr">
         <is>
           <t>POST /auth/revotp/webhook is @Public with no shared secret — an unauthenticated account-provisioning primitive</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="21" t="inlineStr">
+      <c r="A35" s="22" t="inlineStr">
         <is>
           <t>VC-007</t>
         </is>
       </c>
-      <c r="B35" s="22" t="inlineStr">
+      <c r="B35" s="23" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C35" s="23" t="inlineStr">
+      <c r="C35" s="24" t="inlineStr">
         <is>
           <t>Edge gateway 502s every proxied route while all upstream services are healthy (dev Render deployment)</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="21" t="inlineStr">
+      <c r="A36" s="22" t="inlineStr">
         <is>
           <t>VC-009</t>
         </is>
       </c>
-      <c r="B36" s="22" t="inlineStr">
+      <c r="B36" s="23" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C36" s="23" t="inlineStr">
+      <c r="C36" s="24" t="inlineStr">
         <is>
           <t>POST /conversations/dm returns 404 through the gateway — 'New chat' cannot work</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="21" t="inlineStr">
+      <c r="A37" s="22" t="inlineStr">
         <is>
           <t>VC-016</t>
         </is>
       </c>
-      <c r="B37" s="22" t="inlineStr">
+      <c r="B37" s="23" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="C37" s="23" t="inlineStr">
+      <c r="C37" s="24" t="inlineStr">
         <is>
           <t>MMKV's encryption key is a hardcoded bundle constant, and the Ed25519 device private key is stored inside it</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="21" t="inlineStr">
+      <c r="A38" s="22" t="inlineStr">
         <is>
           <t>VC-017</t>
         </is>
       </c>
-      <c r="B38" s="22" t="inlineStr">
+      <c r="B38" s="23" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C38" s="23" t="inlineStr">
+      <c r="C38" s="24" t="inlineStr">
         <is>
           <t>Message plaintext and the user's own typed replies persist in plaintext SharedPreferences</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="21" t="inlineStr">
+      <c r="A39" s="22" t="inlineStr">
         <is>
           <t>VC-018</t>
         </is>
       </c>
-      <c r="B39" s="22" t="inlineStr">
+      <c r="B39" s="23" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C39" s="23" t="inlineStr">
+      <c r="C39" s="24" t="inlineStr">
         <is>
           <t>No certificate pinning anywhere, in JS or native</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="21" t="inlineStr">
+      <c r="A40" s="22" t="inlineStr">
         <is>
           <t>VC-032</t>
         </is>
       </c>
-      <c r="B40" s="22" t="inlineStr">
+      <c r="B40" s="23" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C40" s="23" t="inlineStr">
+      <c r="C40" s="24" t="inlineStr">
         <is>
           <t>No duplicate-notification suppression, though the monotonic watermark to do it already exists</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="21" t="inlineStr">
+      <c r="A41" s="22" t="inlineStr">
         <is>
           <t>VC-033</t>
         </is>
       </c>
-      <c r="B41" s="22" t="inlineStr">
+      <c r="B41" s="23" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C41" s="23" t="inlineStr">
+      <c r="C41" s="24" t="inlineStr">
         <is>
           <t>Native pending-event queue is a lock-free read-modify-write that can wipe a reply enqueued mid-drain</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="21" t="inlineStr">
+      <c r="A42" s="22" t="inlineStr">
         <is>
           <t>VC-039</t>
         </is>
       </c>
-      <c r="B42" s="22" t="inlineStr">
+      <c r="B42" s="23" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="C42" s="23" t="inlineStr">
+      <c r="C42" s="24" t="inlineStr">
         <is>
           <t>Any authenticated user can READ and WRITE any conversation — no authorization on the chat routes, and conversation ids are derivable offline</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="21" t="inlineStr">
+      <c r="A43" s="22" t="inlineStr">
         <is>
           <t>VC-040</t>
         </is>
       </c>
-      <c r="B43" s="22" t="inlineStr">
+      <c r="B43" s="23" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C43" s="23" t="inlineStr">
+      <c r="C43" s="24" t="inlineStr">
         <is>
           <t>A push endpoint can be registered against another account's userId, redirecting their push wake-ups</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="21" t="inlineStr">
+      <c r="A44" s="22" t="inlineStr">
         <is>
           <t>VC-041</t>
         </is>
       </c>
-      <c r="B44" s="22" t="inlineStr">
+      <c r="B44" s="23" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C44" s="23" t="inlineStr">
+      <c r="C44" s="24" t="inlineStr">
         <is>
           <t>POST /chat/messages accepts a conversationId that does not exist</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="21" t="inlineStr">
+      <c r="A45" s="22" t="inlineStr">
         <is>
           <t>VC-043</t>
         </is>
       </c>
-      <c r="B45" s="22" t="inlineStr">
+      <c r="B45" s="23" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C45" s="23" t="inlineStr">
+      <c r="C45" s="24" t="inlineStr">
         <is>
           <t>Concurrent refresh-token requests can all succeed — rotation is not race-safe</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="21" t="inlineStr">
+      <c r="A46" s="22" t="inlineStr">
         <is>
           <t>VC-045</t>
         </is>
       </c>
-      <c r="B46" s="22" t="inlineStr">
+      <c r="B46" s="23" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="C46" s="23" t="inlineStr">
+      <c r="C46" s="24" t="inlineStr">
         <is>
           <t>Real-time messaging and notification-reply sync needs multi-scenario two-device verification</t>
         </is>
@@ -18709,10 +18721,10 @@
         <v>92</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G2" s="5" t="n">
         <v>0</v>
@@ -18724,41 +18736,41 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="26" t="inlineStr">
+      <c r="A4" s="27" t="inlineStr">
         <is>
           <t>Devices NOT covered in this run</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="28" t="inlineStr">
         <is>
           <t>3 GB Android 10 handset</t>
         </is>
       </c>
-      <c r="B5" s="28" t="inlineStr">
+      <c r="B5" s="29" t="inlineStr">
         <is>
           <t>Android 10 (API 29)</t>
         </is>
       </c>
-      <c r="C5" s="28" t="inlineStr">
+      <c r="C5" s="29" t="inlineStr">
         <is>
           <t>The §M0 reference device. No such device or AVD available. VC-006/VC-012-class is Android &lt;= 12 only and needs it.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="27" t="inlineStr">
+      <c r="A6" s="28" t="inlineStr">
         <is>
           <t>iOS (any)</t>
         </is>
       </c>
-      <c r="B6" s="28" t="inlineStr">
+      <c r="B6" s="29" t="inlineStr">
         <is>
           <t>iOS 17+</t>
         </is>
       </c>
-      <c r="C6" s="28" t="inlineStr">
+      <c r="C6" s="29" t="inlineStr">
         <is>
           <t>Cannot be built on Windows — no macOS/Xcode/CocoaPods.</t>
         </is>
@@ -19717,7 +19729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -19767,9 +19779,68 @@
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="23" t="inlineStr">
-        <is>
-          <t>No test has produced different results across runs. A retry that changes a result is recorded as FLAKY and investigated — never silently promoted to PASS (§42/§46).</t>
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>VC-AUTH-027</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>concurrent refreshes of the same token do not both succeed</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>33%</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>node-harness</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>http://localhost:8080</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>VC-RT-030</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>a `delivered` receipt from B reaches A (grey double tick)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>node-harness</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>http://localhost:8080</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(qa): record the live two-device findings and which of them are fixed
VC-051..VC-061 filed from the chat + notification live pass (Jira VC-52..VC-62),
VC-045/VC-046/VC-048 updated with what the session actually observed, and the
seven fixed entries annotated with their root cause and on-device verification.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA/reports/VelChat-QA-Report.xlsx
+++ b/QA/reports/VelChat-QA-Report.xlsx
@@ -641,7 +641,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-14 04:21 UTC</t>
+          <t>Generated 2026-09-14 04:40 UTC</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -18351,7 +18351,7 @@
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr">
@@ -18445,7 +18445,8 @@
       </c>
       <c r="AA53" s="5" t="inlineStr">
         <is>
-          <t>Evidence: scratchpad/shots/b_fg_follow.png (B at the bottom, F1-F3 arrive, list stays on S8 and the jump FAB appears), scratchpad/shots/b_one.png (single message ONE1 arrives, list left exactly one bubble short), scratchpad/shots/a_own_follow.png (A's OWN sent ONE1 clipped behind the composer), scratchpad/shots/b_offline_send.png (own offline sends clipped). The race explains the intermittency: sometimes the manual scroll lands after the anchor adjustment and it looks fine.</t>
+          <t>Evidence: scratchpad/shots/b_fg_follow.png (B at the bottom, F1-F3 arrive, list stays on S8 and the jump FAB appears), scratchpad/shots/b_one.png (single message ONE1 arrives, list left exactly one bubble short), scratchpad/shots/a_own_follow.png (A's OWN sent ONE1 clipped behind the composer), scratchpad/shots/b_offline_send.png (own offline sends clipped). The race explains the intermittency: sometimes the manual scroll lands after the anchor adjustment and it looks fine.
+FIX: the follow now goes through FlashList's `scrollToIndex({index:0})` instead of `scrollToOffset({offset:0})`, fired from `onContentSizeChange` rather than the data effect. Root cause confirmed by reading useRecyclerViewController.js: on every data change FlashList measures how far the FIRST VISIBLE item moved and calls scrollAnchorRef.scrollBy(diff) to cancel the shift, gated on a `pauseOffsetCorrection` ref that ONLY scrollToIndex raises — so a plain offset scroll was undone every time and the thread landed exactly one bubble short. Firing from onContentSizeChange means index 0 has a real layout instead of the stale one it would have in the same commit. Anchoring is deliberately kept: it is the right behaviour for a reader scrolled up in history, whom shouldScrollToLatest still leaves alone; a drag cancels any pending follow so loadOlder growing the content is never mistaken for a new message. An intermediate attempt using scrollToOffset from onContentSizeChange plus a requestAnimationFrame retry was built and tested on device and still landed one bubble short — that is what identified the pauseOffsetCorrection gate. VERIFIED ON DEVICE: a four-message burst now ends with the newest message fully visible above the composer (scratchpad/shots/v2_own_follow.png) where the same burst on the previous build left it clipped (v_own_follow.png). Still to verify with a second device: the INCOMING-message path, and the notification tap-through landing position.</t>
         </is>
       </c>
       <c r="AB53" s="5" t="inlineStr"/>
@@ -18479,7 +18480,7 @@
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H54" s="5" t="inlineStr">
@@ -18574,7 +18575,8 @@
       </c>
       <c r="AA54" s="5" t="inlineStr">
         <is>
-          <t>Evidence: scratchpad/shots/b_tapthrough.png and b_jump.png (header 'Chats' after notification tap) vs scratchpad/shots/b_off_kbd.png (header 'Aayush Jain 🤗' for the same chat opened from the list). Relates to VC-048, which reported the tap-through as not opening the chat at all; the open now works, this is the remaining defect on that path.</t>
+          <t>Evidence: scratchpad/shots/b_tapthrough.png and b_jump.png (header 'Chats' after notification tap) vs scratchpad/shots/b_off_kbd.png (header 'Aayush Jain 🤗' for the same chat opened from the list). Relates to VC-048, which reported the tap-through as not opening the chat at all; the open now works, this is the remaining defect on that path.
+FIX: new pure helper `chatTitle(routeName, rowName, fallback)` in ui/chat/chatModel.ts, covered by chatTitle.test.ts (4 cases, RED first). ChatHeader now resolves the title from the route name, then the conversation row it was already observing for the avatar, and only then a generic label; blank counts as absent in both sources. The avatar initial is taken from the resolved name with an empty fallback, so a genuinely unnamed conversation still falls back to the person glyph instead of showing the initial of a tab label. Needs a second device to re-verify the live tap-through.</t>
         </is>
       </c>
       <c r="AB54" s="5" t="inlineStr"/>
@@ -18608,7 +18610,7 @@
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr">
@@ -18702,7 +18704,8 @@
       </c>
       <c r="AA55" s="5" t="inlineStr">
         <is>
-          <t>Evidence: dumpsys output captured twice in the live session (8 messages -&gt; '5 new messages'; 1 message -&gt; '5 new messages').</t>
+          <t>Evidence: dumpsys output captured twice in the live session (8 messages -&gt; '5 new messages'; 1 message -&gt; '5 new messages').
+FIX: added `PushStore.countedMessages()`, which sums the per-conversation counters the store already held, and postSummary now formats that instead of `countedConversations()`. The &lt;=1 guard that suppresses the summary for a single chat still uses the conversation count, which is correct. Needs a second device to re-verify live.</t>
         </is>
       </c>
       <c r="AB55" s="5" t="inlineStr"/>
@@ -18736,7 +18739,7 @@
       </c>
       <c r="G56" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H56" s="5" t="inlineStr">
@@ -18830,7 +18833,8 @@
       </c>
       <c r="AA56" s="5" t="inlineStr">
         <is>
-          <t>Confirmed by reading tokens.ts (brandFrom '#0B0B0C' / '#F5F5F7') against push_strings.xml (#7C5CFF) and by the live dumpsys record color=0xff7c5cff.</t>
+          <t>Confirmed by reading tokens.ts (brandFrom '#0B0B0C' / '#F5F5F7') against push_strings.xml (#7C5CFF) and by the live dumpsys record color=0xff7c5cff.
+FIX: push_accent is now #0B0B0C, the monochrome brand accent from design-system/tokens.ts, and the misleading resource comment about a violet gradient is replaced. Android resolves this against the shade background for contrast. Needs a second device to re-verify live.</t>
         </is>
       </c>
       <c r="AB56" s="5" t="inlineStr"/>
@@ -19121,7 +19125,7 @@
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H59" s="5" t="inlineStr">
@@ -19214,7 +19218,8 @@
       </c>
       <c r="AA59" s="5" t="inlineStr">
         <is>
-          <t>Evidence: scratchpad/shots/b_after_reply.png (row reads 'KILL1' while KILL2 was newer). Fix is to move the preview write inside the same freshness check as the timestamp.</t>
+          <t>Evidence: scratchpad/shots/b_after_reply.png (row reads 'KILL1' while KILL2 was newer). Fix is to move the preview write inside the same freshness check as the timestamp.
+FIX: the preview write now sits behind the same freshness check as the sort key in upsertConversation — a single `fresher` predicate gates both, so a stale patch can no longer overwrite what the row says while being correctly refused a reorder.</t>
         </is>
       </c>
       <c r="AB59" s="5" t="inlineStr"/>
@@ -19375,7 +19380,7 @@
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr">
@@ -19469,7 +19474,8 @@
       </c>
       <c r="AA61" s="5" t="inlineStr">
         <is>
-          <t>Evidence: scratchpad/shots/a_relaunch.png — the 'kkr' and 'h' bubbles in light theme. Fix options: give the incoming bubble a hairline in BOTH schemes, or darken `bgSubtle` for this use.</t>
+          <t>Evidence: scratchpad/shots/a_relaunch.png — the 'kkr' and 'h' bubbles in light theme. Fix options: give the incoming bubble a hairline in BOTH schemes, or darken `bgSubtle` for this use.
+FIX: the incoming-bubble hairline is no longer dark-only; it applies in both schemes, using the wallpaper-supplied border when the chat has a decorated ground and t.colors.hairline otherwise.</t>
         </is>
       </c>
       <c r="AB61" s="5" t="inlineStr"/>
@@ -19503,7 +19509,7 @@
       </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H62" s="5" t="inlineStr">
@@ -19596,7 +19602,8 @@
       </c>
       <c r="AA62" s="5" t="inlineStr">
         <is>
-          <t>Evidence: scratchpad/shots/a_cal.png and a_own_follow.png — the white band between the composer pill and the keyboard's suggestion strip. Same file also sets `borderTopWidth: 0` alongside a `borderTopColor`, so the intended separator between the thread and the composer never draws.</t>
+          <t>Evidence: scratchpad/shots/a_cal.png and a_own_follow.png — the white band between the composer pill and the keyboard's suggestion strip. Same file also sets `borderTopWidth: 0` alongside a `borderTopColor`, so the intended separator between the thread and the composer never draws.
+FIX: keyboard-up paddingBottom drops from spacing.huge (48dp) to spacing.xs (8dp), and borderTopWidth goes from 0 to 1 so the separator the style always declared actually draws. VERIFIED ON DEVICE: scratchpad/shots/v2_own_follow.png shows the hairline above the composer and the composer sitting close to the keyboard.</t>
         </is>
       </c>
       <c r="AB62" s="5" t="inlineStr"/>
@@ -19613,7 +19620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -19799,7 +19806,7 @@
         </is>
       </c>
       <c r="B18" s="23" t="n">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="C18" s="24" t="inlineStr"/>
     </row>
@@ -19810,7 +19817,7 @@
         </is>
       </c>
       <c r="B19" s="23" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="C19" s="24" t="inlineStr"/>
     </row>
@@ -19869,7 +19876,7 @@
       </c>
       <c r="C26" s="26" t="inlineStr">
         <is>
-          <t>20 open P0/P1 defect(s) block the build.</t>
+          <t>18 open P0/P1 defect(s) block the build.</t>
         </is>
       </c>
     </row>
@@ -20185,40 +20192,6 @@
       <c r="C46" s="24" t="inlineStr">
         <is>
           <t>A message the device was pushed for never reaches the chat, and no reconnect ever heals it — the sender still sees blue read ticks</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="22" t="inlineStr">
-        <is>
-          <t>VC-052</t>
-        </is>
-      </c>
-      <c r="B47" s="23" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C47" s="24" t="inlineStr">
-        <is>
-          <t>Chat thread does not follow the newest message — incoming and own-sent bubbles land hidden behind the composer</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="22" t="inlineStr">
-        <is>
-          <t>VC-053</t>
-        </is>
-      </c>
-      <c r="B48" s="23" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C48" s="24" t="inlineStr">
-        <is>
-          <t>Chat opened from a notification is titled "Chats" instead of the contact's name, and the avatar loses its initial</t>
         </is>
       </c>
     </row>
@@ -20371,7 +20344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21405,6 +21378,251 @@
       <c r="H27" s="5" t="inlineStr">
         <is>
           <t>FIX: split the two questions the bootstrap had conflated — "can we show the app" and "is the access token fresh enough for a socket". If a session exists on the device at all (hasSession(), presence-only), the app now hydrates and reports ready IMMEDIATELY, whatever the token age; the chat list renders from the local DB, the HTTP client refreshes on its first 401, and the socket heals itself via 4001 -&gt; refresh -&gt; reconnect. VC-036 is not regressed: a fresh token is still wanted as early as possible so the first handshake is not doomed, so the refresh is still fired at once — it just runs BEHIND the app instead of in front of it. The no-session path (signed out but a device key survives) still attempts a silent restore, but is now bounded by MAX_SILENT_RESTORE_MS = 4000 so a hibernating backend cannot freeze the splash; a restore that lands later still navigates home on its own, because RootNavigator follows the auth store (state === active). Verified: full jest suite 521/521 pass (5 new hook tests, two of which fail against the old code by hanging until waitFor times out), tsc --noEmit clean, eslint 0 errors. Measured on device: not yet — needs a launch on real hardware to confirm the wall-clock improvement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>VC-052</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Chat thread does not follow the newest message — incoming and own-sent bubbles land hidden behind the composer</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>dev branch, 2026-09-14</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr"/>
+      <c r="F28" s="5" t="inlineStr"/>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>Not independently tested</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: scratchpad/shots/b_fg_follow.png (B at the bottom, F1-F3 arrive, list stays on S8 and the jump FAB appears), scratchpad/shots/b_one.png (single message ONE1 arrives, list left exactly one bubble short), scratchpad/shots/a_own_follow.png (A's OWN sent ONE1 clipped behind the composer), scratchpad/shots/b_offline_send.png (own offline sends clipped). The race explains the intermittency: sometimes the manual scroll lands after the anchor adjustment and it looks fine.
+FIX: the follow now goes through FlashList's `scrollToIndex({index:0})` instead of `scrollToOffset({offset:0})`, fired from `onContentSizeChange` rather than the data effect. Root cause confirmed by reading useRecyclerViewController.js: on every data change FlashList measures how far the FIRST VISIBLE item moved and calls scrollAnchorRef.scrollBy(diff) to cancel the shift, gated on a `pauseOffsetCorrection` ref that ONLY scrollToIndex raises — so a plain offset scroll was undone every time and the thread landed exactly one bubble short. Firing from onContentSizeChange means index 0 has a real layout instead of the stale one it would have in the same commit. Anchoring is deliberately kept: it is the right behaviour for a reader scrolled up in history, whom shouldScrollToLatest still leaves alone; a drag cancels any pending follow so loadOlder growing the content is never mistaken for a new message. An intermediate attempt using scrollToOffset from onContentSizeChange plus a requestAnimationFrame retry was built and tested on device and still landed one bubble short — that is what identified the pauseOffsetCorrection gate. VERIFIED ON DEVICE: a four-message burst now ends with the newest message fully visible above the composer (scratchpad/shots/v2_own_follow.png) where the same burst on the previous build left it clipped (v_own_follow.png). Still to verify with a second device: the INCOMING-message path, and the notification tap-through landing position.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>VC-053</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Chat opened from a notification is titled "Chats" instead of the contact's name, and the avatar loses its initial</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>dev branch, 2026-09-14</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr"/>
+      <c r="F29" s="5" t="inlineStr"/>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>Not independently tested</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: scratchpad/shots/b_tapthrough.png and b_jump.png (header 'Chats' after notification tap) vs scratchpad/shots/b_off_kbd.png (header 'Aayush Jain 🤗' for the same chat opened from the list). Relates to VC-048, which reported the tap-through as not opening the chat at all; the open now works, this is the remaining defect on that path.
+FIX: new pure helper `chatTitle(routeName, rowName, fallback)` in ui/chat/chatModel.ts, covered by chatTitle.test.ts (4 cases, RED first). ChatHeader now resolves the title from the route name, then the conversation row it was already observing for the avatar, and only then a generic label; blank counts as absent in both sources. The avatar initial is taken from the resolved name with an empty fallback, so a genuinely unnamed conversation still falls back to the person glyph instead of showing the initial of a tab label. Needs a second device to re-verify the live tap-through.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>VC-054</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Notification group summary says "N new messages" but N is the number of chats, not the number of messages</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>dev branch, 2026-09-14</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr"/>
+      <c r="F30" s="5" t="inlineStr"/>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>Not independently tested</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: dumpsys output captured twice in the live session (8 messages -&gt; '5 new messages'; 1 message -&gt; '5 new messages').
+FIX: added `PushStore.countedMessages()`, which sums the per-conversation counters the store already held, and postSummary now formats that instead of `countedConversations()`. The &lt;=1 guard that suppresses the summary for a single chat still uses the conversation count, which is correct. Needs a second device to re-verify live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>VC-055</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Every notification is tinted the abandoned violet #7C5CFF, which matches nothing in the shipped monochrome theme</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>dev branch, 2026-09-14</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr"/>
+      <c r="F31" s="5" t="inlineStr"/>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>Not independently tested</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed by reading tokens.ts (brandFrom '#0B0B0C' / '#F5F5F7') against push_strings.xml (#7C5CFF) and by the live dumpsys record color=0xff7c5cff.
+FIX: push_accent is now #0B0B0C, the monochrome brand accent from design-system/tokens.ts, and the misleading resource comment about a violet gradient is replaced. Android resolves this against the shade background for contrast. Needs a second device to re-verify live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>VC-058</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Chat-list preview can regress to an older message — the preview is written unconditionally while the timestamp is guarded</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>dev branch, 2026-09-14</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr"/>
+      <c r="F32" s="5" t="inlineStr"/>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>Not independently tested</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: scratchpad/shots/b_after_reply.png (row reads 'KILL1' while KILL2 was newer). Fix is to move the preview write inside the same freshness check as the timestamp.
+FIX: the preview write now sits behind the same freshness check as the sort key in upsertConversation — a single `fresher` predicate gates both, so a stale patch can no longer overwrite what the row says while being correctly refused a reorder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>VC-060</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Incoming message bubbles are nearly invisible in light theme — #F7F7F8 on #FFFFFF with no border (1.04:1)</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>dev branch, 2026-09-14</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr"/>
+      <c r="F33" s="5" t="inlineStr"/>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>Not independently tested</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: scratchpad/shots/a_relaunch.png — the 'kkr' and 'h' bubbles in light theme. Fix options: give the incoming bubble a hairline in BOTH schemes, or darken `bgSubtle` for this use.
+FIX: the incoming-bubble hairline is no longer dark-only; it applies in both schemes, using the wallpaper-supplied border when the chat has a decorated ground and t.colors.hairline otherwise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>VC-061</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>A 48dp empty band sits between the composer and the keyboard whenever the keyboard is open</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>dev branch, 2026-09-14</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr"/>
+      <c r="F34" s="5" t="inlineStr"/>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>Not independently tested</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: scratchpad/shots/a_cal.png and a_own_follow.png — the white band between the composer pill and the keyboard's suggestion strip. Same file also sets `borderTopWidth: 0` alongside a `borderTopColor`, so the intended separator between the thread and the composer never draws.
+FIX: keyboard-up paddingBottom drops from spacing.huge (48dp) to spacing.xs (8dp), and borderTopWidth goes from 0 to 1 so the separator the style always declared actually draws. VERIFIED ON DEVICE: scratchpad/shots/v2_own_follow.png shows the hairline above the composer and the composer sitting close to the keyboard.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(qa): file seven more chat/notification defects from the code-level audit
VC-063..VC-069 (Jira VC-64..VC-70), found by auditing the same two areas the live
session covered for the failures live testing cannot reach — races, lifecycle
leaks and dead error paths. Two are severe: a body-less realtime frame renders a
permanently blank bubble because the REST recovery is unreachable and the list
would not re-render anyway, and a notification tap into an already-open chat
reuses the screen instance so an unsent draft can be sent to the wrong person.
VC-069 is the false read watermark split out of VC-051, which is now fixed.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA/reports/VelChat-QA-Report.xlsx
+++ b/QA/reports/VelChat-QA-Report.xlsx
@@ -641,7 +641,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-14 04:45 UTC</t>
+          <t>Generated 2026-09-19 08:20 UTC</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -11043,7 +11043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB63"/>
+  <dimension ref="A1:AB70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -18202,7 +18202,11 @@
           <t>VC-52</t>
         </is>
       </c>
-      <c r="C52" s="5" t="inlineStr"/>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>failureScenarios.test.ts: a message dropped by fan-out</t>
+        </is>
+      </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
           <t>A message the device was pushed for never reaches the chat, and no reconnect ever heals it — the sender still sees blue read ticks</t>
@@ -18220,7 +18224,7 @@
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H52" s="5" t="inlineStr">
@@ -18298,7 +18302,11 @@
           <t>Two candidates, not yet separated: (a) the headless push wake posts the notification but its DB write is lost when the process is reaped before the WatermelonDB write commits; (b) the message is never durably fanned out (see VC-001) and the reconnect backfill does not re-request it. Either way the CLIENT-side defect is the same: the `sync {cursor}` + `afterSeq` backfill is not self-healing — a gap that exists once stays forever. The false `read` receipt means a receipt is being emitted from a path that does not require the message row to exist locally.</t>
         </is>
       </c>
-      <c r="V52" s="5" t="inlineStr"/>
+      <c r="V52" s="5" t="inlineStr">
+        <is>
+          <t>CONFIRMED by tracing the whole path. THREE facts compose into permanent loss. (1) A data push delivered to a DEAD process is handled entirely in Kotlin — VelChatMessagingService.handleMessage posts the notification and acks "delivered", then calls PushBridge.emit whose return value is discarded; PushBridge.liveContext() returns null when there is no JS to emit to and, unlike onNewToken/onDeletedMessages, there is NO store.enqueueEvent fallback. So the wake never writes the message to WatermelonDB and leaves no durable record that anything was missed. The only remaining route to the DB is a later REST backfill. (2) Every backfill cursor in the client is MAX(seq) — SyncEngine.pageBackfill, backfillInbox, and the content-fill and load-older paths all derive from maxSeqForConversation/minSeqForConversation — so once ANY newer message lands, the missing seq sits below the cursor and no afterSeq request can ever reach it again. (3) onInboundMessage already did the hard part: it reads localMax BEFORE applying, and shouldProbeGap correctly proves a hole exists — then it called backfillConversation, which re-reads MAX *after* applyServerMessage has moved it up to the revealing seq, so it fetched from ABOVE the hole and repaired nothing. The precisely-correct lower edge was captured, used for the predicate and the loop-guard memo, and then thrown away instead of being used as the fetch cursor.</t>
+        </is>
+      </c>
       <c r="W52" s="5" t="inlineStr"/>
       <c r="X52" s="5" t="inlineStr">
         <is>
@@ -18317,7 +18325,9 @@
       </c>
       <c r="AA52" s="5" t="inlineStr">
         <is>
-          <t>Evidence: scratchpad/shots/a_inline_rx.png (A shows KILL2 09:39 with blue ticks) vs scratchpad/shots/b_kill2_check.png (B's thread jumps BG1 09:37 -&gt; KILL1 09:37 -&gt; hhh 09:40, no KILL2). Related backend defect VC-001 may be the upstream cause, but the client must still heal the gap on reconnect and must not report `read` for a message it does not hold.</t>
+          <t>Evidence: scratchpad/shots/a_inline_rx.png (A shows KILL2 09:39 with blue ticks) vs scratchpad/shots/b_kill2_check.png (B's thread jumps BG1 09:37 -&gt; KILL1 09:37 -&gt; hhh 09:40, no KILL2). Related backend defect VC-001 may be the upstream cause, but the client must still heal the gap on reconnect and must not report `read` for a message it does not hold.
+FIX (frontend): pageBackfill/backfillConversation take an optional `fromSeq`, and the gap probe passes the pre-apply `localMax` — so the repair asks the server from the LOWER edge of the hole instead of from the message that revealed it. Re-fetching the rows already held between localMax and the incoming seq is free: applyServerMessages dedups on (conversation_id, seq) and on client_msg_id inside the write lock. Three end-to-end tests added to failureScenarios.test.ts, driving the real engine against the fake server, written RED first — and rewritten once when the first version passed for the wrong reason (bootConnected’s own reconnect backfill was healing the hole), so each test now brings the socket up while the device is already caught up. Verified: 537/537 jest, tsc clean, eslint 0 errors.
+STILL OPEN, tracked separately: (a) the FALSE READ TICK is not this fix — markConversationRead and read-on-arrival emit a CUMULATIVE read watermark at the local MAX, which covers a missing seq beneath it; clamping every read/delivered watermark to the highest CONTIGUOUS seq actually held is the correct fix and is filed as its own bug because it changes tick semantics everywhere and needs its own tests. (b) a hole detected once is only remembered in memory (gapProbedFrom), so a hole that a probe fails to close is forgotten on restart — persisting unhealed holes for retry is follow-up work. (c) VelChatMessagingService could enqueue a durable `resync` marker when JS is dead, the same fallback its siblings already have. (d) If the backend never durably stored or re-serves the message, no client change recovers it (see VC-001) — the fix then converts silent loss into an honest grey tick rather than a recovery.</t>
         </is>
       </c>
       <c r="AB52" s="5" t="inlineStr"/>
@@ -19742,6 +19752,904 @@
         </is>
       </c>
       <c r="AB63" s="5" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="17" t="inlineStr">
+        <is>
+          <t>VC-063</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>VC-64</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr"/>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>A message whose realtime frame carries no body renders a permanently blank bubble — the REST recovery is dead code and the list would not re-render anyway</t>
+        </is>
+      </c>
+      <c r="E64" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F64" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H64" s="5" t="inlineStr">
+        <is>
+          <t>CLIENT</t>
+        </is>
+      </c>
+      <c r="I64" s="5" t="inlineStr">
+        <is>
+          <t>Chat / messaging — inbound content fill</t>
+        </is>
+      </c>
+      <c r="J64" s="5" t="inlineStr">
+        <is>
+          <t>apps/mobile/src/domain/sync/SyncEngine.ts:1009-1023 + infra/db/syncLogic.ts:20-22 + infra/db/messages.ts:56</t>
+        </is>
+      </c>
+      <c r="K64" s="5" t="inlineStr">
+        <is>
+          <t>Production build</t>
+        </is>
+      </c>
+      <c r="L64" s="5" t="inlineStr">
+        <is>
+          <t>Any Android</t>
+        </is>
+      </c>
+      <c r="M64" s="5" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="N64" s="5" t="inlineStr">
+        <is>
+          <t>Every inbound message whose fan-out frame has no body</t>
+        </is>
+      </c>
+      <c r="O64" s="5" t="inlineStr">
+        <is>
+          <t>Deterministic by code inspection; not yet reproduced live because today's plaintext messages happen to carry `text` on the wire.</t>
+        </is>
+      </c>
+      <c r="P64" s="5" t="inlineStr">
+        <is>
+          <t>A peer sends a message the gateway relays WITHOUT a body — per docs/backend-integration-reference.md §4 the WS payload carries an optional `text`, so media and (at the E2EE phase) every message arrive metadata-only.</t>
+        </is>
+      </c>
+      <c r="Q64" s="5" t="inlineStr">
+        <is>
+          <t>1. Have a peer send a message the gateway relays with no `text` field while the chat is open.
+2. Watch the bubble that appears.
+3. Leave the chat and come back.</t>
+        </is>
+      </c>
+      <c r="R64" s="5" t="inlineStr">
+        <is>
+          <t>The bubble shows the message. SyncEngine already tries: `if (m.content === undefined || m.content === '') { const filled = await fetchMessagesAfter(conv, m.seq - 1); await applyServerMessages(filled); }`.</t>
+        </is>
+      </c>
+      <c r="S64" s="5" t="inlineStr">
+        <is>
+          <t>An empty bubble with only a timestamp, and an empty preview on the chat list. The recovery cannot work, for two independent reasons, and both must be fixed or the bubble stays blank.</t>
+        </is>
+      </c>
+      <c r="T64" s="5" t="inlineStr">
+        <is>
+          <t>A received message shows as blank. The user has no idea what was said and no way to recover it inside the app. At the E2EE phase this would be every single inbound message.</t>
+        </is>
+      </c>
+      <c r="U64" s="5" t="inlineStr">
+        <is>
+          <t>(a) THE FILL IS SKIPPED AS A DUPLICATE. `fetchMessagesAfter(conv, seq-1)` returns the same message, and `reconcileDecision` (syncLogic.ts:20-22) is `if (hasClientMsgIdRow) return 'update'; if (hasSeqRow) return 'skip';`. `hasSeqRow` is true — the row was inserted milliseconds earlier by the `applyServerMessage` on the line above. `hasClientMsgIdRow` can never be true for a peer's message: there is no client_msg_id on the wire, so the insert synthesises `srv_&lt;conversationId&gt;_&lt;seq&gt;` while the REST row carries the sender's real id. The decision is always 'skip', so content_plain is never written and the whole block is dead code for exactly the case its comment names. Every later catch-up funnels through the same decision, so the comment 'content syncs on next catch-up' is also untrue. (b) EVEN IF (a) IS FIXED, NOTHING RE-RENDERS. `observeMessages` is `.observeWithColumns(['state'])`, and WatermelonDB only emits when the matched-record SET changes or a NAMED column changes — a content_plain-only update on an already-matched row emits nothing.</t>
+        </is>
+      </c>
+      <c r="V64" s="5" t="inlineStr"/>
+      <c r="W64" s="5" t="inlineStr"/>
+      <c r="X64" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Y64" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Z64" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA64" s="5" t="inlineStr">
+        <is>
+          <t>Found by a code-level audit after the live session. Fix needs both halves: let the fill update a row matched by seq (e.g. treat a seq row with empty content as 'update'), and name `content_plain` in observeMessages' column list.</t>
+        </is>
+      </c>
+      <c r="AB64" s="5" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="17" t="inlineStr">
+        <is>
+          <t>VC-064</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>VC-65</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr"/>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>Opening a chat from a notification while another chat is on screen keeps the unsent draft — one tap can send it to the wrong person</t>
+        </is>
+      </c>
+      <c r="E65" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F65" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H65" s="5" t="inlineStr">
+        <is>
+          <t>CLIENT</t>
+        </is>
+      </c>
+      <c r="I65" s="5" t="inlineStr">
+        <is>
+          <t>Chat / messaging — notification deep link into a live screen</t>
+        </is>
+      </c>
+      <c r="J65" s="5" t="inlineStr">
+        <is>
+          <t>apps/mobile/src/features/chat/ui/ChatScreen.tsx (local useState) + navigation/RootNavigator.tsx (no getId on the Chat screen)</t>
+        </is>
+      </c>
+      <c r="K65" s="5" t="inlineStr">
+        <is>
+          <t>Production build</t>
+        </is>
+      </c>
+      <c r="L65" s="5" t="inlineStr">
+        <is>
+          <t>Any Android</t>
+        </is>
+      </c>
+      <c r="M65" s="5" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="N65" s="5" t="inlineStr">
+        <is>
+          <t>Every notification tap taken while a different chat is already open</t>
+        </is>
+      </c>
+      <c r="O65" s="5" t="inlineStr">
+        <is>
+          <t>Deterministic by code inspection — the same param-update path that VC-053 was filed and fixed on.</t>
+        </is>
+      </c>
+      <c r="P65" s="5" t="inlineStr">
+        <is>
+          <t>The user is on a chat screen with unsent text in the composer, and taps a notification for a DIFFERENT conversation.</t>
+        </is>
+      </c>
+      <c r="Q65" s="5" t="inlineStr">
+        <is>
+          <t>1. Open the chat with contact A and type a message WITHOUT sending it.
+2. Lock the phone or switch apps, leaving the chat screen mounted.
+3. Receive a message from contact B and tap its notification.
+4. Look at the composer, then press send.</t>
+        </is>
+      </c>
+      <c r="R65" s="5" t="inlineStr">
+        <is>
+          <t>Opening a different conversation starts with an empty composer. A draft belongs to the chat it was written in.</t>
+        </is>
+      </c>
+      <c r="S65" s="5" t="inlineStr">
+        <is>
+          <t>The screen is REUSED, not remounted: the deep link dispatches a NAVIGATE to `Chat`, and with no `getId` configured on the Chat screen the stack router reuses the current route's key and only swaps `route.params`. `useMessages`, `useConversationIdentity` and `useChatHeaderPresence` all re-run on the new conversationId, but every `useState` in ChatScreen survives — so the composer still holds A's text while `send` is now bound to B. One tap sends A's private message to B.</t>
+        </is>
+      </c>
+      <c r="T65" s="5" t="inlineStr">
+        <is>
+          <t>A private message can be delivered to the wrong person with a single tap and no warning. That is a confidentiality failure, not just a UX slip. Lesser symptoms from the same cause: the first keystroke after the switch emits a typing signal to B while the field shows A's words; `offsetRef` carries over, so if the user had scrolled up in A's chat the auto-follow is silently disabled in B's until they scroll once; the jump-to-latest button can appear for a chat already at the bottom.</t>
+        </is>
+      </c>
+      <c r="U65" s="5" t="inlineStr">
+        <is>
+          <t>ChatScreen holds `text`, `offsetRef`, `showJump`/`showJumpRef` and `newestIdRef` in component state and nothing resets them when `conversationId` changes. Fix: either give the Chat screen a `getId: ({ params }) =&gt; params.conversationId` so the deep link remounts it, or reset every piece of local state in an effect keyed on conversationId.</t>
+        </is>
+      </c>
+      <c r="V65" s="5" t="inlineStr"/>
+      <c r="W65" s="5" t="inlineStr"/>
+      <c r="X65" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Y65" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Z65" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA65" s="5" t="inlineStr">
+        <is>
+          <t>Found by a code-level audit. VC-053 fixed the TITLE on this exact entry point, which confirms the param-update path is real and exercised; the state carry-over was not addressed then.</t>
+        </is>
+      </c>
+      <c r="AB65" s="5" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="17" t="inlineStr">
+        <is>
+          <t>VC-065</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>VC-66</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr"/>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>Backing out of a chat mid-resolve strands a 20s presence timer, and can permanently disable the only code that clears it</t>
+        </is>
+      </c>
+      <c r="E66" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F66" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H66" s="5" t="inlineStr">
+        <is>
+          <t>CLIENT</t>
+        </is>
+      </c>
+      <c r="I66" s="5" t="inlineStr">
+        <is>
+          <t>Chat / messaging — header presence</t>
+        </is>
+      </c>
+      <c r="J66" s="5" t="inlineStr">
+        <is>
+          <t>apps/mobile/src/domain/sync/SyncEngine.ts (activatePresence / deactivatePresence / startPeerPresencePolling) + features/chat/hooks/useChatHeaderPresence.ts</t>
+        </is>
+      </c>
+      <c r="K66" s="5" t="inlineStr">
+        <is>
+          <t>Production build</t>
+        </is>
+      </c>
+      <c r="L66" s="5" t="inlineStr">
+        <is>
+          <t>Any Android</t>
+        </is>
+      </c>
+      <c r="M66" s="5" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="N66" s="5" t="inlineStr">
+        <is>
+          <t>Whenever a chat is closed before its presence resolve finishes — a sub-second window, hit often on a slow network or a busy DB</t>
+        </is>
+      </c>
+      <c r="O66" s="5" t="inlineStr">
+        <is>
+          <t>Deterministic by code inspection; needs the chat closed inside the await window.</t>
+        </is>
+      </c>
+      <c r="P66" s="5" t="inlineStr">
+        <is>
+          <t>Open a chat and leave it again before the presence lookup completes.</t>
+        </is>
+      </c>
+      <c r="Q66" s="5" t="inlineStr">
+        <is>
+          <t>1. Open a chat and press back within roughly 300 ms, i.e. before the GET /presence round trip resolves.
+2. Stay out of every chat.
+3. Watch for JS-thread wakeups, or instrument startPeerPresencePolling.</t>
+        </is>
+      </c>
+      <c r="R66" s="5" t="inlineStr">
+        <is>
+          <t>Leaving a chat releases everything it started. Per M7: every timer, listener, socket, subscription and worker is owned and disposable.</t>
+        </is>
+      </c>
+      <c r="S66" s="5" t="inlineStr">
+        <is>
+          <t>activatePresence registers its map entry and starts its interval AFTER two awaits, and no cancellation token reaches it. The screen cleanup runs deactivatePresence first, so the map is empty and clearPeerPresenceTimer has nothing to clear; the promise then resumes and starts a 20 s setInterval for a chat that is closed. Its own guard makes every tick a no-op, so it is an invisible timer waking the JS thread every 20 s until the next chat is opened, a background suspend, or engine stop — and when push is unavailable scheduleSuspend returns early, so it ticks all night. Worse, if the back happens during the SHORTER await (a WatermelonDB find, which blocks behind any in-flight write such as an inbound message batch), deactivatePresence deletes nothing and the entry is written afterwards: activePresencePeers then holds a permanent ghost, its size can never reach 0 again, and clearPeerPresenceTimer inside deactivatePresence becomes dead code for the rest of the session. From then on, closing ANY chat stops clearing its presence poll.</t>
+        </is>
+      </c>
+      <c r="T66" s="5" t="inlineStr">
+        <is>
+          <t>Battery and wakeups on the 3 GB reference device, exactly what the overnight-background contract M13 forbids. Silent, and a later chat open masks it because startPeerPresencePolling clears the timer first — which is why live testing never catches it.</t>
+        </is>
+      </c>
+      <c r="U66" s="5" t="inlineStr">
+        <is>
+          <t>State is registered after awaits with no cancellation. Fix: capture a generation token before the first await and bail if deactivatePresence has run since, or register the map entry BEFORE the awaits so deactivate can always see it.</t>
+        </is>
+      </c>
+      <c r="V66" s="5" t="inlineStr"/>
+      <c r="W66" s="5" t="inlineStr"/>
+      <c r="X66" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Y66" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Z66" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA66" s="5" t="inlineStr">
+        <is>
+          <t>Found by a code-level audit after the live two-device session.</t>
+        </is>
+      </c>
+      <c r="AB66" s="5" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="17" t="inlineStr">
+        <is>
+          <t>VC-066</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>VC-67</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr"/>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>PushStore's JSON blobs are read-modify-write across three threads — notification lines and counts can be lost or resurrected</t>
+        </is>
+      </c>
+      <c r="E67" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F67" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H67" s="5" t="inlineStr">
+        <is>
+          <t>CLIENT</t>
+        </is>
+      </c>
+      <c r="I67" s="5" t="inlineStr">
+        <is>
+          <t>Notifications — native state store</t>
+        </is>
+      </c>
+      <c r="J67" s="5" t="inlineStr">
+        <is>
+          <t>apps/mobile/android/app/src/main/java/com/velchat/push/PushStore.kt (appendLine, clearLines, bumpCount, clearCount, setLastSeq, setMuted, setAvatars)</t>
+        </is>
+      </c>
+      <c r="K67" s="5" t="inlineStr">
+        <is>
+          <t>Production build</t>
+        </is>
+      </c>
+      <c r="L67" s="5" t="inlineStr">
+        <is>
+          <t>Any Android</t>
+        </is>
+      </c>
+      <c r="M67" s="5" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="N67" s="5" t="inlineStr">
+        <is>
+          <t>Whenever two of the three writer threads overlap — a push landing while a chat is opened or a notification dismissed</t>
+        </is>
+      </c>
+      <c r="O67" s="5" t="inlineStr">
+        <is>
+          <t>Race — rare per attempt, inevitable at scale.</t>
+        </is>
+      </c>
+      <c r="P67" s="5" t="inlineStr">
+        <is>
+          <t>A push for one conversation arriving while the app clears another conversation's notification.</t>
+        </is>
+      </c>
+      <c r="Q67" s="5" t="inlineStr">
+        <is>
+          <t>1. Open chat B from its notification, so the RN native-modules thread runs clearLines for B.
+2. In the same window, have a push for chat A arrive, so the FCM delivery thread runs appendLine for A.
+3. Later, receive one new message in chat B and expand its notification.</t>
+        </is>
+      </c>
+      <c r="R67" s="5" t="inlineStr">
+        <is>
+          <t>Each conversation's stored lines and counts are independent, and every update is durable.</t>
+        </is>
+      </c>
+      <c r="S67" s="5" t="inlineStr">
+        <is>
+          <t>Each of the five maps — lines, counts, lastSeq, muted, avatars — is ONE SharedPreferences string holding every conversation, read whole and written back whole. Two threads that read before either writes will have the later write clobber the earlier. If the FCM thread wins, B's six lines survive its cancellation and the next message in B rebuilds the thread with every line the user already read — the VC-057 symptom, resurrected as a race rather than a missing call. If the other side wins, A's new line is lost and the notification shows only older lines for the message that just arrived. The same shape on counts either re-establishes a count the user just dismissed or drops a bump, and those counts feed the group summary total.</t>
+        </is>
+      </c>
+      <c r="T67" s="5" t="inlineStr">
+        <is>
+          <t>Notifications intermittently re-show read messages, drop the message that just arrived, or report a total that matches nothing. Non-deterministic, so it reads to the user as the app being unreliable.</t>
+        </is>
+      </c>
+      <c r="U67" s="5" t="inlineStr">
+        <is>
+          <t>The class doc claims every accessor is safe from any thread because SharedPreferences is internally synchronised. That is true for a single getString or putString and false for the read-then-write pairs used throughout. Three writers in one process: VelChatMessagingService on FCM's delivery thread, PushActionReceiver on the main thread, VelChatPushModule on the RN native-modules thread. Fix: one synchronized lock around every read-modify-write in the class; all callers share a single SharedPreferences instance in a single process, so that is sufficient.</t>
+        </is>
+      </c>
+      <c r="V67" s="5" t="inlineStr"/>
+      <c r="W67" s="5" t="inlineStr"/>
+      <c r="X67" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Y67" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Z67" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA67" s="5" t="inlineStr">
+        <is>
+          <t>Distinct from VC-033, which is about the pending-event queue. This is the other five maps. Found by a code-level audit after the live two-device session.</t>
+        </is>
+      </c>
+      <c r="AB67" s="5" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="17" t="inlineStr">
+        <is>
+          <t>VC-067</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>VC-68</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr"/>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>Swiping a notification away clears its count but keeps its message lines, so dismissed messages reappear in the next notification</t>
+        </is>
+      </c>
+      <c r="E68" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F68" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H68" s="5" t="inlineStr">
+        <is>
+          <t>CLIENT</t>
+        </is>
+      </c>
+      <c r="I68" s="5" t="inlineStr">
+        <is>
+          <t>Notifications — dismiss</t>
+        </is>
+      </c>
+      <c r="J68" s="5" t="inlineStr">
+        <is>
+          <t>apps/mobile/android/app/src/main/java/com/velchat/push/PushActionReceiver.kt (ACTION_DISMISS) + PushNotifications.kt (postSummary has no delete intent)</t>
+        </is>
+      </c>
+      <c r="K68" s="5" t="inlineStr">
+        <is>
+          <t>Production build</t>
+        </is>
+      </c>
+      <c r="L68" s="5" t="inlineStr">
+        <is>
+          <t>Any Android</t>
+        </is>
+      </c>
+      <c r="M68" s="5" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="N68" s="5" t="inlineStr">
+        <is>
+          <t>Every dismissed notification followed by a new message in the same chat</t>
+        </is>
+      </c>
+      <c r="O68" s="5" t="inlineStr">
+        <is>
+          <t>Deterministic</t>
+        </is>
+      </c>
+      <c r="P68" s="5" t="inlineStr">
+        <is>
+          <t>A conversation whose notification the user swiped away without reading.</t>
+        </is>
+      </c>
+      <c r="Q68" s="5" t="inlineStr">
+        <is>
+          <t>1. Let three messages from one contact arrive while the app is backgrounded; the notification lists three lines.
+2. Swipe the notification away without opening the chat.
+3. Have that contact send one more message.
+4. Expand the new notification.</t>
+        </is>
+      </c>
+      <c r="R68" s="5" t="inlineStr">
+        <is>
+          <t>The new notification lists only the new message. Every other teardown path clears both halves — PushNotifications.cancel does clearCount AND clearLines, with a comment saying exactly why.</t>
+        </is>
+      </c>
+      <c r="S68" s="5" t="inlineStr">
+        <is>
+          <t>The dismiss branch clears only the count and returns. The stored lines survive, so appendLine returns all four and the rebuilt MessagingStyle re-lists the three messages the user deliberately dismissed, while setNumber says 1.</t>
+        </is>
+      </c>
+      <c r="T68" s="5" t="inlineStr">
+        <is>
+          <t>Dismissing a notification does not actually dismiss its contents. The user reads four new messages for one new arrival, and the dismissal gesture stops meaning anything.</t>
+        </is>
+      </c>
+      <c r="U68" s="5" t="inlineStr">
+        <is>
+          <t>A separate receiver branch that the VC-057 fix did not reach; it needs the same clearLines the cancel path has. SECONDARY, same area: postSummary builds the group summary with setGroupSummary true and NO delete intent, unlike every per-conversation notification — so dismissing the bundle runs none of our clearing for the summary, and on any OEM build that does not deliver child delete intents on a group dismissal the counts survive wholesale and the next single message re-posts a summary counting messages already swept away.</t>
+        </is>
+      </c>
+      <c r="V68" s="5" t="inlineStr"/>
+      <c r="W68" s="5" t="inlineStr"/>
+      <c r="X68" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Y68" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Z68" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA68" s="5" t="inlineStr">
+        <is>
+          <t>Found by a code-level audit after the live two-device session. Deterministic, unlike the race in the sibling PushStore report.</t>
+        </is>
+      </c>
+      <c r="AB68" s="5" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="17" t="inlineStr">
+        <is>
+          <t>VC-068</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>VC-69</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr"/>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>Every load-older page re-runs the open-the-chat side effects, briefly un-suppressing notifications for the chat on screen</t>
+        </is>
+      </c>
+      <c r="E69" s="19" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F69" s="19" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H69" s="5" t="inlineStr">
+        <is>
+          <t>CLIENT</t>
+        </is>
+      </c>
+      <c r="I69" s="5" t="inlineStr">
+        <is>
+          <t>Chat / messaging — history pagination</t>
+        </is>
+      </c>
+      <c r="J69" s="5" t="inlineStr">
+        <is>
+          <t>apps/mobile/src/features/chat/hooks/useMessages.ts (the effect's dependency array includes limit)</t>
+        </is>
+      </c>
+      <c r="K69" s="5" t="inlineStr">
+        <is>
+          <t>Production build</t>
+        </is>
+      </c>
+      <c r="L69" s="5" t="inlineStr">
+        <is>
+          <t>Any Android</t>
+        </is>
+      </c>
+      <c r="M69" s="5" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="N69" s="5" t="inlineStr">
+        <is>
+          <t>Once per page of scrollback</t>
+        </is>
+      </c>
+      <c r="O69" s="5" t="inlineStr">
+        <is>
+          <t>Deterministic for the wasted work; the notification window is a race inside it.</t>
+        </is>
+      </c>
+      <c r="P69" s="5" t="inlineStr">
+        <is>
+          <t>A conversation with enough history to page through.</t>
+        </is>
+      </c>
+      <c r="Q69" s="5" t="inlineStr">
+        <is>
+          <t>1. Open a long chat and scroll up through several pages of history.
+2. Watch the network: a receipts fetch and a read frame go out per page.
+3. Have the peer send a message during the scrollback.</t>
+        </is>
+      </c>
+      <c r="R69" s="5" t="inlineStr">
+        <is>
+          <t>Opening a chat is a one-time act. Growing the local window should only re-subscribe the message query.</t>
+        </is>
+      </c>
+      <c r="S69" s="5" t="inlineStr">
+        <is>
+          <t>The effect is keyed on conversationId, meId and limit, but only observeMessages depends on limit. Each loadOlder therefore tears the effect down and re-runs ALL of it: a receipts GET, a read receipt frame, a clearConversation bridge call, and the pair setActiveConversationForPush(null) then setActiveConversationForPush(conversationId). Those two are async bridge calls, so for the length of one native round trip the native side believes NO chat is on screen — and a push landing in that window posts a heads-up notification for the chat the user is staring at, the exact failure the active-conversation mechanism exists to prevent. Ten pages of scrollback is ten such windows.</t>
+        </is>
+      </c>
+      <c r="T69" s="5" t="inlineStr">
+        <is>
+          <t>Redundant network on every page of scrollback, and an occasional notification for the conversation that is currently open. The engine's own window is zero-width because setActiveConversation is synchronous; only the native mirror is exposed.</t>
+        </is>
+      </c>
+      <c r="U69" s="5" t="inlineStr">
+        <is>
+          <t>One effect doing two jobs. Split it: keep the observeMessages subscription keyed on limit, and move the open-the-chat actions plus the AppState listener into an effect keyed on conversationId alone.</t>
+        </is>
+      </c>
+      <c r="V69" s="5" t="inlineStr"/>
+      <c r="W69" s="5" t="inlineStr"/>
+      <c r="X69" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Y69" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Z69" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA69" s="5" t="inlineStr">
+        <is>
+          <t>Found by a code-level audit after the live two-device session.</t>
+        </is>
+      </c>
+      <c r="AB69" s="5" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="17" t="inlineStr">
+        <is>
+          <t>VC-069</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>VC-70</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr"/>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>The read watermark is sent at the local MAX seq, so it covers messages the device does not hold — the sender gets a blue tick for a message that was never received</t>
+        </is>
+      </c>
+      <c r="E70" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F70" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G70" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H70" s="5" t="inlineStr">
+        <is>
+          <t>CLIENT</t>
+        </is>
+      </c>
+      <c r="I70" s="5" t="inlineStr">
+        <is>
+          <t>Chat / messaging — read receipts</t>
+        </is>
+      </c>
+      <c r="J70" s="5" t="inlineStr">
+        <is>
+          <t>apps/mobile/src/domain/sync/SyncEngine.ts (markConversationRead, read-on-arrival, pageBackfill) + infra/db/receiptLedger.ts</t>
+        </is>
+      </c>
+      <c r="K70" s="5" t="inlineStr">
+        <is>
+          <t>Production build, live backend</t>
+        </is>
+      </c>
+      <c r="L70" s="5" t="inlineStr">
+        <is>
+          <t>Both test devices</t>
+        </is>
+      </c>
+      <c r="M70" s="5" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="N70" s="5" t="inlineStr">
+        <is>
+          <t>Every time a conversation has a hole in its seq range</t>
+        </is>
+      </c>
+      <c r="O70" s="5" t="inlineStr">
+        <is>
+          <t>Observed live twice, and confirmed deterministic by code inspection.</t>
+        </is>
+      </c>
+      <c r="P70" s="5" t="inlineStr">
+        <is>
+          <t>The device is missing a message at some seq N while holding messages above it — e.g. after a fan-out drop, the exact condition VC-051 describes.</t>
+        </is>
+      </c>
+      <c r="Q70" s="5" t="inlineStr">
+        <is>
+          <t>1. Arrange for a message at seq N to be missing locally while N+1 and above are present (see VC-051 for the repro).
+2. Open that conversation on the recipient device.
+3. Look at the tick state for message N on the SENDER.</t>
+        </is>
+      </c>
+      <c r="R70" s="5" t="inlineStr">
+        <is>
+          <t>A read receipt means the recipient saw the message. A device must never acknowledge a seq it does not hold.</t>
+        </is>
+      </c>
+      <c r="S70" s="5" t="inlineStr">
+        <is>
+          <t>Receipts are cumulative watermarks — one frame carries upToSeq and covers every message at or below it — and every emitter derives that number from the local MAX seq, not the highest CONTIGUOUS seq. markConversationRead runs on every chat open and on the notification read and reply actions, and uses maxSeqForConversation; read-on-arrival uses the incoming seq itself, so the very frame that OPENS a hole immediately reports read up to its own seq; the backfill loop does the same with its highest page seq. A native path acknowledges read straight over REST from a process with no database open at all. Nothing anywhere checks that a row exists for the seq being acknowledged, and mergeWatermark is monotonic, so an over-advanced read is permanent for the life of the install.</t>
+        </is>
+      </c>
+      <c r="T70" s="5" t="inlineStr">
+        <is>
+          <t>Read receipts stop meaning anything in exactly the situation where they matter most. A sender is told a message was read when the recipient never received it and never will — which is how the VC-051 message loss stayed invisible to both sides. It also clears the recipient's unread badge for messages they have never seen.</t>
+        </is>
+      </c>
+      <c r="U70" s="5" t="inlineStr">
+        <is>
+          <t>CONFIRMED in code. Fix: replace the maxSeqForConversation used for RECEIPTS with a highest-contiguous-seq query (highest seq with no hole beneath it, relative to the conversation's known floor so that trimmed history and deleted messages are not mistaken for holes), and clamp the read-on-arrival seq to that value so the frame that opens a hole reports only up to the previous localMax. The same clamp applies to the delivered watermark fed from push. Deliberately NOT bundled with the VC-051 backfill fix: it changes tick semantics on every path and needs its own tests, and getting the floor wrong would under-report reads, which is a worse bug than the one being fixed.</t>
+        </is>
+      </c>
+      <c r="V70" s="5" t="inlineStr"/>
+      <c r="W70" s="5" t="inlineStr"/>
+      <c r="X70" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Y70" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Z70" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA70" s="5" t="inlineStr">
+        <is>
+          <t>Split out of VC-051 during that investigation. VC-062 (a backgrounded-but-mounted chat marking arrivals read) widened the window and is fixed; this is the independent, underlying defect.</t>
+        </is>
+      </c>
+      <c r="AB70" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:AB1"/>
@@ -19755,7 +20663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -19908,7 +20816,7 @@
         </is>
       </c>
       <c r="B15" s="23" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C15" s="24" t="inlineStr"/>
     </row>
@@ -19919,7 +20827,7 @@
         </is>
       </c>
       <c r="B16" s="23" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C16" s="24" t="inlineStr"/>
     </row>
@@ -19930,7 +20838,7 @@
         </is>
       </c>
       <c r="B17" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C17" s="24" t="inlineStr"/>
     </row>
@@ -19941,7 +20849,7 @@
         </is>
       </c>
       <c r="B18" s="23" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C18" s="24" t="inlineStr"/>
     </row>
@@ -19952,7 +20860,7 @@
         </is>
       </c>
       <c r="B19" s="23" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C19" s="24" t="inlineStr"/>
     </row>
@@ -20011,7 +20919,7 @@
       </c>
       <c r="C26" s="26" t="inlineStr">
         <is>
-          <t>18 open P0/P1 defect(s) block the build.</t>
+          <t>20 open P0/P1 defect(s) block the build.</t>
         </is>
       </c>
     </row>
@@ -20316,17 +21224,51 @@
     <row r="46">
       <c r="A46" s="22" t="inlineStr">
         <is>
-          <t>VC-051</t>
+          <t>VC-063</t>
         </is>
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="C46" s="24" t="inlineStr">
         <is>
-          <t>A message the device was pushed for never reaches the chat, and no reconnect ever heals it — the sender still sees blue read ticks</t>
+          <t>A message whose realtime frame carries no body renders a permanently blank bubble — the REST recovery is dead code and the list would not re-render anyway</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="22" t="inlineStr">
+        <is>
+          <t>VC-064</t>
+        </is>
+      </c>
+      <c r="B47" s="23" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C47" s="24" t="inlineStr">
+        <is>
+          <t>Opening a chat from a notification while another chat is on screen keeps the unsent draft — one tap can send it to the wrong person</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="22" t="inlineStr">
+        <is>
+          <t>VC-069</t>
+        </is>
+      </c>
+      <c r="B48" s="23" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C48" s="24" t="inlineStr">
+        <is>
+          <t>The read watermark is sent at the local MAX seq, so it covers messages the device does not hold — the sender gets a blue tick for a message that was never received</t>
         </is>
       </c>
     </row>
@@ -20479,7 +21421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -21519,25 +22461,29 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>VC-052</t>
+          <t>VC-051</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Chat thread does not follow the newest message — incoming and own-sent bubbles land hidden behind the composer</t>
+          <t>A message the device was pushed for never reaches the chat, and no reconnect ever heals it — the sender still sees blue read ticks</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>dev branch, 2026-09-14</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr"/>
+          <t>dev branch, 2026-09-19</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>failureScenarios.test.ts: a message dropped by fan-out</t>
+        </is>
+      </c>
       <c r="F28" s="5" t="inlineStr"/>
       <c r="G28" s="5" t="inlineStr">
         <is>
@@ -21546,20 +22492,21 @@
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>Evidence: scratchpad/shots/b_fg_follow.png (B at the bottom, F1-F3 arrive, list stays on S8 and the jump FAB appears), scratchpad/shots/b_one.png (single message ONE1 arrives, list left exactly one bubble short), scratchpad/shots/a_own_follow.png (A's OWN sent ONE1 clipped behind the composer), scratchpad/shots/b_offline_send.png (own offline sends clipped). The race explains the intermittency: sometimes the manual scroll lands after the anchor adjustment and it looks fine.
-FIX: the follow now goes through FlashList's `scrollToIndex({index:0})` instead of `scrollToOffset({offset:0})`, fired from `onContentSizeChange` rather than the data effect. Root cause confirmed by reading useRecyclerViewController.js: on every data change FlashList measures how far the FIRST VISIBLE item moved and calls scrollAnchorRef.scrollBy(diff) to cancel the shift, gated on a `pauseOffsetCorrection` ref that ONLY scrollToIndex raises — so a plain offset scroll was undone every time and the thread landed exactly one bubble short. Firing from onContentSizeChange means index 0 has a real layout instead of the stale one it would have in the same commit. Anchoring is deliberately kept: it is the right behaviour for a reader scrolled up in history, whom shouldScrollToLatest still leaves alone; a drag cancels any pending follow so loadOlder growing the content is never mistaken for a new message. An intermediate attempt using scrollToOffset from onContentSizeChange plus a requestAnimationFrame retry was built and tested on device and still landed one bubble short — that is what identified the pauseOffsetCorrection gate. VERIFIED ON DEVICE: a four-message burst now ends with the newest message fully visible above the composer (scratchpad/shots/v2_own_follow.png) where the same burst on the previous build left it clipped (v_own_follow.png). Still to verify with a second device: the INCOMING-message path, and the notification tap-through landing position.</t>
+          <t>Evidence: scratchpad/shots/a_inline_rx.png (A shows KILL2 09:39 with blue ticks) vs scratchpad/shots/b_kill2_check.png (B's thread jumps BG1 09:37 -&gt; KILL1 09:37 -&gt; hhh 09:40, no KILL2). Related backend defect VC-001 may be the upstream cause, but the client must still heal the gap on reconnect and must not report `read` for a message it does not hold.
+FIX (frontend): pageBackfill/backfillConversation take an optional `fromSeq`, and the gap probe passes the pre-apply `localMax` — so the repair asks the server from the LOWER edge of the hole instead of from the message that revealed it. Re-fetching the rows already held between localMax and the incoming seq is free: applyServerMessages dedups on (conversation_id, seq) and on client_msg_id inside the write lock. Three end-to-end tests added to failureScenarios.test.ts, driving the real engine against the fake server, written RED first — and rewritten once when the first version passed for the wrong reason (bootConnected’s own reconnect backfill was healing the hole), so each test now brings the socket up while the device is already caught up. Verified: 537/537 jest, tsc clean, eslint 0 errors.
+STILL OPEN, tracked separately: (a) the FALSE READ TICK is not this fix — markConversationRead and read-on-arrival emit a CUMULATIVE read watermark at the local MAX, which covers a missing seq beneath it; clamping every read/delivered watermark to the highest CONTIGUOUS seq actually held is the correct fix and is filed as its own bug because it changes tick semantics everywhere and needs its own tests. (b) a hole detected once is only remembered in memory (gapProbedFrom), so a hole that a probe fails to close is forgotten on restart — persisting unhealed holes for retry is follow-up work. (c) VelChatMessagingService could enqueue a durable `resync` marker when JS is dead, the same fallback its siblings already have. (d) If the backend never durably stored or re-serves the message, no client change recovers it (see VC-001) — the fix then converts silent loss into an honest grey tick rather than a recovery.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>VC-053</t>
+          <t>VC-052</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Chat opened from a notification is titled "Chats" instead of the contact's name, and the avatar loses its initial</t>
+          <t>Chat thread does not follow the newest message — incoming and own-sent bubbles land hidden behind the composer</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
@@ -21581,25 +22528,25 @@
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>Evidence: scratchpad/shots/b_tapthrough.png and b_jump.png (header 'Chats' after notification tap) vs scratchpad/shots/b_off_kbd.png (header 'Aayush Jain 🤗' for the same chat opened from the list). Relates to VC-048, which reported the tap-through as not opening the chat at all; the open now works, this is the remaining defect on that path.
-FIX: new pure helper `chatTitle(routeName, rowName, fallback)` in ui/chat/chatModel.ts, covered by chatTitle.test.ts (4 cases, RED first). ChatHeader now resolves the title from the route name, then the conversation row it was already observing for the avatar, and only then a generic label; blank counts as absent in both sources. The avatar initial is taken from the resolved name with an empty fallback, so a genuinely unnamed conversation still falls back to the person glyph instead of showing the initial of a tab label. Needs a second device to re-verify the live tap-through.</t>
+          <t>Evidence: scratchpad/shots/b_fg_follow.png (B at the bottom, F1-F3 arrive, list stays on S8 and the jump FAB appears), scratchpad/shots/b_one.png (single message ONE1 arrives, list left exactly one bubble short), scratchpad/shots/a_own_follow.png (A's OWN sent ONE1 clipped behind the composer), scratchpad/shots/b_offline_send.png (own offline sends clipped). The race explains the intermittency: sometimes the manual scroll lands after the anchor adjustment and it looks fine.
+FIX: the follow now goes through FlashList's `scrollToIndex({index:0})` instead of `scrollToOffset({offset:0})`, fired from `onContentSizeChange` rather than the data effect. Root cause confirmed by reading useRecyclerViewController.js: on every data change FlashList measures how far the FIRST VISIBLE item moved and calls scrollAnchorRef.scrollBy(diff) to cancel the shift, gated on a `pauseOffsetCorrection` ref that ONLY scrollToIndex raises — so a plain offset scroll was undone every time and the thread landed exactly one bubble short. Firing from onContentSizeChange means index 0 has a real layout instead of the stale one it would have in the same commit. Anchoring is deliberately kept: it is the right behaviour for a reader scrolled up in history, whom shouldScrollToLatest still leaves alone; a drag cancels any pending follow so loadOlder growing the content is never mistaken for a new message. An intermediate attempt using scrollToOffset from onContentSizeChange plus a requestAnimationFrame retry was built and tested on device and still landed one bubble short — that is what identified the pauseOffsetCorrection gate. VERIFIED ON DEVICE: a four-message burst now ends with the newest message fully visible above the composer (scratchpad/shots/v2_own_follow.png) where the same burst on the previous build left it clipped (v_own_follow.png). Still to verify with a second device: the INCOMING-message path, and the notification tap-through landing position.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>VC-054</t>
+          <t>VC-053</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Notification group summary says "N new messages" but N is the number of chats, not the number of messages</t>
+          <t>Chat opened from a notification is titled "Chats" instead of the contact's name, and the avatar loses its initial</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
@@ -21616,20 +22563,20 @@
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>Evidence: dumpsys output captured twice in the live session (8 messages -&gt; '5 new messages'; 1 message -&gt; '5 new messages').
-FIX: added `PushStore.countedMessages()`, which sums the per-conversation counters the store already held, and postSummary now formats that instead of `countedConversations()`. The &lt;=1 guard that suppresses the summary for a single chat still uses the conversation count, which is correct. Needs a second device to re-verify live.</t>
+          <t>Evidence: scratchpad/shots/b_tapthrough.png and b_jump.png (header 'Chats' after notification tap) vs scratchpad/shots/b_off_kbd.png (header 'Aayush Jain 🤗' for the same chat opened from the list). Relates to VC-048, which reported the tap-through as not opening the chat at all; the open now works, this is the remaining defect on that path.
+FIX: new pure helper `chatTitle(routeName, rowName, fallback)` in ui/chat/chatModel.ts, covered by chatTitle.test.ts (4 cases, RED first). ChatHeader now resolves the title from the route name, then the conversation row it was already observing for the avatar, and only then a generic label; blank counts as absent in both sources. The avatar initial is taken from the resolved name with an empty fallback, so a genuinely unnamed conversation still falls back to the person glyph instead of showing the initial of a tab label. Needs a second device to re-verify the live tap-through.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>VC-055</t>
+          <t>VC-054</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Every notification is tinted the abandoned violet #7C5CFF, which matches nothing in the shipped monochrome theme</t>
+          <t>Notification group summary says "N new messages" but N is the number of chats, not the number of messages</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
@@ -21651,20 +22598,20 @@
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>Confirmed by reading tokens.ts (brandFrom '#0B0B0C' / '#F5F5F7') against push_strings.xml (#7C5CFF) and by the live dumpsys record color=0xff7c5cff.
-FIX: push_accent is now #0B0B0C, the monochrome brand accent from design-system/tokens.ts, and the misleading resource comment about a violet gradient is replaced. Android resolves this against the shade background for contrast. Needs a second device to re-verify live.</t>
+          <t>Evidence: dumpsys output captured twice in the live session (8 messages -&gt; '5 new messages'; 1 message -&gt; '5 new messages').
+FIX: added `PushStore.countedMessages()`, which sums the per-conversation counters the store already held, and postSummary now formats that instead of `countedConversations()`. The &lt;=1 guard that suppresses the summary for a single chat still uses the conversation count, which is correct. Needs a second device to re-verify live.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>VC-057</t>
+          <t>VC-055</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Notification re-lists messages the user has already read once the chat is reopened and a new message arrives</t>
+          <t>Every notification is tinted the abandoned violet #7C5CFF, which matches nothing in the shipped monochrome theme</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
@@ -21686,20 +22633,20 @@
       </c>
       <c r="H32" s="5" t="inlineStr">
         <is>
-          <t>Evidence: scratchpad/shots/b_shade.png (S3..S8 before opening), scratchpad/shots/b_tapthrough.png (chat opened, tray cleared, all read), scratchpad/shots/b_reply_open.png (next notification still carries S6, S7, S8, BG1).
-ROOT CAUSE FOUND and FIXED via VC-062. The clearing path was wired correctly all along — clearConversationNotification -&gt; VelChatPushModule.clearConversation -&gt; PushNotifications.cancel -&gt; store.clearLines — but it only ran from the chat screen's MOUNT effect. A notification tap RESUMES an already-mounted ChatScreen, so that effect never re-ran, and the tray entry disappearing was just the notification's own AUTO_CANCEL flag removing the posted notification while the stored lines and counters survived. useMessages now also clears on every return to the foreground. Live re-verification pending a second device.</t>
+          <t>Confirmed by reading tokens.ts (brandFrom '#0B0B0C' / '#F5F5F7') against push_strings.xml (#7C5CFF) and by the live dumpsys record color=0xff7c5cff.
+FIX: push_accent is now #0B0B0C, the monochrome brand accent from design-system/tokens.ts, and the misleading resource comment about a violet gradient is replaced. Android resolves this against the shade background for contrast. Needs a second device to re-verify live.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>VC-058</t>
+          <t>VC-057</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Chat-list preview can regress to an older message — the preview is written unconditionally while the timestamp is guarded</t>
+          <t>Notification re-lists messages the user has already read once the chat is reopened and a new message arrives</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -21721,25 +22668,25 @@
       </c>
       <c r="H33" s="5" t="inlineStr">
         <is>
-          <t>Evidence: scratchpad/shots/b_after_reply.png (row reads 'KILL1' while KILL2 was newer). Fix is to move the preview write inside the same freshness check as the timestamp.
-FIX: the preview write now sits behind the same freshness check as the sort key in upsertConversation — a single `fresher` predicate gates both, so a stale patch can no longer overwrite what the row says while being correctly refused a reorder.</t>
+          <t>Evidence: scratchpad/shots/b_shade.png (S3..S8 before opening), scratchpad/shots/b_tapthrough.png (chat opened, tray cleared, all read), scratchpad/shots/b_reply_open.png (next notification still carries S6, S7, S8, BG1).
+ROOT CAUSE FOUND and FIXED via VC-062. The clearing path was wired correctly all along — clearConversationNotification -&gt; VelChatPushModule.clearConversation -&gt; PushNotifications.cancel -&gt; store.clearLines — but it only ran from the chat screen's MOUNT effect. A notification tap RESUMES an already-mounted ChatScreen, so that effect never re-ran, and the tray entry disappearing was just the notification's own AUTO_CANCEL flag removing the posted notification while the stored lines and counters survived. useMessages now also clears on every return to the foreground. Live re-verification pending a second device.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>VC-060</t>
+          <t>VC-058</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Incoming message bubbles are nearly invisible in light theme — #F7F7F8 on #FFFFFF with no border (1.04:1)</t>
+          <t>Chat-list preview can regress to an older message — the preview is written unconditionally while the timestamp is guarded</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
@@ -21756,20 +22703,20 @@
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>Evidence: scratchpad/shots/a_relaunch.png — the 'kkr' and 'h' bubbles in light theme. Fix options: give the incoming bubble a hairline in BOTH schemes, or darken `bgSubtle` for this use.
-FIX: the incoming-bubble hairline is no longer dark-only; it applies in both schemes, using the wallpaper-supplied border when the chat has a decorated ground and t.colors.hairline otherwise.</t>
+          <t>Evidence: scratchpad/shots/b_after_reply.png (row reads 'KILL1' while KILL2 was newer). Fix is to move the preview write inside the same freshness check as the timestamp.
+FIX: the preview write now sits behind the same freshness check as the sort key in upsertConversation — a single `fresher` predicate gates both, so a stale patch can no longer overwrite what the row says while being correctly refused a reorder.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>VC-061</t>
+          <t>VC-060</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>A 48dp empty band sits between the composer and the keyboard whenever the keyboard is open</t>
+          <t>Incoming message bubbles are nearly invisible in light theme — #F7F7F8 on #FFFFFF with no border (1.04:1)</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
@@ -21791,44 +22738,79 @@
       </c>
       <c r="H35" s="5" t="inlineStr">
         <is>
+          <t>Evidence: scratchpad/shots/a_relaunch.png — the 'kkr' and 'h' bubbles in light theme. Fix options: give the incoming bubble a hairline in BOTH schemes, or darken `bgSubtle` for this use.
+FIX: the incoming-bubble hairline is no longer dark-only; it applies in both schemes, using the wallpaper-supplied border when the chat has a decorated ground and t.colors.hairline otherwise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>VC-061</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>A 48dp empty band sits between the composer and the keyboard whenever the keyboard is open</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>dev branch, 2026-09-14</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr"/>
+      <c r="F36" s="5" t="inlineStr"/>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>Not independently tested</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
           <t>Evidence: scratchpad/shots/a_cal.png and a_own_follow.png — the white band between the composer pill and the keyboard's suggestion strip. Same file also sets `borderTopWidth: 0` alongside a `borderTopColor`, so the intended separator between the thread and the composer never draws.
 FIX: keyboard-up paddingBottom drops from spacing.huge (48dp) to spacing.xs (8dp), and borderTopWidth goes from 0 to 1 so the separator the style always declared actually draws. VERIFIED ON DEVICE: scratchpad/shots/v2_own_follow.png shows the hairline above the composer and the composer sitting close to the keyboard.</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>VC-062</t>
         </is>
       </c>
-      <c r="B36" s="5" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>A chat left open while the app is backgrounded keeps marking arriving messages read — the sender gets a blue tick for a message nobody has seen</t>
         </is>
       </c>
-      <c r="C36" s="5" t="inlineStr">
+      <c r="C37" s="5" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D36" s="5" t="inlineStr">
+      <c r="D37" s="5" t="inlineStr">
         <is>
           <t>dev branch, 2026-09-14</t>
         </is>
       </c>
-      <c r="E36" s="5" t="inlineStr">
+      <c r="E37" s="5" t="inlineStr">
         <is>
           <t>chatVisibility.test.tsx: the chat only counts as on screen while it is visible</t>
         </is>
       </c>
-      <c r="F36" s="5" t="inlineStr"/>
-      <c r="G36" s="5" t="inlineStr">
+      <c r="F37" s="5" t="inlineStr"/>
+      <c r="G37" s="5" t="inlineStr">
         <is>
           <t>Not independently tested</t>
         </is>
       </c>
-      <c r="H36" s="5" t="inlineStr">
+      <c r="H37" s="5" t="inlineStr">
         <is>
           <t>Found while tracing VC-057. Same listener is also the only place a notification TAP can clear a conversation's stored notification lines, because tapping resumes an ALREADY-MOUNTED chat screen and the mount effect never re-runs.
 FIX: the AppState listener in useMessages now withdraws and re-asserts the ENGINE's active conversation alongside the push layer's, and on returning to the foreground it re-reports the read and clears the conversation notification. Three new hook tests (chatVisibility.test.tsx) cover it, written RED first: before the change the background case recorded zero setActiveConversation calls, which is the bug exactly. Clearing on resume is also what fixes VC-057 — a notification TAP resumes an ALREADY-MOUNTED chat screen, so the mount effect never re-ran and the stored MessagingStyle lines were never dropped. Verified: 534/534 jest, tsc clean, eslint 0 errors. Live two-device re-verification still pending — the test phone was disconnected before it could be run.</t>

</xml_diff>

<commit_message>
chore(qa): correct VC-061 — the composer padding is load-bearing, only the border was a defect
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA/reports/VelChat-QA-Report.xlsx
+++ b/QA/reports/VelChat-QA-Report.xlsx
@@ -641,7 +641,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-19 08:20 UTC</t>
+          <t>Generated 2026-09-19 08:22 UTC</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -19614,7 +19614,8 @@
       <c r="AA62" s="5" t="inlineStr">
         <is>
           <t>Evidence: scratchpad/shots/a_cal.png and a_own_follow.png — the white band between the composer pill and the keyboard's suggestion strip. Same file also sets `borderTopWidth: 0` alongside a `borderTopColor`, so the intended separator between the thread and the composer never draws.
-FIX: keyboard-up paddingBottom drops from spacing.huge (48dp) to spacing.xs (8dp), and borderTopWidth goes from 0 to 1 so the separator the style always declared actually draws. VERIFIED ON DEVICE: scratchpad/shots/v2_own_follow.png shows the hairline above the composer and the composer sitting close to the keyboard.</t>
+FIX: keyboard-up paddingBottom drops from spacing.huge (48dp) to spacing.xs (8dp), and borderTopWidth goes from 0 to 1 so the separator the style always declared actually draws. VERIFIED ON DEVICE: scratchpad/shots/v2_own_follow.png shows the hairline above the composer and the composer sitting close to the keyboard.
+CORRECTION after on-device testing. Only HALF of this was a defect. The borderTopWidth 0 -&gt; 1 fix is right and shipped: the separator the style always declared now draws. The 48dp padding is NOT over-generous, it is LOAD-BEARING — the parent lifts the bar by keyboardDidShow.endCoordinates.height, and under RN 0.86 Android edge-to-edge that value lands short of the keyboard the user actually sees. Trimming it to 8dp moved the input 40dp down and put it BEHIND the keyboard on a 3-button-nav CPH2643; caught on the device and reverted before it could ship. The white band is cosmetic and invisible against a light keyboard. The real fix is to correct the LIFT, not the padding, and that is separate work.</t>
         </is>
       </c>
       <c r="AB62" s="5" t="inlineStr"/>
@@ -22774,7 +22775,8 @@
       <c r="H36" s="5" t="inlineStr">
         <is>
           <t>Evidence: scratchpad/shots/a_cal.png and a_own_follow.png — the white band between the composer pill and the keyboard's suggestion strip. Same file also sets `borderTopWidth: 0` alongside a `borderTopColor`, so the intended separator between the thread and the composer never draws.
-FIX: keyboard-up paddingBottom drops from spacing.huge (48dp) to spacing.xs (8dp), and borderTopWidth goes from 0 to 1 so the separator the style always declared actually draws. VERIFIED ON DEVICE: scratchpad/shots/v2_own_follow.png shows the hairline above the composer and the composer sitting close to the keyboard.</t>
+FIX: keyboard-up paddingBottom drops from spacing.huge (48dp) to spacing.xs (8dp), and borderTopWidth goes from 0 to 1 so the separator the style always declared actually draws. VERIFIED ON DEVICE: scratchpad/shots/v2_own_follow.png shows the hairline above the composer and the composer sitting close to the keyboard.
+CORRECTION after on-device testing. Only HALF of this was a defect. The borderTopWidth 0 -&gt; 1 fix is right and shipped: the separator the style always declared now draws. The 48dp padding is NOT over-generous, it is LOAD-BEARING — the parent lifts the bar by keyboardDidShow.endCoordinates.height, and under RN 0.86 Android edge-to-edge that value lands short of the keyboard the user actually sees. Trimming it to 8dp moved the input 40dp down and put it BEHIND the keyboard on a 3-button-nav CPH2643; caught on the device and reverted before it could ship. The white band is cosmetic and invisible against a light keyboard. The real fix is to correct the LIFT, not the padding, and that is separate work.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(qa): file VC-071..VC-073 and record the live notification re-tests
VC-071 Mark-as-read carried the arriving seq rather than the highest seen, so a
late out-of-order push acknowledged below the newest message. VC-072 the collapsed
row could show one person's words beside another's face. Both found by an
adversarial review of the same day's notification work and fixed with it.

VC-073 is the narrow remainder of VC-069, split out so that entry reading Fixed is
not taken to cover it: the notification's own ack goes straight to REST from a
process with no database open, so it cannot compute the contiguous watermark the
JS emitters now use.

VC-056, VC-057 and VC-067 re-tested live against their own repro steps, with the
one thing that could not be forced on the day recorded as a caveat rather than
claimed as proof.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA/reports/VelChat-QA-Report.xlsx
+++ b/QA/reports/VelChat-QA-Report.xlsx
@@ -641,7 +641,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-19 14:32 UTC</t>
+          <t>Generated 2026-09-19 14:58 UTC</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -11043,7 +11043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB71"/>
+  <dimension ref="A1:AB74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -18456,7 +18456,8 @@
       <c r="AA53" s="5" t="inlineStr">
         <is>
           <t>Evidence: scratchpad/shots/b_fg_follow.png (B at the bottom, F1-F3 arrive, list stays on S8 and the jump FAB appears), scratchpad/shots/b_one.png (single message ONE1 arrives, list left exactly one bubble short), scratchpad/shots/a_own_follow.png (A's OWN sent ONE1 clipped behind the composer), scratchpad/shots/b_offline_send.png (own offline sends clipped). The race explains the intermittency: sometimes the manual scroll lands after the anchor adjustment and it looks fine.
-FIX: the follow now goes through FlashList's `scrollToIndex({index:0})` instead of `scrollToOffset({offset:0})`, fired from `onContentSizeChange` rather than the data effect. Root cause confirmed by reading useRecyclerViewController.js: on every data change FlashList measures how far the FIRST VISIBLE item moved and calls scrollAnchorRef.scrollBy(diff) to cancel the shift, gated on a `pauseOffsetCorrection` ref that ONLY scrollToIndex raises — so a plain offset scroll was undone every time and the thread landed exactly one bubble short. Firing from onContentSizeChange means index 0 has a real layout instead of the stale one it would have in the same commit. Anchoring is deliberately kept: it is the right behaviour for a reader scrolled up in history, whom shouldScrollToLatest still leaves alone; a drag cancels any pending follow so loadOlder growing the content is never mistaken for a new message. An intermediate attempt using scrollToOffset from onContentSizeChange plus a requestAnimationFrame retry was built and tested on device and still landed one bubble short — that is what identified the pauseOffsetCorrection gate. VERIFIED ON DEVICE: a four-message burst now ends with the newest message fully visible above the composer (scratchpad/shots/v2_own_follow.png) where the same burst on the previous build left it clipped (v_own_follow.png). Still to verify with a second device: the INCOMING-message path, and the notification tap-through landing position.</t>
+FIX: the follow now goes through FlashList's `scrollToIndex({index:0})` instead of `scrollToOffset({offset:0})`, fired from `onContentSizeChange` rather than the data effect. Root cause confirmed by reading useRecyclerViewController.js: on every data change FlashList measures how far the FIRST VISIBLE item moved and calls scrollAnchorRef.scrollBy(diff) to cancel the shift, gated on a `pauseOffsetCorrection` ref that ONLY scrollToIndex raises — so a plain offset scroll was undone every time and the thread landed exactly one bubble short. Firing from onContentSizeChange means index 0 has a real layout instead of the stale one it would have in the same commit. Anchoring is deliberately kept: it is the right behaviour for a reader scrolled up in history, whom shouldScrollToLatest still leaves alone; a drag cancels any pending follow so loadOlder growing the content is never mistaken for a new message. An intermediate attempt using scrollToOffset from onContentSizeChange plus a requestAnimationFrame retry was built and tested on device and still landed one bubble short — that is what identified the pauseOffsetCorrection gate. VERIFIED ON DEVICE: a four-message burst now ends with the newest message fully visible above the composer (scratchpad/shots/v2_own_follow.png) where the same burst on the previous build left it clipped (v_own_follow.png). Still to verify with a second device: the INCOMING-message path, and the notification tap-through landing position.
+REGRESSED AND RE-FIXED, properly this time. The scroll-command approach was wrong in kind, not in detail: three versions were tried (scrollToOffset, scrollToOffset plus a frame, scrollToIndex plus a 180ms retry) and all three lost the same race, because FlashList re-pins the viewport through an invisible ScrollAnchor and that is a STATE update landing a render or two after any callback we can scroll from. The newest bubble kept ending up one message below the fold, intermittently — and it came back on the product owner reproducing it with the keyboard up. FINAL FIX: the list uses the library own chat pattern. Not inverted, rows reversed into ascending order at the list (never in the query, so every grouping flag stays attached to its own row and the rendered result is identical to what the inverted list drew), maintainVisibleContentPosition.autoscrollToBottomThreshold pins the end, startRenderingFromBottom opens on the newest, and loadOlder moves from onEndReached to onStartReached. There is no scroll command left to lose a race. shouldScrollToLatest is gone; autoScroll.ts now only measures distance-from-bottom for the jump button. VERIFIED ON THE REAL DEVICE with the keyboard up, the exact case that was failing: five messages sent, the newest fully visible above the composer, no jump button.</t>
         </is>
       </c>
       <c r="AB53" s="5" t="inlineStr"/>
@@ -18976,7 +18977,8 @@
 FIX: `PushStore.Line` now carries the message's own `seq`, persisted as the JSON key `"q"`, and `showMessage` passes the push's seq into `appendLine`. `appendLine` SORTS before applying the `MAX_LINES` cap, and that order is the fix rather than a detail: capping first dropped whichever line FCM happened to deliver earliest, so an out-of-order push could evict a message newer than the one it kept. `setContentText` and `setLargeIcon` now read the newest INCOMING line (`lines.lastOrNull { !it.mine }`) instead of the message that arrived last, so the collapsed row and the face on it agree with the expanded thread — incoming only, because an inline reply can sort last and quoting the user's own words back at them is not a notification about anything.
 MIGRATION for installs whose stored lines predate `q`: in `sortBySeq` each entry inherits the rank of the one before it and the sort is stable, so a legacy thread ranks entirely at zero and comes back exactly as stored — the only order anyone ever knew for it — while an inline reply (also seq 0) ranks immediately after the message it answered.
 KNOWN LIMITATION, left open deliberately: `Line.at` is still the ARRIVAL timestamp (`System.currentTimeMillis()` at `showMessage`), because the push payload carries no message timestamp. MessagingStyle stamps each line with it, so a REORDERED thread can show non-monotonic times until the backend sends a message timestamp. The order is now right; the clock beside it is not.
-NO AUTOMATED TEST: this project has no Kotlin test source set at all — `android/app/src` holds only `main`, `dev` and `prod` — so nothing in the push package is reachable from Jest. Verified by code review against the report; the live repro still needs re-running on a device.</t>
+NO AUTOMATED TEST: this project has no Kotlin test source set at all — `android/app/src` holds only `main`, `dev` and `prod` — so nothing in the push package is reachable from Jest. Verified by code review against the report; the live repro still needs re-running on a device.
+LIVE RE-TEST 2026-09-19 on the two-device setup, following this entry's own steps (recipient package force-stopped so FCM holds a message, app launched to clear FLAG_STOPPED, a second message sent into the release window). RESULT: the expanded thread came back in seq order with the newest line last (OK4, FIN1, FIN2, FIN3, FIN4, ORD2) and the collapsed row quoted the newest, where the pre-fix run of the same procedure had produced KILL2 above KILL1. Both messages also landed in the conversation in the right order with nothing lost. CAVEAT recorded honestly: FCM released the held message quickly enough that a strictly OUT-OF-ORDER delivery was not forced on this run, so what this proves is correct ordering and no regression, not the reordering path itself firing. That path is covered by code review only (there is no Kotlin test source set in this project).</t>
         </is>
       </c>
       <c r="AB57" s="5" t="inlineStr"/>
@@ -19106,7 +19108,8 @@
       <c r="AA58" s="5" t="inlineStr">
         <is>
           <t>Evidence: scratchpad/shots/b_shade.png (S3..S8 before opening), scratchpad/shots/b_tapthrough.png (chat opened, tray cleared, all read), scratchpad/shots/b_reply_open.png (next notification still carries S6, S7, S8, BG1).
-ROOT CAUSE FOUND and FIXED via VC-062. The clearing path was wired correctly all along — clearConversationNotification -&gt; VelChatPushModule.clearConversation -&gt; PushNotifications.cancel -&gt; store.clearLines — but it only ran from the chat screen's MOUNT effect. A notification tap RESUMES an already-mounted ChatScreen, so that effect never re-ran, and the tray entry disappearing was just the notification's own AUTO_CANCEL flag removing the posted notification while the stored lines and counters survived. useMessages now also clears on every return to the foreground. Live re-verification pending a second device.</t>
+ROOT CAUSE FOUND and FIXED via VC-062. The clearing path was wired correctly all along — clearConversationNotification -&gt; VelChatPushModule.clearConversation -&gt; PushNotifications.cancel -&gt; store.clearLines — but it only ran from the chat screen's MOUNT effect. A notification tap RESUMES an already-mounted ChatScreen, so that effect never re-ran, and the tray entry disappearing was just the notification's own AUTO_CANCEL flag removing the posted notification while the stored lines and counters survived. useMessages now also clears on every return to the foreground. Live re-verification pending a second device.
+LIVE VERIFIED 2026-09-19: after opening the chat and backgrounding again, the next notification carried only the new messages — no line from the batch the user had already read.</t>
         </is>
       </c>
       <c r="AB58" s="5" t="inlineStr"/>
@@ -20432,7 +20435,8 @@
           <t>Found by a code-level audit after the live two-device session. Deterministic, unlike the race in the sibling PushStore report.
 FIX: the `ACTION_DISMISS` branch now calls `store.clearLines(conversationId)` alongside `clearCount`, matching `PushNotifications.cancel`, which has always dropped both halves.
 The SECONDARY half of this report is fixed too, because a backstop that does half of what it backs up just relocates the bug to the group path. `postSummary` gained `setDeleteIntent(summaryDismissIntent(context))`, carrying a new `ACTION_DISMISS_SUMMARY` that `PushActionReceiver.onReceive` answers BEFORE the conversation-id extra is demanded — the summary belongs to no single conversation, so it carries no id and the existing `getStringExtra(...) ?: return` would have swallowed it silently. That branch clears counts AND lines wholesale (`clearAllCounts` + `clearAllLines`). It is idempotent on builds where the children's delete intents do arrive, and it is the only clearing that happens on the OEM builds where they do not.
-NO AUTOMATED TEST: this project has no Kotlin test source set at all — `android/app/src` holds only `main`, `dev` and `prod` — so nothing in the push package is reachable from Jest. Verified by code review against the report; the live repro still needs re-running on a device.</t>
+NO AUTOMATED TEST: this project has no Kotlin test source set at all — `android/app/src` holds only `main`, `dev` and `prod` — so nothing in the push package is reachable from Jest. Verified by code review against the report; the live repro still needs re-running on a device.
+LIVE VERIFIED 2026-09-19 following this entry's own steps: three messages arrived while backgrounded and were swiped away unread, then one more was sent. The rebuilt notification reported android.messages = Parcelable[] (1) — one line, not four. Pre-fix the same procedure re-listed every dismissed message.</t>
         </is>
       </c>
       <c r="AB68" s="5" t="inlineStr"/>
@@ -20836,6 +20840,392 @@
         </is>
       </c>
       <c r="AB71" s="5" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="17" t="inlineStr">
+        <is>
+          <t>VC-071</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>VC-72</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr"/>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>A notification's Mark-as-read carries the arriving seq, so a late out-of-order push acknowledges below the newest message</t>
+        </is>
+      </c>
+      <c r="E72" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F72" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="H72" s="5" t="inlineStr">
+        <is>
+          <t>CLIENT</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>Notifications — Mark as read action</t>
+        </is>
+      </c>
+      <c r="J72" s="5" t="inlineStr">
+        <is>
+          <t>apps/mobile/android/app/src/main/java/com/velchat/push/PushNotifications.kt (showMessage: replyAction / markReadAction)</t>
+        </is>
+      </c>
+      <c r="K72" s="5" t="inlineStr">
+        <is>
+          <t>Production build</t>
+        </is>
+      </c>
+      <c r="L72" s="5" t="inlineStr">
+        <is>
+          <t>Any Android</t>
+        </is>
+      </c>
+      <c r="M72" s="5" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="N72" s="5" t="inlineStr">
+        <is>
+          <t>Whenever FCM delivers two messages for one chat out of order</t>
+        </is>
+      </c>
+      <c r="O72" s="5" t="inlineStr">
+        <is>
+          <t>Deterministic once the pushes land out of order.</t>
+        </is>
+      </c>
+      <c r="P72" s="5" t="inlineStr">
+        <is>
+          <t>Two messages for the same conversation where the later-sent one is delivered first.</t>
+        </is>
+      </c>
+      <c r="Q72" s="5" t="inlineStr">
+        <is>
+          <t>1. Arrange for push seq 10 to land, then push seq 9 to land after it.
+2. The collapsed notification correctly quotes message 10.
+3. Tap Mark as read.
+4. Check what the sender sees for message 10.</t>
+        </is>
+      </c>
+      <c r="R72" s="5" t="inlineStr">
+        <is>
+          <t>The action acknowledges the newest message the notification represents — which is what the rebuild after an inline reply already does, reading store.lastSeq.</t>
+        </is>
+      </c>
+      <c r="S72" s="5" t="inlineStr">
+        <is>
+          <t>Both the Reply and the Mark-as-read PendingIntents were built with showMessage's own `seq` parameter, i.e. the message that happened to arrive last. The notification's PendingIntents carry FLAG_UPDATE_CURRENT, so a late push genuinely rewrites the extras to the LOWER seq. Tapping Mark as read then acknowledges up to the late message and dismisses the notification, leaving the newer one unread to its sender until the app is opened.</t>
+        </is>
+      </c>
+      <c r="T72" s="5" t="inlineStr">
+        <is>
+          <t>The user marks a chat read and the sender still sees an unread message. Silent, and only in the out-of-order case the notification-ordering work exists to handle.</t>
+        </is>
+      </c>
+      <c r="U72" s="5" t="inlineStr">
+        <is>
+          <t>The actions were built from the arriving message rather than from the per-conversation high-water mark the store already keeps. Fixed by reading store.lastSeq after it has been bumped, exactly as showOwnReply does.</t>
+        </is>
+      </c>
+      <c r="V72" s="5" t="inlineStr"/>
+      <c r="W72" s="5" t="inlineStr"/>
+      <c r="X72" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Y72" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Z72" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA72" s="5" t="inlineStr">
+        <is>
+          <t>Found by an adversarial code review of the notification changes made the same day. Same function as the line-ordering fix, whose premise (FCM does not guarantee order) is what makes this reachable.</t>
+        </is>
+      </c>
+      <c r="AB72" s="5" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="17" t="inlineStr">
+        <is>
+          <t>VC-072</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>VC-73</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr"/>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>A notification's collapsed row can show one person's words beside another person's face</t>
+        </is>
+      </c>
+      <c r="E73" s="19" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F73" s="19" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="H73" s="5" t="inlineStr">
+        <is>
+          <t>CLIENT</t>
+        </is>
+      </c>
+      <c r="I73" s="5" t="inlineStr">
+        <is>
+          <t>Notifications — collapsed row avatar</t>
+        </is>
+      </c>
+      <c r="J73" s="5" t="inlineStr">
+        <is>
+          <t>apps/mobile/android/app/src/main/java/com/velchat/push/PushNotifications.kt (showMessage: newestSenderId)</t>
+        </is>
+      </c>
+      <c r="K73" s="5" t="inlineStr">
+        <is>
+          <t>Production build</t>
+        </is>
+      </c>
+      <c r="L73" s="5" t="inlineStr">
+        <is>
+          <t>Any Android</t>
+        </is>
+      </c>
+      <c r="M73" s="5" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="N73" s="5" t="inlineStr">
+        <is>
+          <t>Group chats where a stored line has no sender id</t>
+        </is>
+      </c>
+      <c r="O73" s="5" t="inlineStr">
+        <is>
+          <t>Needs a stored line whose sender id was blank.</t>
+        </is>
+      </c>
+      <c r="P73" s="5" t="inlineStr">
+        <is>
+          <t>A group conversation whose notification thread holds a line stored without a sender id.</t>
+        </is>
+      </c>
+      <c r="Q73" s="5" t="inlineStr">
+        <is>
+          <t>1. Receive several messages in a group so the notification thread holds more than one line.
+2. Ensure one stored line has a blank sender id (an older build, or a push with no senderId).
+3. Receive one more message from a DIFFERENT member and look at the collapsed notification.</t>
+        </is>
+      </c>
+      <c r="R73" s="5" t="inlineStr">
+        <is>
+          <t>The collapsed row's avatar belongs to whoever wrote the text shown beside it.</t>
+        </is>
+      </c>
+      <c r="S73" s="5" t="inlineStr">
+        <is>
+          <t>`newestSenderId` fell back with `newest?.senderId ?: senderId`, so when the newest line exists but its stored sender id reads back as null, the row showed that line's TEXT with the ARRIVING message's avatar.</t>
+        </is>
+      </c>
+      <c r="T73" s="5" t="inlineStr">
+        <is>
+          <t>In a group, the notification attributes a message to the wrong person at a glance. Small, but it is a misattribution on the lock screen.</t>
+        </is>
+      </c>
+      <c r="U73" s="5" t="inlineStr">
+        <is>
+          <t>The elvis guarded the sender id rather than the line. Fixed by guarding on `newest` itself, so the fallback only applies when there is no newest incoming line at all.</t>
+        </is>
+      </c>
+      <c r="V73" s="5" t="inlineStr"/>
+      <c r="W73" s="5" t="inlineStr"/>
+      <c r="X73" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Y73" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Z73" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA73" s="5" t="inlineStr">
+        <is>
+          <t>Found by an adversarial code review of the notification changes made the same day.</t>
+        </is>
+      </c>
+      <c r="AB73" s="5" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="17" t="inlineStr">
+        <is>
+          <t>VC-073</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>VC-74</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr"/>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>Mark-as-read and inline reply acknowledge straight over REST from a process with no database, so they can still claim a message the device does not hold</t>
+        </is>
+      </c>
+      <c r="E74" s="19" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F74" s="19" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H74" s="5" t="inlineStr">
+        <is>
+          <t>CLIENT</t>
+        </is>
+      </c>
+      <c r="I74" s="5" t="inlineStr">
+        <is>
+          <t>Notifications — native receipt ack</t>
+        </is>
+      </c>
+      <c r="J74" s="5" t="inlineStr">
+        <is>
+          <t>apps/mobile/android/app/src/main/java/com/velchat/push/PushActionReceiver.kt (ACTION_MARK_READ, ACTION_REPLY) + PushAckClient</t>
+        </is>
+      </c>
+      <c r="K74" s="5" t="inlineStr">
+        <is>
+          <t>Production build</t>
+        </is>
+      </c>
+      <c r="L74" s="5" t="inlineStr">
+        <is>
+          <t>Any Android</t>
+        </is>
+      </c>
+      <c r="M74" s="5" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="N74" s="5" t="inlineStr">
+        <is>
+          <t>Only for a conversation that already has a seq hole</t>
+        </is>
+      </c>
+      <c r="O74" s="5" t="inlineStr">
+        <is>
+          <t>Needs the hole from VC-051 plus a notification action taken while the app is not running.</t>
+        </is>
+      </c>
+      <c r="P74" s="5" t="inlineStr">
+        <is>
+          <t>A conversation missing a message at some seq, and a notification for a later message in it.</t>
+        </is>
+      </c>
+      <c r="Q74" s="5" t="inlineStr">
+        <is>
+          <t>1. Get the device into the VC-051 state: a message at seq N missing locally while N+1 and above are present.
+2. Receive a later message so a notification appears, with the app not running.
+3. Tap Mark as read (or send an inline Reply) without opening the app.
+4. Look at the tick state for message N on the sender.</t>
+        </is>
+      </c>
+      <c r="R74" s="5" t="inlineStr">
+        <is>
+          <t>No path acknowledges a seq the device does not hold — the same rule the JS emitters now follow.</t>
+        </is>
+      </c>
+      <c r="S74" s="5" t="inlineStr">
+        <is>
+          <t>The receiver posts the notification's own seq to POST /notifications/ack directly. Receipts are cumulative, so that covers the missing message. The three JS emitters are clamped to the highest contiguous seq the device holds; this one is not.</t>
+        </is>
+      </c>
+      <c r="T74" s="5" t="inlineStr">
+        <is>
+          <t>The narrow remainder of VC-069: a sender can still be told a message was read when the recipient never received it, but only via a notification action on an already-holed conversation.</t>
+        </is>
+      </c>
+      <c r="U74" s="5" t="inlineStr">
+        <is>
+          <t>By design, not oversight — the broadcast receiver runs in a process with no WatermelonDB open, so it cannot compute the contiguous watermark the JS path uses. Closing it needs either a native mirror of the highest safe seq (written by JS whenever it changes) or deferring the ack to the next JS wake, which costs the user the immediate feedback the action exists for.</t>
+        </is>
+      </c>
+      <c r="V74" s="5" t="inlineStr"/>
+      <c r="W74" s="5" t="inlineStr"/>
+      <c r="X74" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Y74" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Z74" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA74" s="5" t="inlineStr">
+        <is>
+          <t>Split out of VC-069 while verifying that fix. Recorded so the VC-069 entry, which reads Fixed, is not taken to cover this path.</t>
+        </is>
+      </c>
+      <c r="AB74" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:AB1"/>
@@ -21013,7 +21403,7 @@
         </is>
       </c>
       <c r="B16" s="23" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C16" s="24" t="inlineStr"/>
     </row>
@@ -21024,7 +21414,7 @@
         </is>
       </c>
       <c r="B17" s="23" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C17" s="24" t="inlineStr"/>
     </row>
@@ -21035,7 +21425,7 @@
         </is>
       </c>
       <c r="B18" s="23" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C18" s="24" t="inlineStr"/>
     </row>
@@ -21046,7 +21436,7 @@
         </is>
       </c>
       <c r="B19" s="23" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C19" s="24" t="inlineStr"/>
     </row>
@@ -21556,7 +21946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -22664,7 +23054,8 @@
       <c r="H29" s="5" t="inlineStr">
         <is>
           <t>Evidence: scratchpad/shots/b_fg_follow.png (B at the bottom, F1-F3 arrive, list stays on S8 and the jump FAB appears), scratchpad/shots/b_one.png (single message ONE1 arrives, list left exactly one bubble short), scratchpad/shots/a_own_follow.png (A's OWN sent ONE1 clipped behind the composer), scratchpad/shots/b_offline_send.png (own offline sends clipped). The race explains the intermittency: sometimes the manual scroll lands after the anchor adjustment and it looks fine.
-FIX: the follow now goes through FlashList's `scrollToIndex({index:0})` instead of `scrollToOffset({offset:0})`, fired from `onContentSizeChange` rather than the data effect. Root cause confirmed by reading useRecyclerViewController.js: on every data change FlashList measures how far the FIRST VISIBLE item moved and calls scrollAnchorRef.scrollBy(diff) to cancel the shift, gated on a `pauseOffsetCorrection` ref that ONLY scrollToIndex raises — so a plain offset scroll was undone every time and the thread landed exactly one bubble short. Firing from onContentSizeChange means index 0 has a real layout instead of the stale one it would have in the same commit. Anchoring is deliberately kept: it is the right behaviour for a reader scrolled up in history, whom shouldScrollToLatest still leaves alone; a drag cancels any pending follow so loadOlder growing the content is never mistaken for a new message. An intermediate attempt using scrollToOffset from onContentSizeChange plus a requestAnimationFrame retry was built and tested on device and still landed one bubble short — that is what identified the pauseOffsetCorrection gate. VERIFIED ON DEVICE: a four-message burst now ends with the newest message fully visible above the composer (scratchpad/shots/v2_own_follow.png) where the same burst on the previous build left it clipped (v_own_follow.png). Still to verify with a second device: the INCOMING-message path, and the notification tap-through landing position.</t>
+FIX: the follow now goes through FlashList's `scrollToIndex({index:0})` instead of `scrollToOffset({offset:0})`, fired from `onContentSizeChange` rather than the data effect. Root cause confirmed by reading useRecyclerViewController.js: on every data change FlashList measures how far the FIRST VISIBLE item moved and calls scrollAnchorRef.scrollBy(diff) to cancel the shift, gated on a `pauseOffsetCorrection` ref that ONLY scrollToIndex raises — so a plain offset scroll was undone every time and the thread landed exactly one bubble short. Firing from onContentSizeChange means index 0 has a real layout instead of the stale one it would have in the same commit. Anchoring is deliberately kept: it is the right behaviour for a reader scrolled up in history, whom shouldScrollToLatest still leaves alone; a drag cancels any pending follow so loadOlder growing the content is never mistaken for a new message. An intermediate attempt using scrollToOffset from onContentSizeChange plus a requestAnimationFrame retry was built and tested on device and still landed one bubble short — that is what identified the pauseOffsetCorrection gate. VERIFIED ON DEVICE: a four-message burst now ends with the newest message fully visible above the composer (scratchpad/shots/v2_own_follow.png) where the same burst on the previous build left it clipped (v_own_follow.png). Still to verify with a second device: the INCOMING-message path, and the notification tap-through landing position.
+REGRESSED AND RE-FIXED, properly this time. The scroll-command approach was wrong in kind, not in detail: three versions were tried (scrollToOffset, scrollToOffset plus a frame, scrollToIndex plus a 180ms retry) and all three lost the same race, because FlashList re-pins the viewport through an invisible ScrollAnchor and that is a STATE update landing a render or two after any callback we can scroll from. The newest bubble kept ending up one message below the fold, intermittently — and it came back on the product owner reproducing it with the keyboard up. FINAL FIX: the list uses the library own chat pattern. Not inverted, rows reversed into ascending order at the list (never in the query, so every grouping flag stays attached to its own row and the rendered result is identical to what the inverted list drew), maintainVisibleContentPosition.autoscrollToBottomThreshold pins the end, startRenderingFromBottom opens on the newest, and loadOlder moves from onEndReached to onStartReached. There is no scroll command left to lose a race. shouldScrollToLatest is gone; autoScroll.ts now only measures distance-from-bottom for the jump button. VERIFIED ON THE REAL DEVICE with the keyboard up, the exact case that was failing: five messages sent, the newest fully visible above the composer, no jump button.</t>
         </is>
       </c>
     </row>
@@ -22807,7 +23198,8 @@
 FIX: `PushStore.Line` now carries the message's own `seq`, persisted as the JSON key `"q"`, and `showMessage` passes the push's seq into `appendLine`. `appendLine` SORTS before applying the `MAX_LINES` cap, and that order is the fix rather than a detail: capping first dropped whichever line FCM happened to deliver earliest, so an out-of-order push could evict a message newer than the one it kept. `setContentText` and `setLargeIcon` now read the newest INCOMING line (`lines.lastOrNull { !it.mine }`) instead of the message that arrived last, so the collapsed row and the face on it agree with the expanded thread — incoming only, because an inline reply can sort last and quoting the user's own words back at them is not a notification about anything.
 MIGRATION for installs whose stored lines predate `q`: in `sortBySeq` each entry inherits the rank of the one before it and the sort is stable, so a legacy thread ranks entirely at zero and comes back exactly as stored — the only order anyone ever knew for it — while an inline reply (also seq 0) ranks immediately after the message it answered.
 KNOWN LIMITATION, left open deliberately: `Line.at` is still the ARRIVAL timestamp (`System.currentTimeMillis()` at `showMessage`), because the push payload carries no message timestamp. MessagingStyle stamps each line with it, so a REORDERED thread can show non-monotonic times until the backend sends a message timestamp. The order is now right; the clock beside it is not.
-NO AUTOMATED TEST: this project has no Kotlin test source set at all — `android/app/src` holds only `main`, `dev` and `prod` — so nothing in the push package is reachable from Jest. Verified by code review against the report; the live repro still needs re-running on a device.</t>
+NO AUTOMATED TEST: this project has no Kotlin test source set at all — `android/app/src` holds only `main`, `dev` and `prod` — so nothing in the push package is reachable from Jest. Verified by code review against the report; the live repro still needs re-running on a device.
+LIVE RE-TEST 2026-09-19 on the two-device setup, following this entry's own steps (recipient package force-stopped so FCM holds a message, app launched to clear FLAG_STOPPED, a second message sent into the release window). RESULT: the expanded thread came back in seq order with the newest line last (OK4, FIN1, FIN2, FIN3, FIN4, ORD2) and the collapsed row quoted the newest, where the pre-fix run of the same procedure had produced KILL2 above KILL1. Both messages also landed in the conversation in the right order with nothing lost. CAVEAT recorded honestly: FCM released the held message quickly enough that a strictly OUT-OF-ORDER delivery was not forced on this run, so what this proves is correct ordering and no regression, not the reordering path itself firing. That path is covered by code review only (there is no Kotlin test source set in this project).</t>
         </is>
       </c>
     </row>
@@ -22842,7 +23234,8 @@
       <c r="H34" s="5" t="inlineStr">
         <is>
           <t>Evidence: scratchpad/shots/b_shade.png (S3..S8 before opening), scratchpad/shots/b_tapthrough.png (chat opened, tray cleared, all read), scratchpad/shots/b_reply_open.png (next notification still carries S6, S7, S8, BG1).
-ROOT CAUSE FOUND and FIXED via VC-062. The clearing path was wired correctly all along — clearConversationNotification -&gt; VelChatPushModule.clearConversation -&gt; PushNotifications.cancel -&gt; store.clearLines — but it only ran from the chat screen's MOUNT effect. A notification tap RESUMES an already-mounted ChatScreen, so that effect never re-ran, and the tray entry disappearing was just the notification's own AUTO_CANCEL flag removing the posted notification while the stored lines and counters survived. useMessages now also clears on every return to the foreground. Live re-verification pending a second device.</t>
+ROOT CAUSE FOUND and FIXED via VC-062. The clearing path was wired correctly all along — clearConversationNotification -&gt; VelChatPushModule.clearConversation -&gt; PushNotifications.cancel -&gt; store.clearLines — but it only ran from the chat screen's MOUNT effect. A notification tap RESUMES an already-mounted ChatScreen, so that effect never re-ran, and the tray entry disappearing was just the notification's own AUTO_CANCEL flag removing the posted notification while the stored lines and counters survived. useMessages now also clears on every return to the foreground. Live re-verification pending a second device.
+LIVE VERIFIED 2026-09-19: after opening the chat and backgrounding again, the next notification carried only the new messages — no line from the batch the user had already read.</t>
         </is>
       </c>
     </row>
@@ -23228,7 +23621,8 @@
           <t>Found by a code-level audit after the live two-device session. Deterministic, unlike the race in the sibling PushStore report.
 FIX: the `ACTION_DISMISS` branch now calls `store.clearLines(conversationId)` alongside `clearCount`, matching `PushNotifications.cancel`, which has always dropped both halves.
 The SECONDARY half of this report is fixed too, because a backstop that does half of what it backs up just relocates the bug to the group path. `postSummary` gained `setDeleteIntent(summaryDismissIntent(context))`, carrying a new `ACTION_DISMISS_SUMMARY` that `PushActionReceiver.onReceive` answers BEFORE the conversation-id extra is demanded — the summary belongs to no single conversation, so it carries no id and the existing `getStringExtra(...) ?: return` would have swallowed it silently. That branch clears counts AND lines wholesale (`clearAllCounts` + `clearAllLines`). It is idempotent on builds where the children's delete intents do arrive, and it is the only clearing that happens on the OEM builds where they do not.
-NO AUTOMATED TEST: this project has no Kotlin test source set at all — `android/app/src` holds only `main`, `dev` and `prod` — so nothing in the push package is reachable from Jest. Verified by code review against the report; the live repro still needs re-running on a device.</t>
+NO AUTOMATED TEST: this project has no Kotlin test source set at all — `android/app/src` holds only `main`, `dev` and `prod` — so nothing in the push package is reachable from Jest. Verified by code review against the report; the live repro still needs re-running on a device.
+LIVE VERIFIED 2026-09-19 following this entry's own steps: three messages arrived while backgrounded and were swiped away unread, then one more was sent. The rebuilt notification reported android.messages = Parcelable[] (1) — one line, not four. Pre-fix the same procedure re-listed every dismissed message.</t>
         </is>
       </c>
     </row>
@@ -23314,6 +23708,74 @@
 `markConversationRead` now uses it in place of `maxSeqForConversation`. `pageBackfill` computes it once per page and clamps BOTH cumulative watermarks with it — `noteDelivered(Math.min(highestInbound, contiguous))` and `noteRead(Math.min(highest, contiguous))` — one extra query per page, on the reconnect path only. Read-on-arrival is clamped for free with the `localMax` the gap check already holds in hand (`m.seq &lt;= localMax + 1 ? m.seq : localMax`, with `localMax === 0` treated as unloaded history rather than a hole), so the inbound hot path pays nothing: the very frame that OPENS a hole now reports read only up to the previous local max instead of claiming everything it skipped.
 Covered by `contiguousSeq.test.ts` (6 cases), including both under-reporting traps named above: unloaded history is not a hole, and a tombstone is not a hole.
 RESIDUAL, NOT FIXED HERE: the NATIVE ack path this report also named. `PushActionReceiver`'s Mark-as-read and inline-reply branches still POST `/notifications/ack` with the notification's own `seq` unclamped, because that process has no database open to scan — exactly the reason the report called it out. A native Mark-as-read on a conversation with a hole can therefore still over-claim. Worth its own entry if it is judged to matter; the three JS emitters, which are every path that runs with the app alive, are fixed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>VC-071</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>A notification's Mark-as-read carries the arriving seq, so a late out-of-order push acknowledges below the newest message</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>dev branch, 2026-09-19</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr"/>
+      <c r="F47" s="5" t="inlineStr"/>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>Not independently tested</t>
+        </is>
+      </c>
+      <c r="H47" s="5" t="inlineStr">
+        <is>
+          <t>Found by an adversarial code review of the notification changes made the same day. Same function as the line-ordering fix, whose premise (FCM does not guarantee order) is what makes this reachable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>VC-072</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>A notification's collapsed row can show one person's words beside another person's face</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>dev branch, 2026-09-19</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr"/>
+      <c r="F48" s="5" t="inlineStr"/>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>Not independently tested</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
+          <t>Found by an adversarial code review of the notification changes made the same day.</t>
         </is>
       </c>
     </row>

</xml_diff>